<commit_message>
Update berita 2026-08-08 18:24 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -430,7 +430,7 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -715,8 +715,619 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BEI catat investor saham tumbuh 16,83 persen capai 10,05 juta SID</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 01:18:31 +0700</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PT Bursa Efek Indonesia (BEI) melaporkan jumlah investor saham mencapai 10.052.059 Single Investor Identification (SID) ...</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686141/bei-catat-investor-saham-tumbuh-1683-persen-capai-1005-juta-sid</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IHSG-ditutup-menguat-65-94-poin-070826-Fah-1.jpg</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Alonso sebut Marco Palestra cepat beradaptasi jadi pemain serbaguna</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 01:07:11 +0700</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Manajer Chelsea Xabi Alonso menyebutkan pemain rekrutan baru Marco Palestra cepat beradaptasi menjadi pemain serbaguna ...</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686140/alonso-sebut-marco-palestra-cepat-beradaptasi-jadi-pemain-serbaguna</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/65c3991c-4f05-473d-80c4-08c88de490fd.jpeg</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ruben Amorim sebut permainan Milan sedang dalam perubahan total</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 01:03:05 +0700</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Pelatih AC Milan Ruben Amorim mengatakan permainan tim asuhannya sedang mengalami perubahan secara total menuju gaya ...</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686136/ruben-amorim-sebut-permainan-milan-sedang-dalam-perubahan-total</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/chelsea-kalahkan-ac-milan-2837604.jpg</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kemkomdigi pastikan reaktivasi IGRS ditargetkan rampung 2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 01:01:19 +0700</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Kementerian Komunikasi dan Digital (Kemkomdigi) memastikan reaktivasi dari Indonesia Game Rating System (IGRS) ...</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686135/kemkomdigi-pastikan-reaktivasi-igrs-ditargetkan-rampung-2026</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/pexels-yankrukov-9072317.jpg</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sambut HUT RI, Gebyar Lampu Hias di Pemalang hidupkan suasana kampung</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 00:55:28 +0700</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ANTARA - Ribuan lampu hias seakan menyulap Desa Kandang, Kabupaten Pemalang, Jawa Tengah, menjadi wisata malam selama ...</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686125/sambut-hut-ri-gebyar-lampu-hias-di-pemalang-hidupkan-suasana-kampung</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_SAMBUT-HUT-RI-GEBYAR-LAMPU-HIAS-DI-PEMALANG-HIDUPKAN-SUASANA-KAMPUNG.jpg</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TNBTS tutup seluruh akses wisata Bromo guna efektifkan pemadaman</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 00:43:47 +0700</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Balai Besar Taman Nasional Bromo Tengger Semeru (TNBTS) menutup total seluruh akses wisata ke Gunung Bromo untuk ...</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686132/tnbts-tutup-seluruh-akses-wisata-bromo-guna-efektifkan-pemadaman</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001408308.jpg</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Karhutla di Gunung Bromo semakin meluas akibat angin kencang</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 00:36:32 +0700</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan dan lahan (karhutla) di Gunung Bromo yang merupakan kawasan Taman Nasional Bromo Tengger Semeru ...</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686129/karhutla-di-gunung-bromo-semakin-meluas-akibat-angin-kencang</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-23.40.10.jpeg</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Dirut Bulog: Penyaluran bantuan pangan di Alor bentuk kehadiran negara</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 00:27:12 +0700</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Direktur Utama Perum Bulog Ahmad Rizal Ramdhani menegaskan penyaluran bantuan pangan perdana di Kabupaten Alor, Nusa ...</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686121/dirut-bulog-penyaluran-bantuan-pangan-di-alor-bentuk-kehadiran-negara</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/7DC8B9F4-A15A-4720-A6C2-10221860E10D.jpeg</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ABG di Mamuju Diperkosa 15 Pria, 2 Pelaku Paman Korban</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 00:34:24 +0700</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Hafis Hamdan</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Seorang remaja berusia 15 tahun di Kabupaten Mamuju, menjadi korban pemerkosaan oleh 15 pria. Mirisnya, dua pelaku di antaranya merupakan paman korban.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610415/abg-di-mamuju-diperkosa-15-pria-2-pelaku-paman-korban</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/12/02/ilustrasi-pemerkosaan-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Momen Gibran Spontan Turun dari Mobil Lihat Sekolah Rusak Akibat Bencana di Aceh</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 01:19:18 +0700</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Wapres Gibran mendadak turun dari kendaraan saat meninjau sekolah terdampak bencana di Kabupaten Bireuen, Aceh.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865850/momen-gibran-spontan-turun-dari-mobil-lihat-sekolah-rusak-akibat-bencana-di-aceh</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/gsMDovjxARMQjvNbNFaxQoCpmDM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/gibran-tinjau-sekolah-rusak.jpg</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Koperasi Desa Merah Putih Didorong Jadi Penggerak Ekonomi Desa dan Putus Mata Rantai Tengkulak</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 00:52:26 +0700</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>KDMP didorong menjadi penggerak ekonomi desa dan membantu petani memutus ketergantungan terhadap tengkulak melalui koperasi.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865849/koperasi-desa-merah-putih-didorong-jadi-penggerak-ekonomi-desa-dan-putus-mata-rantai-tengkulak</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/7LB8PJZyvtENrzKYRsBztYhAzXY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/GMPP-dan-jatubu.jpg</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Budi Utomo Hingga Banjaratma jadi Inspirasi Perkembangan Busana Kontemporer</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 00:43:17 +0700</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>11 mahasiswa IKJ mengangkat tradisi, budaya, dan sejarah Indonesia sebagai inspirasi koleksi busana dalam Graduate Competition</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/lifestyle/7865848/budi-utomo-hingga-banjaratma-jadi-inspirasi-perkembangan-busana-kontemporer</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/37ZoNvQhuzkYGv9iQ_Y_FHx2UlE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/defiant-movement.jpg</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Gus Salam Siap Bersaing di Muktamar NU: Yang Penting Restu dan Doa Masyayikh</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 00:33:02 +0700</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Muktamar ke-35 NU akan digelar 27–31 Agustus 2026 di Tambakberas, Jombang, dengan sejumlah kandidat mulai mengonsolidasikan dukungan.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865847/gus-salam-siap-bersaing-di-muktamar-nu-yang-penting-restu-dan-doa-masyayikh</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/nq8oCNsST3sV1fJPgf9kNjv_O90=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Gus-Salam-Abdussalam-Shohib-berdiskusi-Mustasyar-PBNU-KH-Muhtadi-Dimyati-Banten.jpg</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I6"/>
+  <autoFilter ref="A1:I19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 19:25 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1326,8 +1326,196 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Komisi VI DPR RI sosialisasikan kemitraan BUMN di Situbondo</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 02:07:12 +0700</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Komisi VI DPR RI dan PT Bank Rakyat Indonesia (Persero) Tbk Cabang Situbondo, Jawa Timur, menyosialisasikan kemitraan ...</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686148/komisi-vi-dpr-ri-sosialisasikan-kemitraan-bumn-di-situbondo</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG-20260809-WA0004.jpg</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Jorge Martin juara sprint MotoGP Inggris 2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 01:56:54 +0700</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Pebalap Aprilia, Jorge Martin juara sprint MotoGP Inggris  2026 setelah melesat sejak start untuk memimpin seluruh ...</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686145/jorge-martin-juara-sprint-motogp-inggris-2026</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000043245.jpg</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Diabetes Bikin Badan Makin Kurus, Benarkah Tanda Sehat? Dokter Ungkap Kaitannya dengan Insulin</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 02:19:24 +0700</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Diabetes tipe 2 awal sering berkaitan dengan obesitas, tetapi seiring penyakit berlangsung lama, penderita bisa semakin kurus.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865852/diabetes-bikin-badan-makin-kurus-benarkah-tanda-sehat-dokter-ungkap-kaitannya-dengan-insulin</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0XnUcyO36kmboN0RjAEedskMcq8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-turunkan-berat-badan.jpg</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Kabar Baik Pasien Diabetes: Remisi Bukan Sembuh Tapi Bisa Bebas Obat, Ini Caranya</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 01:51:23 +0700</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Diabetes tipe 2 yang baru terdiagnosis berpeluang mengalami remisi, terutama jika kondisi pankreas masih baik dan obesitas serta lemak tubuh.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865851/kabar-baik-pasien-diabetes-remisi-bukan-sembuh-tapi-bisa-bebas-obat-ini-caranya</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/qdE7vg65WvcvRx6ehWWFeAeiSTc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-obat-462626.jpg</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I19"/>
+  <autoFilter ref="A1:I23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 21:22 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1749,8 +1749,196 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Indonesia raih dua medali dari Asian BMX Racing Championships 2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 04:15:54 +0700</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Tim nasional BMX Racing Indonesia meraih dua medali dari Asian BMX Racing Championships 2026 di Arena BMX Nilai, Negeri ...</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686151/indonesia-raih-dua-medali-dari-asian-bmx-racing-championships-2026</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000043259.jpg</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Pelaku Sempat Ngepel Bersihkan Darah di TKP Usai Bunuh Bos Konter HP Ambarawa</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 03:35:59 +0700</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Ardian Dwi Kurnia</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Bukti CCTV itu dibuang pelaku ke kali. Didit dan Taufik kemudian kembali ke lokasi pembunuhan dan membersihkan sisa darah yang berceceran.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610439/pelaku-sempat-ngepel-bersihkan-darah-di-tkp-usai-bunuh-bos-konter-hp-ambarawa</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/pembunuhan-di-semarang-1786196771523_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Bayi Lahir Sesar Berisiko Gangguan Mikrobiota? Begini Penjelasan Pakar</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 03:49:53 +0700</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Bayi lahir caesar tetap dianjurkan mendapat ASI sebagai pilihan pertama untuk mendukung kebutuhan nutrisi dan perkembangan mikrobiota.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865855/bayi-lahir-sesar-berisiko-gangguan-mikrobiota-begini-penjelasan-pakar</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/PrvXmH6DVL8MS-bqugPlsJeI67o=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-melahirkan-ilustrasi-persalinan.jpg</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Badan Kurus Belum Tentu Bebas Diabetes, Waspadai Kondisi 'Skinny Fat'</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 03:09:38 +0700</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Kondisi skinny fat membuat seseorang tampak langsing, tetapi memiliki lemak tubuh tinggi, terutama lemak visceral.</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865854/badan-kurus-belum-tentu-bebas-diabetes-waspadai-kondisi-skinny-fat</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/LuczKHWR7OGSmRRsG6i82GhzA9Q=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/dr-Dicky-Levenus-Tahapary.jpg</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I28"/>
+  <autoFilter ref="A1:I32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 22:19 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,10 +419,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
@@ -1937,8 +1937,196 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Skandal Beruntun Guncang Otoritas Pajak Jepang, Kepercayaan Publik Terancam</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 04:57:33 +0700</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Rentetan skandal mengguncang otoritas pajak Jepang, dari dugaan penggelapan hingga kebocoran data wajib pajak dan praktik papakatsu</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865858/skandal-beruntun-guncang-otoritas-pajak-jepang-kepercayaan-publik-terancam</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/XOZxwkb8Csjru0FL7EV4AOOmAso=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/skandalpajakjepang12223.jpg</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Ratusan Senjata Ditemukan di Sekolah, Menteri PPPA Minta Keamanan Siswa Dijamin</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 04:43:18 +0700</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Kementerian PPPA prihatin atas temuan ratusan senjata, narkotika, dan materi pornografi di sebuah ruangan sekolah di Pondok Pinang.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865857/ratusan-senjata-ditemukan-di-sekolah-menteri-pppa-minta-keamanan-siswa-dijamin</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ItOvBftkxYeWl4YpavOeOzmP3eo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Arifah-Fauzi-Hari-Anak-Nasional_1.jpg</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Kemenag Cairkan BOS Madrasah Tahap II Rp4,1 Triliun, Cek Jadwal Pengajuannya</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 04:12:23 +0700</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Kemenag menyiapkan Rp4,1 triliun untuk BOS Madrasah dan BOP RA Tahap II 2026, terdiri dari Rp3,7 triliun untuk 52 ribu madrasah.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865856/kemenag-cairkan-bos-madrasah-tahap-ii-rp41-triliun-cek-jadwal-pengajuannya</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ZHG5-J1vu7NxJTscg7aMzkVoL3o=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Menteri-Agama-Nasaruddin-Umar-1111.jpg</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Investor Saham RI Tembus 10,05 Juta, BEI Catat Pertumbuhan 16,83 Persen</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 02:31:13 +0700</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- PT Bursa Efek Indonesia (BEI) melaporkan jumlah investor saham domestik telah menembus angka 10,05 juta Single Investor Identification (SID) per 7 Agustus 2026. Pencapaian ini menandai pertumbuhan...</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjgu819530000/investor-saham-ri-tembus-1005-juta-bei-catat-pertumbuhan-1683-persen</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/013233300-1786217473-IHSG-ditutup-menguat-65-94-poi.jpg</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I32"/>
+  <autoFilter ref="A1:I36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 23:23 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2125,8 +2125,948 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>DKI sepekan, kebakaran gedung Bapenda hingga pajak kendaraan listrik</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:14:44 +0700</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Suku Dinas Penanggulangan Kebakaran dan Penyelamatan Jakarta Pusat (Gulkarmat Jakpus) menyatakan kebakaran gedung ...</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686175/dki-sepekan-kebakaran-gedung-bapenda-hingga-pajak-kendaraan-listrik</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/gedung-bapenda-dki-jakarta-kebakaran-2836980_1.jpg</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>RI-Afsel sepakat lestarikan warisan Sheikh Yusuf Al-Makassari</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:12:59 +0700</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Pemerintah Indonesia dan Afrika Selatan (Afsel) sepakat untuk bekerja sama membangun sektor kebudayaan melalui ...</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686173/ri-afsel-sepakat-lestarikan-warisan-sheikh-yusuf-al-makassari</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-20.03.58.jpeg</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Bumibaru Panen 307 Ribu Kg dari Lahan Terdegradasi di Kalteng</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:00:13 +0700</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Palangka Raya (ANTARA) — PT Bumibaru Indonesia Jaya mencatat produksi lebih dari 307 ribu kilogram komoditas ...</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686172/bumibaru-panen-307-ribu-kg-dari-lahan-terdegradasi-di-kalteng</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-08-at-21.42.19.jpeg</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Transaksi QRIS semester I-2026 melesat capai Rp600 triliun</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Volume transaksi dengan Kode Respons Cepat Standar Indonesia (QRIS) melonjak lebih dari 100 persen pada semester I-2026 ...</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5685988/transaksi-qris-semester-i-2026-melesat-capai-rp600-triliun</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/20260808-Transaksi-QRIS-semester-I-2026-melesat-capai-Rp600-triliun.jpg</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Yang hilang bukan sekadar kursi</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:57:50 +0700</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Sebuah kursi besi yang semestinya menjadi tempat warga beristirahat ditemukan berada di atas timbangan lapak barang ...</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686168/yang-hilang-bukan-sekadar-kursi</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Satpol-PP-Amankan-Kursi-Besi-Berlogo-Pemkot-4.jpeg</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Kriminal sepekan, senjata di sekolah lalu Sali Irsalina dianiaya</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:53:45 +0700</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Kepolisian menegaskan tidak ada ekstrakurikuler (ekskul) menembak di sekolah swasta di kawasan Pondok Pinang, ...</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686164/kriminal-sepekan-senjata-di-sekolah-lalu-sali-irsalina-dianiaya</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1001014987.jpg</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Jakarta diprakirakan cerah berawan hari Minggu ini</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:37:11 +0700</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) memprakirakan wilayah Jakarta cerah berawan sepanjang hari Minggu ...</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686161/jakarta-diprakirakan-cerah-berawan-hari-minggu-ini</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/04/1000872408.jpg</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Romeny cetak gol, Hubner starter saat Fortuna Sittard tahan PSV 2-2</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:24:14 +0700</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Fortuna Sittard menahan imbang juara Liga Belanda musim lalu, PSV Eindhoven 2-2 dalam laga pembuka Eredivisie 2026/27 ...</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686157/romeny-cetak-gol-hubner-starter-saat-fortuna-sittard-tahan-psv-2-2</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000043265.jpg</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Mastel dorong platform global andil ke infrastruktur digital nasional</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:16:55 +0700</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Masyarakat Telematika Indonesia (Mastel) mendorong kehadiran ekosistem yang dapat melibatkan platform digital global ...</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686155/mastel-dorong-platform-global-andil-ke-infrastruktur-digital-nasional</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/20260809_040240.jpg</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Data Pajak Aman Usai Gedung Bapenda DKI Kebakaran</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:00:51 +0700</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Kebakaran di Gedung Bapenda DKI Jakarta tidak ganggu data perpajakan. Pemprov pastikan layanan publik tetap berjalan, sementara penyebab kebakaran diselidiki.</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610452/data-pajak-aman-usai-gedung-bapenda-dki-kebakaran</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/puing-kebakaran-gedung-bapenda-dki-mulai-dibersihkan-1786180934323_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Keluarga Resmi Laporkan Kasus Kematian Sutrimo ke Polisi</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:18:25 +0700</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Anang Firmansyah</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Keputusan tersebut diambil usai keluarga ingin mendapatkan kepastian hukum dari sejumlah kabar simpang siur yang beredar terkait kematian Sutrimo.</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610446/keluarga-resmi-laporkan-kasus-kematian-sutrimo-ke-polisi</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/sutrimo-1786212205527_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Dea Annisa Menangis Mohon Maaf kepada Ibunda di Pengajian Jelang Pernikahan</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:22:05 +0700</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Desi Puspasari</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Dea Annisa atau Dea Imut menggelar acara pengajian jelang pernikahan pada Sabtu (8/8/2026). Ini momen haru Dea ketika memohon maaf kepada ibunda.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610337/dea-annisa-menangis-mohon-maaf-kepada-ibunda-di-pengajian-jelang-pernikahan</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/dea-annisa-1786198675603_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Jadwal SEA V Cup 2026 Hari Ini: Timnas Voli Putri Indonesia Usung Misi Kebangkitan vs Filipina</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:55:26 +0700</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Jadwal SEA V Cup 2026 Putri hari ini, Minggu (9/8), di mana Timnas Voli Putri Indonesia usung misi kebangkitan saat lawan Filipina.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865865/jadwal-sea-v-cup-2026-hari-ini-timnas-voli-putri-indonesia-usung-misi-kebangkitan-vs-filipina</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/OOLBbprQcY1cr22b0ssNHi4GdCM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Voli-Vietnam-vs-Indonesia-sea-v-cup.jpg</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Misteri Lansia Tewas dalam Sumur di Kuningan, Ada Bercak Darah di Dapur dan Luka di Tubuh</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:55:24 +0700</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Lansia di Kuningan ditemukan tewas dalam sumur setelah keluarga menemukan bercak darah di dapur. Polisi menemukan luka dan dalami penyebab kematian</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865864/misteri-lansia-tewas-dalam-sumur-di-kuningan-ada-bercak-darah-di-dapur-dan-luka-di-tubuh</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/FbeO1FKfjZTDxzjDOCfTfhc7LE4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/mayatdikuningan11111.jpg</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>17 Tahun Jadi Barista, Katsushi Iwata Puji Kopi Indonesia dan Ingin Kunjungi Bali</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:32:32 +0700</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Barista Jepang Katsushi Iwata kagum dengan kopi Indonesia dan ingin berkunjung ke Bali. Ia juga mencatat sejumlah prestasi di kompetisi latte art</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865863/17-tahun-jadi-barista-katsushi-iwata-puji-kopi-indonesia-dan-ingin-kunjungi-bali</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0nsutAhx2Ib3OXkHYVqoZGp6PEs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/baristajepang2221.jpg</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Kabar Abroad Timnas Indonesia: Ole Romeny Nyekor di Liga Belanda, Dean James Kalahkan Nathan</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:26:44 +0700</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Kabar abroad Timnas Indonesia datang dari Liga Belanda seperti Ole Romeny hingga Dean James. Sedangkan Joey Pelupessy main penuh di Liga Belgia.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865862/kabar-abroad-timnas-indonesia-ole-romeny-nyekor-di-liga-belanda-dean-james-kalahkan-nathan</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/CBg5h7IxyaxlQnqkJAtR4aQq5qE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Selebrasi-Ole-Romeny-Usai-Bobol-Gawang-China_20250605_222811.jpg</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Penembakan di Festival Lembah Baliem Lukai 2 Warga, TPNPB-OPM Klaim Bertanggung Jawab</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:22:42 +0700</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Penembakan terjadi di tengah Festival Budaya Lembah Baliem di Jayawijaya. Dua warga terluka, sementara TPNPB-OPM mengklaim bertanggung jawab</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865861/penembakan-di-festival-lembah-baliem-lukai-2-warga-tpnpb-opm-klaim-bertanggung-jawab</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/JWrpJ5u-5Hdb7EHda7BOWOmgDhM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/penembakanpapua112222.jpg</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Jadwal Final GOTF 2026 Hari Ini: ONIC vs Bigetron, Piala Dipastikan Pulang ke Indonesia</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:16:36 +0700</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Jadwal final GOTF 2026 yang digelar hari ini, Minggu (9/8) mempertemukan dua wakil Indonesia, ONIC vs Bigetron.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/e-sport/7865860/jadwal-final-gotf-2026-hari-ini-onic-vs-bigetron-piala-dipastikan-pulang-ke-indonesia</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ne-o3xsng5kpxrlh_KI2cPrtxBI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ONIC-dan-Bigetron-lolos-ke-final-GOTF-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Jemput Skuad AC Milan, Pendaratan Airbus A380-800 di Bandara Soekarno-Hatta Disambut Antusias Warga</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:00:52 +0700</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Pesawat Airbus A380-800 Perdana Mendarat di Bandara Soekarno-Hatta, Warga Tangerang Ramai-Ramai Abadikan Pesawat Jumbo</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865859/jemput-skuad-ac-milan-pendaratan-airbus-a380-800-di-bandara-soekarno-hatta-disambut-antusias-warga</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/FgoO27dgNj710RWe1KkvfJQFvn8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Airbus-A380-800-milik-maskapai-Emirates.jpg</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Terungkap Pelaku Penembakan di Festival Lembah Baliem</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 05:27:22 +0700</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Akibat penembakan itu, dua warga mengalami luka.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265384/terungkap-pelaku-penembakan-di-festival-lembah-baliem</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/hisaV6SdNRoLD0GloBD8UgYAlx8=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319281/original/087646100_1786228035-1002607642.jpg</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I36"/>
+  <autoFilter ref="A1:I56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 00:47 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="43" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -3065,8 +3065,1747 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Pakar paru ingatkan cuaca panas berlebihan tingkat risiko ISPA</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:41:20 +0700</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Ketua Majelis Kehormatan Perhimpunan Dokter Paru Indonesia Prof Tjandra Yoga Aditama mengingatkan fenomena El Nino dan ...</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686209/pakar-paru-ingatkan-cuaca-panas-berlebihan-tingkat-risiko-ispa</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/01/14/InShot_20250114_085854319.jpg</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Minggu, BMKG: Cuaca kota-kota besar RI berawan hingga berawan tebal</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:35:11 +0700</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) memprakirakan kondisi cuaca di kota-kota besar di Indonesia pada ...</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686205/minggu-bmkg-cuaca-kota-kota-besar-ri-berawan-hingga-berawan-tebal</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/15/1000851457_1.jpg</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Dwayne Johnson tanggapi kurang berhasilnya film Moana di Box Office</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:33:35 +0700</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Aktor Dwayne Johnson memberikan tanggapan pribadinya atas isu yang menyatakan film live-action "Moana" kurang ...</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686201/dwayne-johnson-tanggapi-kurang-berhasilnya-film-moana-di-box-office</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-18.04.39.jpeg</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Dua lokasi SIM Keliling di Jakarta pada Minguu</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:31:55 +0700</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Direktorat Lalu Lintas (Ditlantas) Polda Metro Jaya membuka layanan Surat Izin Mengemudi (SIM) Keliling di lima ...</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686197/dua-lokasi-sim-keliling-di-jakarta-pada-minguu</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/09/1000841588.jpg</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Nusa Dua Eco Market perkuat ekosistem UMKM produk ramah lingkungan</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:12:38 +0700</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ANTARA - InJourney Tourism Development Corporation (ITDC) bersama Bank Rakyat Indonesia (BRI) memperkuat ekosistem UMKM ...</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686189/nusa-dua-eco-market-perkuat-ekosistem-umkm-produk-ramah-lingkungan</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_NUSA-DUA-ECO-MARKET-PERKUAT-EKOSISTEM-UMKM-PRODUK-RAMAH-LINGKUNGAN_1.jpg</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Gaikindo optimistis dengan tren positif GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:47:39 +0700</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Ketua Harian sekaligus Ketua Penyelenggara Pameran dan Konferensi Gaikindo Anton Kumonty menyatakan optimistis dengan ...</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5686191/gaikindo-optimistis-dengan-tren-positif-giias-2026</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/41886ebe-cba8-411e-b7c6-52d447d4f08c.jpeg</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Udara Jakarta tercatat tak sehat Minggu pagi</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:40:41 +0700</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Kualitas udara Kota Jakarta tercatat tidak sehat sehingga masyarakat disarankan memakai masker saat berada di luar ...</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686185/udara-jakarta-tercatat-tak-sehat-minggu-pagi</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/01/KLH-catat-penyebab-polusi-udara-di-Jabodetabek-250625-sth-04.jpg</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Bontang Kuala, kehangatan hidup kampung nelayan terapung</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:37:29 +0700</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Di pesisir Kota Bontang, Kalimantan Timur, berdiri Kelurahan Bontang Kuala di Kecamatan Bontang Utara, sebuah ...</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686183/bontang-kuala-kehangatan-hidup-kampung-nelayan-terapung</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/bontang-kuala-3_1.jpg</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Dishub DKI: Pengaturan lalin tetap jalan pascakebakaran gedung Bapenda</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:35:42 +0700</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) DKI Jakarta memastikan layanan pengaturan lalu lintas tetap berjalan pascakebakaran ...</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686179/dishub-dki-pengaturan-lalin-tetap-jalan-pascakebakaran-gedung-bapenda</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000317121.jpg</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Pramono Putuskan Bongkar 1 JPO Viral Dekat tapi Tak Tersambung di Rasuna Said</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:29:17 +0700</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Dia menjelaskan jika kedua JPO tersebut disambungkan akan tetap memiliki ketinggian yang berbeda sehingga tidak bisa dimanfaatkan disabilitas.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610484/pramono-putuskan-bongkar-1-jpo-viral-dekat-tapi-tak-tersambung-di-rasuna-said</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/pramono-anung-muliadetikcom-1786235173314_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Kabar Terkini Terkait Temuan Nyaris Seribu Senjata di Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:04:01 +0700</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Teka-teki temuan hampir seribu senjata dalam ruang Ketua Yayasan sekolah swasta di Jaksel mulai terkuak. Jenis mayoritas senjata itu kini telah dipetakan polisi</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610461/kabar-terkini-terkait-temuan-nyaris-seribu-senjata-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/temuan-ratusan-pucuk-senjata-di-sekolah-swasta-di-pondok-pinang-jakarta-selatan-1786014363566_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Kematian Tak Wajar Sutrimo Sudah Dilaporkan ke Polisi, Pelapor Minta Ekshumasi</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:44:40 +0700</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Polisi menyelidiki kematian Sutrimo di depan klinik kecantikan di Jakarta. Kondisi kematiannya dianggap tidak wajar, pelapor minta ekshumasi.</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610458/kematian-tak-wajar-sutrimo-sudah-dilaporkan-ke-polisi-pelapor-minta-ekshumasi</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/27/puslabfor-polri-menggelar-olah-tempat-kejadian-perkara-tkp-di-klinik-mordent-kawasan-kebayoran-baru-jakarta-selatan-1785134569014_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Penampakan Pelat Berdarah Saksi Bisu Pembunuhan Bos Konter HP Ambarawa</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:26:19 +0700</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Ardian Dwi Kurnia</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Polisi juga menampilkan pelat AD-1398-YJ yang terdapat bercak darah pada bagian kiri bawah. Benda ini berada di dalam bagasi tempat jenazah korban diletakkan.</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610457/penampakan-pelat-berdarah-saksi-bisu-pembunuhan-bos-konter-hp-ambarawa</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/pembunuhan-di-semarang-1786188318705_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Saat Perusahaan AS Cuan Triliunan Per Hari Gara-gara Harga Minyak Tinggi</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:30:13 +0700</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Raksasa minyak asal Amerika Serikat (AS) seperti ExxonMobil dan Chevron berhasil meraup keuntungan yang sangat besar.</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8610239/saat-perusahaan-as-cuan-triliunan-per-hari-gara-gara-harga-minyak-tinggi</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2016/05/01/6ac41af0-b4c0-4701-b837-2a7851f6e4bc_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Langsung Merapat ke Transmart Full Day Sale! Pesta Diskon Meriah 50% + 20%</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Aulia Damayanti</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Transmart Full Day Sale hadir lagi hari ini, Minggu 9 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609349/langsung-merapat-ke-transmart-full-day-sale-pesta-diskon-meriah-50-20</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/transmart-full-day-sale-9-agustus-2026-1786121298154_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Mentan Turun Tangan Bikin Harga Beras di Alor Jadi Rp 13.000/Kg</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:30:14 +0700</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Beras sudah aman, ada di gudang-gudang sekarang. Harga itu Rp 13.000, sama dengan harga Jakarta. Kita sekarang tidak akan kesulitan beras, ujar Amran.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610229/mentan-turun-tangan-bikin-harga-beras-di-alor-jadi-rp-13-000-kg</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/menteri-pertanian-mentan-andi-amran-sulaiman-1786178494091_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>PCPM Bank Indonesia Dibuka Hari Ini, Cek Syaratnya</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:00:58 +0700</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Bank Indonesia (BI) membuka pendaftaran lowongan kerja melalui program Pendidikan Calon Pegawai Asisten Manajer (PCPM) mulai hari ini, Minggu (9/8).</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/lainnya/d-8610226/pcpm-bank-indonesia-dibuka-hari-ini-cek-syaratnya</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/10/29/ilustrasi-bank-indonesia-6_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Tasyi Athasyia Polisikan Karyawan atas Dugaan Pencurian Senilai Rp500 Juta</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:08:35 +0700</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Tasyi Athasyia melaporkan karyawan atas dugaan pencurian barang branded senilai Rp500 juta. Ia menempuh jalur hukum setelah menemukan bukti transaksi penjualan.</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610466/tasyi-athasyia-polisikan-karyawan-atas-dugaan-pencurian-senilai-rp500-juta</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/09/tasyi-athasyia-1780994166890_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>10 Contoh Pidato HUT RI 17 Agustus Singkat, Cocok untuk Acara Sekolah hingga Kampung</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:38:09 +0700</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Simak kumpulan contoh pidato HUT ke-81 RI yang singkat dan penuh makna, cocok untuk acara di sekolah hingga kampung.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865877/10-contoh-pidato-hut-ri-17-agustus-singkat-cocok-untuk-acara-sekolah-hingga-kampung</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/CDmWNBJNXqrhUyeQoHOUutROwRE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/malam-tirakatan-di-kelurahan-muja-muju.jpg</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>6 Tuntutan Iran ke AS jika Ingin Selat Hormuz Dibuka, Minta Ganti Rugi hingga Hapus Sanksi</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:36:58 +0700</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Pemerintah Iran memberikan enam tuntutan yang harus dipenuhi oleh Amerika Serikat (AS) jika ingin Selat Hormuz dibuka.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865876/6-tuntutan-iran-ke-as-jika-ingin-selat-hormuz-dibuka-minta-ganti-rugi-hingga-hapus-sanksi</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/sykTorehl5Nq1lIUzlqoRmb2FiY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/selat-hormuz-ramai-juni-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Ruben Onsu Bongkar Komunikasi dengan Anak-anak di Tengah Konflik dengan Sarwendah</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:33:49 +0700</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Di tengah konflik dengan Sarwendah dan gugatan hak asuh anak, Ruben Onsu mengungkap komunikasi yang masih terjalin dengan anak-anaknya.</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865875/ruben-onsu-bongkar-komunikasi-dengan-anak-anak-di-tengah-konflik-dengan-sarwendah</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/GHpt62tuig514FSTblvdMr1GGQc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ruben-Onsu-ketemu-anak22.jpg</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Rashford Kembali ke Manchester United, Carrick Siapkan Panggung Pembuktian Lawan Leeds</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:20:54 +0700</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Michael Carrick sambut kembalinya Marcus Rashford di Manchester United untuk menjalani pramusim di Dublin melawan Leeds United,</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865874/rashford-kembali-ke-manchester-united-carrick-siapkan-panggung-pembuktian-lawan-leeds</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rUPG4n-YQc8DyP71l6MuTLUdAoA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Logo-klub-Manchester-United.jpg</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Kedalaman Skuad Arsenal Gak Ada Obat, Bruno Guimaraes Tambah Kepusingan Mikel Arteta</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:20:24 +0700</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Pusing yang menyenangkan menjadi tajuk dari keberhasilan Arsenal merekrut Bruno Guimaraes di jendela transfer musim panas ini.</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865873/kedalaman-skuad-arsenal-gak-ada-obat-bruno-guimaraes-tambah-kepusingan-mikel-arteta</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WJRweGk0z2quznJZ-d5GqV5lGCQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Logo-klub-Liga-Inggris-Arsenal.jpg</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Bantah Provokasi Duluan, Ruben Onsu: Saya Hanya Meluruskan yang Dilontarkan Sarwendah</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:11:51 +0700</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Ruben Onsu membantah sengaja memprovokasi Sarwendah. Ia mengaku hanya meluruskan pernyataan yang lebih dulu disampaikan sang mantan istri.</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865872/bantah-provokasi-duluan-ruben-onsu-saya-hanya-meluruskan-yang-dilontarkan-sarwendah</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/17MeeNABlB64uNZ5bi9H-74-Xeg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SIDANG-SARWENDAH-RUBEN-onsu.jpg</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Bandung Raya Minggu, 9 Agustus 2026: Seluruh Wilayah Cerah Berawan</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:08:47 +0700</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Simak prakiraan cuaca wilayah Bandung Raya pada Minggu (9/8/2026). Cuaca di seluruh wilayah Bandung Raya diprakirakan cerah berawan.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865871/prakiraan-cuaca-bandung-raya-minggu-9-agustus-2026-seluruh-wilayah-cerah-berawan</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/lDgUVS5zQ1sLN8t3mHbweeriZkY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-cerah-berawan-xx.jpg</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Botol Guinness Berusia 162 Tahun Ditemukan di Kapal Karam Inggris, Isinya Diduga Masih Bisa Diminum</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:07:26 +0700</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Botol Guinness dari 1864 ditemukan utuh di bangkai kapal Dover. Isinya berpotensi mengungkap seperti apa bir Guinness lebih dari 160 tahun lalu</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865870/botol-guinness-berusia-162-tahun-ditemukan-di-kapal-karam-inggris-isinya-diduga-masih-bisa-diminum</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/PIOyTP7fbLfsgtoxdCwDluOoT4s=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/uk122222.jpg</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Richard Lee Yakin Doktif Beli Produk Kecantikan yang Diperkarakan, Bukan dari Toko Resminya</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:00:20 +0700</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Kasus Richard Lee Vs Doktif masih bergulir di  Pengadilan Negeri Tangerang. Asal produk kecantikan yang menjadi bagian dari perkara t</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865869/richard-lee-yakin-doktif-beli-produk-kecantikan-yang-diperkarakan-bukan-dari-toko-resminya</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/raMS_Fi5E6sdVoc15LmEgpnQh_M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Richard-Lee-bap-doktif.jpg</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Indonesia Saksinya: Main 90 Menit, Misi Terselubung Xabi Alonso Hilangkan Trauma Romeo Lavia</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:41:19 +0700</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Xabi Alonso sengaja biarkan Romeo Lavia main 90 menit lawan AC Milan untuk membantu mengatasi hambatan mental setelah lama berkutat dengan cedera.</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865868/indonesia-saksinya-main-90-menit-misi-terselubung-xabi-alonso-hilangkan-trauma-romeo-lavia</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/b4EDjfafm1mHdVmpCHiGt-ytV24=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Chelsea-FC-vs-AC-Milan_20260808_220023.jpg</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Mourinho Ingin Jinakkan Tantrum Vinicius, Cosplay Figur Ayah di Real Madrid</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:32:34 +0700</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Jose Mourinho siap menjadi figur ayah bagi Vinicius untuk membantu mengontrol emosi dan menghindari kontroversi di lapangan.</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865867/mourinho-ingin-jinakkan-tantrum-vinicius-cosplay-figur-ayah-di-real-madrid</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/E54RA_I8M15KG7G9nmg6eXOU94s=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Logo-klub-Real-Madrid.jpg</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Rambut Perempuan India Ini Capai 2,7 Meter dan Pecahkan Rekor Guinness</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:27:54 +0700</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Renu Dhariyal mencetak rekor Guinness dengan rambut sepanjang 2,7 meter. Ia tidak memotong rambut sejak 2015 dan merawatnya secara alami</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865866/rambut-perempuan-india-ini-capai-27-meter-dan-pecahkan-rekor-guinness</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5iIaoORh3XQZOqHEYLotwCF9KdA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/rambutterpanjang12222.jpg</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Energi</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Presiden Baru Kolombia Hidupkan Kembali Industri Minyak dan Gas</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Gita Amanda</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, BOGOTA -- Presiden baru Kolombia Abelardo de la Espriella berjanji menghidupkan kembali sektor minyak dan gas negara itu, membalik kebijakan energi pemerintahan mantan Presiden Gustavo Petro yang lebih menekankan...</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjh6yp423/presiden-baru-kolombia-hidupkan-kembali-industri-minyak-dan-gas</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/presiden-kolombia-abelardo-de-la-espriella-menyampaikan-pidato-di_260809065950-626.jpg</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Kemenag Siapkan Rp 4,1 Triliun untuk BOS Madrasah dan BOP RA Tahap II</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:36:53 +0700</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Gita Amanda</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Kementerian Agama (Kemenag) tengah memproses penyaluran Bantuan Operasional Sekolah (BOS) Madrasah dan Bantuan Operasional Penyelenggaraan Raudlatul Athfal (BOP RA) Tahap II Tahun Anggaran 2026. Total anggaran yang...</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjh5lh423/kemenag-siapkan-rp-41-triliun-untuk-bos-madrasah-dan-bop-ra-tahap-ii</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/097458600-1721030792-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Pengaturan Lalu Lintas Tetap Berjalan Meski Gedung Bapenda DKI Terbakar</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:29:41 +0700</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Pemprov DKI memastikan layanan pengaturan lalu lintas tetap berjalan.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265405/pengaturan-lalu-lintas-tetap-berjalan-meski-gedung-bapenda-dki-terbakar</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/52lILgt4z3nmJmr6lAjtP2F8ss0=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5574111/original/011344500_1777963166-Kembangan.jpeg</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Dedi Mulyadi Siapkan Knalpot Gratis untuk Pengendara Tak Mampu</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:02:28 +0700</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Pengendara wajib mengganti knalpot nonstandar di lokasi sebelum diperbolehkan kembali melanjutkan perjalanan.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265396/dedi-mulyadi-siapkan-knalpot-gratis-untuk-pengendara-tak-mampu</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/_zjJghz0VtbJVAH9Iry-hZianC8=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5458366/original/038352700_1767077924-IMG_20251230_123004_818.jpg</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Money</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Harga Emas Antam Hari Ini Minggu 9 Agustus 2026, Cek Daftar Terbarunya</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:47:39 +0700</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Harga emas Antam hari ini, Minggu (9/8/2026) terpantau tidak berubah dibandingkan perdagangan sebelumnya.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/08/09/074553026/harga-emas-antam-hari-ini-minggu-9-agustus-2026-cek-daftar-terbarunya</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/zM6BI9IS_-36XIDqLph5kAjGpRU=/0x0:1200x800/1200x675/filters:watermark(data/photo/2026/01/30/697c815e7ef28.png,0,-0,1)/data/photo/2026/06/21/6a37463e5a322.jpg</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Kecelakaan Helikopter Terjadi Lagi di Brasil, 4 Orang Tewas</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:47:39 +0700</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Setidaknya empat orang tewas dalam kecelakaan helikopter di kota Rio de Janeiro, Brasil, Sabtu (8/8/2026).</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/global/read/2026/08/09/070019770/kecelakaan-helikopter-terjadi-lagi-di-brasil-4-orang-tewas</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/GbFkovSLLMEf4Vo4QcgK1EZ47oo=/192x131:1728x1155/1200x675/filters:watermark(data/photo/2026/01/30/697c81ac46b81.png,0,-0,1)/data/photo/2025/08/07/6894887e32329.jpg</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Tren</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Supir Bus di Jerman Tendang Drone yang Berisi Bom di Bandara</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:47:39 +0700</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Seorang supir bus menendang drone dengan bom yang terbang pelan di bandara Jerman. Untungnya, bom tidak meledak.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/tren/read/2026/08/09/060000465/supir-bus-di-jerman-tendang-drone-yang-berisi-bom-di-bandara</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/MUR7vL8oRZ4IRB8DIDRsw4U_OWE=/0x0:1999x1333/1200x675/filters:watermark(data/photo/2026/01/30/697c818d0ca91.png,0,-0,1)/data/photo/2025/02/27/67c033b2c4243.jpg</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I56"/>
+  <autoFilter ref="A1:I93"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 02:59 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$172</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I93"/>
+  <dimension ref="A1:I172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4804,8 +4804,3722 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Jepang akan tingkatkan dukungan bahasa bagi anak-anak asing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:51:33 +0700</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Pemerintah Jepang diperkirakan akan meningkatkan dukungan bagi program bahasa Jepang tingkat pemula untuk anak-anak ...</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686289/jepang-akan-tingkatkan-dukungan-bahasa-bagi-anak-anak-asing</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/29/Jepang.jpg</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Baznas perkuat kapasitas kesiapsiagaan Tim RSB hadapi kebakaran</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:48:56 +0700</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Badan Amil Zakat Nasional (Baznas) RI memberikan pelatihan dan simulasi mitigasi kebakaran bagi personel Rumah Sehat ...</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686285/baznas-perkuat-kapasitas-kesiapsiagaan-tim-rsb-hadapi-kebakaran</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-07-at-13.15.39.jpeg</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Menko Pangan: Pirolisis lengkapi PSEL tangani sampah nasional</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:45:24 +0700</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator (Menko) Bidang Pangan Zulkifli Hasan (Zulhas) mengatakan pemerintah mendorong pemanfaatan teknologi ...</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686283/menko-pangan-pirolisis-lengkapi-psel-tangani-sampah-nasional</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000178838.jpg</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Kasus Bengkulu, KPK sita dokumen usai geledah 3 lokasi selama 3 hari</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:41:45 +0700</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Komisi Pemberantasan Korupsi (KPK) menyita sejumlah dokumen seusai menggeledah tiga lokasi selama 5-7 Agustus 2026 ...</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686280/kasus-bengkulu-kpk-sita-dokumen-usai-geledah-3-lokasi-selama-3-hari</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Portal-1200x800-53.jpg</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Mendag: RI-Brasil pertimbangkan pembentukan PTA Indonesia-Mercosur</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:40:23 +0700</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Menteri Perdagangan (Mendag) Budi Santoso mengatakan pemerintah Indonesia dan Brasil mempertimbangkan pembentukan ...</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686276/mendag-ri-brasil-pertimbangkan-pembentukan-pta-indonesia-mercosur</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_1009.jpeg</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Nagasaki peringati 81 tahun bom atom di tengah debat deterensi nuklir</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:37:05 +0700</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Kota Nagasaki di Jepang, Ahad, memperingati 81 tahun serangan bom atom oleh Amerika Serikat pada Perang Dunia II di ...</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686273/nagasaki-peringati-81-tahun-bom-atom-di-tengah-debat-deterensi-nuklir</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/ilustrasi-peringatan-bom-atom-Jepang.jpg</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Pentagon desak produksi senjata AS digenjot akibat cadangan menipis</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:31:37 +0700</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Departemen Perang Amerika Serikat (Pentagon) mendesak perusahaan pertahanan untuk menggenjot produksi dan pengiriman ...</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686272/pentagon-desak-produksi-senjata-as-digenjot-akibat-cadangan-menipis</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/senjata.jpg</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Penghentian produksi pabrik Honda diperpanjang</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:26:46 +0700</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Ketika produsen mobil besar Jepang seperti Toyota, Nissan, dan Mitsubishi dilaporkan telah kembali memulai produksi ...</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5686271/penghentian-produksi-pabrik-honda-diperpanjang</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/11/06/IMG-20231106-WA0014_copy_2891x2168-01.jpeg</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Laos tetapkan masa berkabung nasional atas meninggalnya ketua parlemen</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:26:46 +0700</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Pemerintah Laos menetapkan masa berkabung nasional selama lima hari untuk menghormati Xaysomphone Phomvihane, ketua ...</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686268/laos-tetapkan-masa-berkabung-nasional-atas-meninggalnya-ketua-parlemen</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2013/12/20131206Laos-ASEAN-001x.jpg</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Kemenhut inisiasi ubah paradigma penegakan hukum terpadu kehutanan</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:21:50 +0700</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Kementerian Kehutanan (Kemenhut) menginisiasi perubahan paradigma penegakan hukum terpadu terkait kehutanan, tumbuhan ...</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686265/kemenhut-inisiasi-ubah-paradigma-penegakan-hukum-terpadu-kehutanan</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/writer_1.jpg</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Mendag: BRICS sepakati mayoritas substansi perdagangan</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:20:09 +0700</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Menteri Perdagangan (Mendag) RI Budi Santoso menyampaikan para menteri perdagangan negara-negara anggota BRICS ...</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686261/mendag-brics-sepakati-mayoritas-substansi-perdagangan</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_1006.jpeg</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Hukum sepekan, pemberantasan korupsi hingga sidang banding Nadiem</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:17:08 +0700</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Beragam berita hukum telah diwartakan Kantor Berita Antara. Berikut kami rangkum lima berita hukum terpopuler dalam ...</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686259/hukum-sepekan-pemberantasan-korupsi-hingga-sidang-banding-nadiem</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/sidang-perdana-banding-vonis-nadiem-makarim-2834681.jpg</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Ekonomi sepekan, harga bensin turun hingga arah insentif EV</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:16:14 +0700</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Berbagai peristiwa ekonomi terjadi selama sepekan (3–8 Agustus), mulai dari penurunan harga bensin pada awal ...</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686257/ekonomi-sepekan-harga-bensin-turun-hingga-arah-insentif-ev</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/20/antisipasi-penyalahgunaan-bbm-bersubsidi-2672569.jpg</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>POPSI nilai tata kelola pembangunan pabrik kelapa sawit perlu dibenahi</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:08:44 +0700</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Perkumpulan Organisasi Petani Kelapa Sawit Indonesia (POPSI) menilai tata kelola pembangunan pabrik kelapa sawit (PKS) ...</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686255/popsi-nilai-tata-kelola-pembangunan-pabrik-kelapa-sawit-perlu-dibenahi</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/22/1001613711.jpg</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Kemenhut berhasil kendalikan karhutla di Sembalun Gunung Rinjani</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:05:01 +0700</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Kementerian Kehutanan melalui Balai Taman Nasional Gunung Rinjani (TNGR) bersama unsur terkait berhasil mengendalikan ...</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686251/kemenhut-berhasil-kendalikan-karhutla-di-sembalun-gunung-rinjani</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/rinjani.jpg</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Bandara Catania di Sisilia ditutup akibat erupsi Gunung Etna</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:02:01 +0700</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Bandar Udara internasional di Kota Catania, Sisilia, Italia, ditutup untuk sementara waktu bagi penerbangan ...</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686249/bandara-catania-di-sisilia-ditutup-akibat-erupsi-gunung-etna</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/12/02/2023-12-01T215111Z_1359423932_RC2HO4A56PY5_RTRMADP_3_ITALY-ETNA.jpg</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan di Kanada paksa lebih dari 20.000 orang mengungsi</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:53:30 +0700</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Lebih dari 20.000 warga mengungsi dari permukiman mereka di dekat Danau Okanagan di British Columbia, Kanada, pada ...</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686248/kebakaran-hutan-di-kanada-paksa-lebih-dari-20000-orang-mengungsi</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/06/01/XxjpbeE007585_20250529_PEPFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Politik sepekan, agenda Presiden hingga ormas kawal program pemerintah</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:48:53 +0700</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Beragam berita politik telah diwartakan Kantor Berita Antara. Berikut kami rangkum lima berita politik terpopuler dalam ...</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686244/politik-sepekan-agenda-presiden-hingga-ormas-kawal-program-pemerintah</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_0992.jpeg</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Christopher Rungkat sebut US Open jadi target utama Aldila SutjiadI</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:45:32 +0700</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Pelatih petenis putri Indonesia Aldila Sutjiadi, Christopher Rungkat, mengatakan rangkaian turnamen lapangan keras di ...</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686240/christopher-rungkat-sebut-us-open-jadi-target-utama-aldila-sutjiadi</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/upscalemedia-transformed-2.jpeg</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Tabrakan kereta di Kroasia, 19 orang terluka</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:38:42 +0700</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Sebuah tabrakan kereta api di wilayah Sveti Ivan Zabno, 65 kilometer dari Zagreb, Kroasia, menyebabkan 19 ...</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686239/tabrakan-kereta-di-kroasia-19-orang-terluka</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2011/10/20111010025.jpg</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Kemenpar dorong yacht tourism perkuat wisata bahari Indonesia</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:35:56 +0700</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Kementerian Pariwisata (Kemenpar) mendorong pengembangan wisata yacht (yacht tourism) untuk memperkuat ekosistem wisata ...</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686237/kemenpar-dorong-yacht-tourism-perkuat-wisata-bahari-indonesia</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-09-at-06.59.48.jpeg</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Gus Kikin paparkan pentingnya Al Qanun Asasi sebagai ruh NU</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:22:42 +0700</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Pengasuh Pondok Pesantren Tebuireng KH. Abdul Hakim Mahfudz menegaskan pentingnya Al-Qanun Al-Asasi sebagai dokumen ...</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686235/gus-kikin-paparkan-pentingnya-al-qanun-asasi-sebagai-ruh-nu</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000177217.jpg</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Ini alasan Pramono bongkar satu JPO viral "Love-Hate" di Rasuna Said</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:18:50 +0700</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung mengungkapkan alasan pembongkaran salah satu jembatan penyeberangan orang (JPO) yang ...</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686231/ini-alasan-pramono-bongkar-satu-jpo-viral-love-hate-di-rasuna-said</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_073343691.jpg</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Menaker: Transformasi Balai K3 garda terdepan cegah kecelakaan kerja</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:17:38 +0700</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Menteri Ketenagakerjaan (Menaker) Yassierli mengatakan transformasi Balai Keselamatan dan Kesehatan Kerja (K3) di ...</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686228/menaker-transformasi-balai-k3-garda-terdepan-cegah-kecelakaan-kerja</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/0ada8d5b-0e63-4beb-8dcc-ffec2308180a.jpeg</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Kemarin, absennya Sophia KATSEYE hingga debut Redmi 17 4G dan 5G</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:12:40 +0700</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Sejumlah berita menarik dari kanal lifestyle, tekno, otomotif dan hiburan pada Sabtu (8/8) masih dapat dibaca kembali ...</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686224/kemarin-absennya-sophia-katseye-hingga-debut-redmi-17-4g-dan-5g</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/InShot_20260808_141122050.jpg</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Psikolog: Perilaku di medsos cerminkan karakter &amp; integritas seseorang</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:11:54 +0700</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Psikolog klinis lulusan Universitas Indonesia (UI) sekaligus Direktur Personal Growth, lembaga yang bergerak di ...</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686223/psikolog-perilaku-di-medsos-cerminkan-karakter-integritas-seseorang</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/11/1001166514.jpg</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Penanganan kubangan akibat gempa di Nokilalaki Sulteng telah rampung</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:10:46 +0700</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Bupati Sigi, Sulawesi Tengah (Sulteng) Moh Rizal Intjenae menyebutkan penanganan seluruh kubangan di Nokilalaki akibat ...</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686221/penanganan-kubangan-akibat-gempa-di-nokilalaki-sulteng-telah-rampung</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/390183.jpg</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Tuide akan debut dengan single berjudul "Sun Kiss"</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:10:00 +0700</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Grup wanita Tuide yang berada di bawah naungan HYBE terafiliasi dengan ABD akan debut dengan membawakan sebuah single ...</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686220/tuide-akan-debut-dengan-single-berjudul-sun-kiss</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-17.52.43.jpeg</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Kemenag segera cairkan Rp4,1 triliun BOS madrasah dan BOP RA tahap II</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:05:02 +0700</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Direktorat Kurikulum, Sarana, Kelembagaan, dan Kesiswaan (KSKK) Madrasah Kementerian Agama (Kemenag) tengah memproses ...</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686217/kemenag-segera-cairkan-rp41-triliun-bos-madrasah-dan-bop-ra-tahap-ii</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000177210.jpg</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Pramono bongkar satu JPO viral "Love-Hate" di Rasuna Said</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:47:37 +0700</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung memutuskan untuk membongkar salah satu Jembatan Penyeberangan Orang (JPO) lama yang ...</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686213/pramono-bongkar-satu-jpo-viral-love-hate-di-rasuna-said</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_073045119.jpg</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Humaniora sepekan, harimau di Aceh Timur hingga target Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:46:02 +0700</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Dalam sepekan, berita humaniora yang mendapat perhatian pembaca dan masih layak untuk kembali disimak lagi, mulai dari ...</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686212/humaniora-sepekan-harimau-di-aceh-timur-hingga-target-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/20260807_161333.jpg</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Dishub DKI Punya Call Center, Bisa Derek Kendaraan-Kawal Mobil Jenazah Gratis</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:43:13 +0700</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Pramono Anung meluncurkan call center Dishub 1500813, menyediakan layanan transportasi darurat, termasuk derek gratis dan pemanduan jenazah.</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610581/dishub-dki-punya-call-center-bisa-derek-kendaraan-kawal-mobil-jenazah-gratis</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/gubernur-dki-jakarta-pramono-anung-saat-peresmian-call-center-dishub-1786243348657_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Polisi Ungkap Pemicu Cekcok Saepul hingga Mutilasi Pria di Depok</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:30:45 +0700</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Saepul (26) membunuh dan memutilasi K (51) di Depok setelah cekcok. Motifnya adalah penolakan hubungan dan niat merampok. Investigasi terus berlanjut.</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610559/polisi-ungkap-pemicu-cekcok-saepul-hingga-mutilasi-pria-di-depok</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/saepul-26-pelaku-mutilasi-pria-inisial-k-di-depok-diperiksa-di-polda-metro-jaya-1786191209681_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Warga Dukung Pembongkaran 1 JPO Viral Dekat tapi Tak Tersambung di Rasuna</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Pramono akan membongkar JPO lama di Jalan HR Rasuna Said yang dekat tapi tak terhubung. Warga setuju rencana Pemprov itu.</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610552/warga-dukung-pembongkaran-1-jpo-viral-dekat-tapi-tak-tersambung-di-rasuna</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/konektivitas-jpo-rasuna-said-disorot-efisiensi-mobilitas-kawasan-bisnis-jadi-sorotan-1785989995417_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Pria di Serang Sayat Leher Istri Usai Korban Minta Cerai</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:13:45 +0700</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Seorang pria di Serang menyayat leher istrinya setelah cekcok soal perceraian. Pelaku ditangkap, dan kasus KDRT ini sedang diselidiki polisi.</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610548/pria-di-serang-sayat-leher-istri-usai-korban-minta-cerai</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2016/08/23/e95af703-19d4-4263-b16f-ca71edd769a2_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Saepul Obral Barang Korban Mutilasi di FB: Motor PCX hingga HP Dijual Murah</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:00:37 +0700</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Polisi ungkap Saepul, pelaku pembunuhan dan mutilasi pria K di Depok. Saepul menjual barang korban di Facebook untuk kebutuhan sehari-hari.</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610540/saepul-obral-barang-korban-mutilasi-di-fb-motor-pcx-hingga-hp-dijual-murah</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-saepul-pelaku-mutilasi-pria-inisial-k-51-di-cipayung-kota-depok-1786188316179_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>MenPPPA Minta Polisi Usut Temuan Senjata di Sekolah, Soroti Kondisi Siswa</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:51:34 +0700</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Menteri PPPA Arifah Fauzi prihatin atas temuan ratusan senjata di sekolah swasta Jakarta. Dia minta kepolisian mengusut tuntas kasus ini demi keamanan anak.</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610534/menpppa-minta-polisi-usut-temuan-senjata-di-sekolah-soroti-kondisi-siswa</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/menteri-pemberdayaan-perempuan-dan-perlindungan-anak-pppa-arifah-fauzi-dokistimewa-1786189553904_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Polisi Ungkap Alasan Saepul Mutilasi Pria di Depok</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:36:17 +0700</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Dasar keahlian itu yang kemudian membuat Saepul nekat memotong tubuh korban usai kebingungan menghilangkan jasad korban K secara utuh.</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610523/polisi-ungkap-alasan-saepul-mutilasi-pria-di-depok</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-saepul-pelaku-mutilasi-pria-inisial-k-51-di-cipayung-kota-depok-1786188316179_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Ini yang Digali Polisi dari Eks Ketua Yayasan soal Temuan Senjata di Sekolah</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:32:32 +0700</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Polisi akan memanggil mantan ketua yayasan sekolah di Jakarta terkait temuan 996 senjata. Penyelidikan dilakukan untuk mengungkap asal dan tujuan penyimpanan.</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610519/ini-yang-digali-polisi-dari-eks-ketua-yayasan-soal-temuan-senjata-di-sekolah</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/kabid-humas-polda-metro-jaya-kombes-budi-hermanto-1786089469648_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Akhir Pelarian Rampok Siang Bolong yang Gondol Duit Puluhan Juta</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:14:49 +0700</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Kawanan perampok di Cibitung, Bekasi, ditangkap setelah menggondol uang puluhan juta. Korban, pegawai koperasi, terluka saat melawan serangan pelaku.</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610512/akhir-pelarian-rampok-siang-bolong-yang-gondol-duit-puluhan-juta</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/perampokan-nasabah-bank-di-siang-bolong-di-cibitung-bekasi-1786238003822_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Detik-detik Gedung Bapenda DKI Kebakaran, Kepulan Asap 'Mengepung' Tiba-tiba</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:11:30 +0700</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda Gedung Bapenda DKI Jakarta, menyebabkan satu pekerja dirawat. Polisi mengungkap kepulan asap 'mengepung' tiba-tiba.</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610509/detik-detik-gedung-bapenda-dki-kebakaran-kepulan-asap-mengepung-tiba-tiba</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-kobaran-api-mengamuk-di-gedung-bapenda-dki-1786160943722_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Sosok Saepul Pelaku Mutilasi: Pernah Masuk TV hingga Dagang Piscok</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:01:07 +0700</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Saepul terlibat dalam kasus pembunuhan dan mutilasi pria K di Depok. Saepul ternyata pernah ikut ajang pencarian bakat dan bekerja sebagai pedagang piscok.</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610502/sosok-saepul-pelaku-mutilasi-pernah-masuk-tv-hingga-dagang-piscok</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/saepul-pelaku-pembunuhan-dan-mutilasi-pria-di-pancoran-mas-depok-ditangkap-subdit-resmob-polda-metro-jaya-1785915706525_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1 JPO Dekat tapi Tak Tersambung di Rasuna Dibongkar, Target Selesai 3 Pekan</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:53:57 +0700</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Proses pembongkaran satu JPO tersebut akan dilakukan di malam hari. Pramono memastikan pembongkaran tidak akan mengganggu jalannya lalu lintas.</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610488/1-jpo-dekat-tapi-tak-tersambung-di-rasuna-dibongkar-target-selesai-3-pekan</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/tak-perlu-putar-jauh-dua-jpo-di-rasuna-said-bakal-terhubung-1785923553622_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Pertamina Ungkap Berbagai Strategi Wujudkan Ketahanan Energi Nasional</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:57:41 +0700</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Pemerintah dan Pertamina berkomitmen untuk ketahanan energi nasional melalui strategi dual growth, mengoptimalkan migas dan mengembangkan energi rendah karbon.</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8610538/pertamina-ungkap-berbagai-strategi-wujudkan-ketahanan-energi-nasional</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kilang-pertamina-1786240625862_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Ekonomi Indonesia: Konduktor, Panglima dan Komando</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:30:46 +0700</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Riant Nugroho</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Dalam praktik pemerintahan modern, keberhasilan ekonomi sering kali tidak ditentukan oleh sistem yang dipilih, melainkan oleh gaya kepemimpinan ekonomi.</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610296/ekonomi-indonesia-konduktor-panglima-dan-komando</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/01/15/masih-dibayangi-pandemi-ekonomi-ri-diprediksi-tumbuh-44-di-2021-2_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Jelang HUT RI, Kostum Pejuang hingga Noni Belanda Laris Disewa</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:30:22 +0700</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Rafida Fauzia</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Permintaan sewa kostum di Malang melonjak jelang HUT ke-81 RI. Penyewaan busana meningkat dua kali lipat menjadi 200 kostum per bulan.</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8610389/jelang-hut-ri-kostum-pejuang-hingga-noni-belanda-laris-disewa</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/jelang-hut-ri-kostum-pejuang-hingga-noni-belanda-laris-disewa-1786207566219.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Tol Jogja-Solo Dibuka Libur Nataru 2027, Begini Progresnya</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:00:21 +0700</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Aulia Damayanti</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Proyek Tol Solo-Yogyakarta-NYIA Kulonprogo (Jogja-Solo) hampir rampung.</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8610250/tol-jogja-solo-dibuka-libur-nataru-2027-begini-progresnya</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/pembangunan-tol-jogja-solo-hampir-rampung-begini-progresnya-1786162440374_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Jakarta Kebakaran, Pramono Anung Pastikan Data Pajak Aman, Sudah Digitalisasi</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:39:46 +0700</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Pramono Anung buka suara terkait kebakaran Gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta yang terjadi Jumat (7/8/2026).</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865910/gedung-bapenda-dki-jakarta-kebakaran-pramono-anung-pastikan-data-pajak-aman-sudah-digitalisasi</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0CAsOgbuZNr9ow6qN43ROkOJbMc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pramono-Anung-bapenda.jpg</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Klasemen Leagues Cup 2026: Tanpa Lionel Messi, Inter Miami Terancam Gagal ke Perempat Final</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:38:01 +0700</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Inter Miami terancam tak lolos ke perempat final Leagues Cup 2026 usai kalah 2-1 dari Monterrey pada matchday kedua.</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865909/klasemen-leagues-cup-2026-tanpa-lionel-messi-inter-miami-terancam-gagal-ke-perempat-final</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/x3mNZJqu4Zy10W-k72JeSd7IQAQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Logo-tim-MLS-Inter-Miami.jpg</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Siapa Febrio Adiono? Sosok yang Antar Sutrimo ke RS Ternyata Eks Ajudan Febrie Adriansyah</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:31:52 +0700</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Febrio Adiono terseret terkait kematian Sutrimo. Dia merupakan eks ajudan dari Febrie Adriansyah. Ia juga yang mengantar Sutrimo ke rumah sakit.</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865908/siapa-febrio-adiono-sosok-yang-antar-sutrimo-ke-rs-ternyata-eks-ajudan-febrie-adriansyah</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/TYMpag4Kl-8VDabiqGKaGE9RBw8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Olah-TKP-Kasus-Tewasnya-Karumga-Sutrimo_1.jpg</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Richard Lee Endus Banyak Kebohongan dari Saksi Dari Doktif, Yakin Bebas dari Jerat Hukum</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:27:23 +0700</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Richard Lee mengendus adanya dugaan kebohongan dalam kasus yang menjeratnya.</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865907/richard-lee-endus-banyak-kebohongan-dari-saksi-dari-doktif-yakin-bebas-dari-jerat-hukum</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/2vW63nHVcL581uBA4ZQTPj4quO4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kontroversi-Doktif-vs-Richard-Lee-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Kota Sorong Akhir Pekan, Minggu 9 Agustus 2026: Cerah di Seluruh Wilayah</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:27:21 +0700</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>BMKG memprakirakan, Kota Sorong, Provinsi Papua Barat Daya bakal cerah pada Minggu (9/8/2026).</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865906/prakiraan-cuaca-kota-sorong-akhir-pekan-minggu-9-agustus-2026-cerah-di-seluruh-wilayah</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/snhhAVeXptZkcESaLrviOJOiojg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Cuaca-cerah-di-Kota-Sorong-232.jpg</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Kepala BPS Jamin Kerahasiaan Data Sensus Ekonomi 2026, Terapkan Sistem Enkripsi</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:19:10 +0700</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>BPS menjamin keamanan data responden Sensus Ekonomi 2026 melalui enkripsi berlapis. BPS juga menggandeng BSSN, Polri, dan Telkom</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865905/kepala-bps-jamin-kerahasiaan-data-sensus-ekonomi-2026-terapkan-sistem-enkripsi</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/F9rZc4PGtQnpYxYHZituBFKuuoA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kepala-BPS-Amalia-Adininggar-Widyasanti-Podcast-di-Tribunnews_20260808_161633.jpg</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Lowongan Kerja Biro Umum Komdigi untuk Lulusan SMA dan S1 Semua Jurusan, Buka 5 Formasi</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:17:26 +0700</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Biro Umum Komdigi buka lowongan kerja sebanyak 3 posisi dengan total kebutuhan 5 orang, terbuka untuk lulusan SLTA/Sederajat dan S1 semua jurusan.</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865904/lowongan-kerja-biro-umum-komdigi-untuk-lulusan-sma-dan-s1-semua-jurusan-buka-5-formasi</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5wbSA5NBy5hb0ApSQYfkujMtjvE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/logo-komdigi-ss.jpg</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Jejak PHK Karyawan Agustus 2026 di Jateng hingga Sulteng, Sasar Sektor Garmen hingga Tambang</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:15:16 +0700</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Pada Agustus 2026 ini, sejumlah perusahaan melakukan pemutusan hubungan kerja (PHK) di Jateng hingga Sulteng.</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865903/jejak-phk-karyawan-agustus-2026-di-jateng-hingga-sulteng-sasar-sektor-garmen-hingga-tambang</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/4mkWJ7DXhUCVZvuupk_1Fw0KgbY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-PHK-1.jpg</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Keluarga Pertanyakan Penyebab Kematian Sutrimo, Awalnya Menerima Kini Tempuh Jalur Hukum</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:12:19 +0700</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Keluarga Sutrimo asal Banyumas lapor polisi, pertanyakan kejanggalan kematian di Jakarta Selatan, tempuh jalur hukum.</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865902/keluarga-pertanyakan-penyebab-kematian-sutrimo-awalnya-menerima-kini-tempuh-jalur-hukum</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/kZFE6PfULAXOD752T0B7EGx5hp4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Rumah-Sutrimo-di-Banyumas-1.jpg</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Penjualan Mobil Elektrifikasi Toyota di GIIAS 2026 Naik Hampir 2 Kali Lipat</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:03:38 +0700</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>SPK kendaraan elektrifikasi Toyota mencapai lebih dari 50 persen, didominasi Innova Zenix, Veloz, dan Yaris Cross Hybrid EV.</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865901/penjualan-mobil-elektrifikasi-toyota-di-giias-2026-naik-hampir-2-kali-lipat</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/RBKOKAP6lEapnyafoJ4pCvQmGwc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Marketing-Director-PT-Toyota-Astra-Motor-Bansar-Maduma-31.jpg</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Koarmada RI Amankan 1.300 Kilogram Diduga Narkotika dari Kapal Berbendera Tanzania</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:58:09 +0700</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Koarmada RI menggagalkan dugaan penyelundupan 1,3 ton ketamine di Bintan. Barang bukti ditemukan dalam 65 karung di kapal MV King Sun</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865900/koarmada-ri-amankan-1300-kilogram-diduga-narkotika-dari-kapal-berbendera-tanzania</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/VzcFCQc2IMkIOdGR40X2tKfLQKo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/narkotikatanzania122.jpg</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Dibantai Chelsea di Indonesia: Pramusim Tanpa Menang, Ujian Sabar AC Milan dengan Ruben Amorim</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:48:14 +0700</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Perjalanan awal karier Ruben Amorim sebagai pelatih baru AC Milan nampaknya belum berjalan mulus.</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865899/dibantai-chelsea-di-indonesia-pramusim-tanpa-menang-ujian-sabar-ac-milan-dengan-ruben-amorim</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/wIj2Ieyz8SVHT4ouMvoXV76dqMU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Chelsea-Bantai-AC-Milan-3-0-di-SUGBK_20260808_235528.jpg</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Orang Tua Wajib Tahu, Ini Tips Mencegah Infeksi Air Kolam Renang saat Liburan</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:44:21 +0700</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Anak-anak rentan terkena infeksi air rekreasi akibat kontaminasi mikroorganisme patogen di kolam renang. Simak tipsnya.</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865898/orang-tua-wajib-tahu-ini-tips-mencegah-infeksi-air-kolam-renang-saat-liburan</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/wOXeAESeLN4Uz28w372Wdaa9FB0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/wisata-ke-kolam-renang-legendaris-karang-setra-waterland_20230518_193034.jpg</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Kanker Prostat Joe Biden Makin Parah, Hunter Biden Sebut Ayahnya Tersiksa: Sangat Menyakitkan</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:43:00 +0700</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Kondisi kesehatan mantan Presiden AS Joe Biden dikabarkan makin memprihatinkan. Sang putra, Hunter Biden sebut kanker prostat ayahnya sudah menyebar.</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865897/kanker-prostat-joe-biden-makin-parah-hunter-biden-sebut-ayahnya-tersiksa-sangat-menyakitkan</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WhS97Ajzfoj3bE4luZGYECKTBv0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/joe-biden-7686.jpg</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Anak 11 Tahun asal India Pecahkan Rekor Dunia Hula Hoop di Sanggul Rambut</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:39:03 +0700</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Anak asal India menyabet gelar Guinness World Records setelah memecahkan rekor putaran hula hoop terbanyak pada sanggul rambut dalam durasi 30 detik.</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865896/anak-11-tahun-asal-india-pecahkan-rekor-dunia-hula-hoop-di-sanggul-rambut</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/c2XGWVEKduD0SQAYhMjCOyRV_oA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/rekor-dunia-hula-hoop-di-sanggul-awokwowkwokwo.jpg</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Kembali Gugat UU ITE, PNS Asal NTT Minta Platform Medsos Verifikasi Identitas Pengguna</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:38:24 +0700</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>PNS NTT Ferdinandus Klau kembali menggugat UU ITE ke MK. Ia meminta platform media sosial diwajibkan memverifikasi identitas asli pengguna</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865895/kembali-gugat-uu-ite-pns-asal-ntt-minta-platform-medsos-verifikasi-identitas-pengguna</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/9oqVKgLejgr4AUtAR9qnfapwJjQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/gedung-mahkamah-konstitusi-gedung-mk-12345.jpg</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Lama Tak Bertemu, Hanya Komunikasi Lewat Chat, Ruben Onsu Makin Rindu Dipanggil ‘Ayah’ oleh Putrinya</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:34:30 +0700</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Ruben Onsu ungkap kerinduannya pada 2 putrinya, buah cintanya dengan Sarwendah. Ia kangen ketika kedua putrinya memanggilnya  'Ayah'.</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865894/lama-tak-bertemu-hanya-komunikasi-lewat-chat-ruben-onsu-makin-rindu-dipanggil-ayah-oleh-putrinya</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/GHpt62tuig514FSTblvdMr1GGQc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ruben-Onsu-ketemu-anak22.jpg</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Prabowo Telah Panggil Sejumlah Kandidat Gubernur BI, Siapa Saja? Berikut Daftar Nama yang Muncul</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:33:29 +0700</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Satu dari sekian nama telah dipanggil Prabowo yaitu Destry Damayanti yang saat ini sebagai Pejabat Gubernur Sementara Bank Indonesia.</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865893/prabowo-telah-panggil-sejumlah-kandidat-gubernur-bi-siapa-saja-berikut-daftar-nama-yang-muncul</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/F0A-gz_PYYWxsd1KxW1nJ6VMlaA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Prabowo-Sidang-Kabinet-aaf.jpg</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>50 Pantun 17 Agustus untuk Memeriahkan HUT RI, Inspiratif hingga Menghibur</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:33:17 +0700</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Simak kumpulan contoh pantun 17 Agustus untuk memeriahkan perayaan HUT RI, ada yang lucu hingga penuh makna.</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865892/50-pantun-17-agustus-untuk-memeriahkan-hut-ri-inspiratif-hingga-menghibur</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iA2C6jPwZkcnpH5GjxixrNuKdck=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/apartemen-kalibata-city-gelar-perlombaan-17-agustusan_20220817_225417.jpg</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Kasus Kematian Sutrimo Dilaporkan ke Bareskrim, Polri Diminta untuk Ekshumasi dan Autopsi</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:31:19 +0700</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Kematian Sutrimo kembali disorot setelah KPI dan keluarga melapor ke polisi. Mereka meminta ekshumasi dan autopsi untuk mencari penyebab kematian</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865891/kasus-kematian-sutrimo-dilaporkan-ke-bareskrim-polri-diminta-untuk-ekshumasi-dan-autopsi</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8pl5ol4WOr7CDkt9Pr-LW4z0KHg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pitra-romadoni-nasution.jpg</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Elon Musk Akan Bangun ‘Raksasa’ Chip AI di Texas, Gedungnya Jadi yang Terbesar Dunia</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:25:21 +0700</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Lida Puspaningtyas</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TEXAS -- Perusahaan milik Elon Musk, SpaceX mengumumkan pekan ini bahwa pabrik semikonduktor yang direncanakan dan diperkirakan akan menjadi gedung terbesar di dunia, dengan luas lebih dari 100...</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhde9502/elon-musk-akan-bangun-raksasa-chip-ai-di-texas-gedungnya-jadi-yang-terbesar-dunia</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/012808200-1702733719-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Perkuat Ekosistem Wisata Bahari, Kemenpar Dorong Yacht Tourism</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:13:17 +0700</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Lida Puspaningtyas</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Kementerian Pariwisata (Kemenpar) mendorong pengembangan wisata yacht (yacht tourism) untuk memperkuat ekosistem wisata bahari Indonesia sekaligus meningkatkan daya saing pariwisata nasional.
+Menteri Pariwisata Widiyanti Putri Wardhana mengatakan wisata...</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhcu5502/perkuat-ekosistem-wisata-bahari-kemenpar-dorong-yacht-tourism</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/beragam-kapal-yacht-tampak-bersandar-di-labuan-bajo-nusa-_191121092347-152.jpg</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Mentan Sebut Pertanian Bisa Jadi Jalan Atasi Kemiskinan di Alor</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:03:00 +0700</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Gita Amanda</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Menteri Pertanian (Mentan) Andi Amran Sulaiman menyebut sektor pertanian bisa menjadi jalan untuk mengatasi kemiskinan di Kabupaten Alor, Nusa Tenggara Timur (NTT). Pemerintah menyiapkan pengembangan pertanian jangka...</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjh8ri423/mentan-sebut-pertanian-bisa-jadi-jalan-atasi-kemiskinan-di-alor</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260809074408-440.png</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Berkat Curhat Mahasiswa, Warga Alor Dapat Bantuan Beras untuk Juli-September 2026</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:25:00 +0700</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Gita Amanda</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Sebanyak 37.338 warga Kabupaten Alor, Nusa Tenggara Timur (NTT), menerima bantuan pangan untuk alokasi Juli, Agustus, dan September 2026. Menteri Pertanian (Mentan) Andi Amran Sulaiman bersama Direktur...</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjh7hu423/berkat-curhat-mahasiswa-warga-alor-dapat-bantuan-beras-untuk-juliseptember-2026</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/menteri-pertanian-mentan-andi-amran-sulaiman-bersama-direktur-utama_260809071638-190.jpg</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Ini Nomor Baru Dishub Jakarta Layani Aduan Jalan</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:57:44 +0700</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Dishub DKI Jakarta meluncurkan Call Center SIAP 1500813, layanan 24 jam untuk aduan transportasi dan lalu lintas.</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265451/ini-nomor-baru-dishub-jakarta-layani-aduan-jalan</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/6uUvWu4cdkuqxQCJ3vfsHSJOEhQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319360/original/021234800_1786244179-493b507a-ec3e-49ca-95c2-7018a9547d82.jpg</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>KPK Geledah 3 Lokasi Usut Suap Proyek di Bengkulu</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:25:43 +0700</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Penggeledahan berlangsung dari hari Rabu, 5 Agustus hingga Jumat, 7 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265438/kpk-geledah-3-lokasi-usut-suap-proyek-di-bengkulu</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/qX7XKsNb9JJUBCFJFaPFXgE0yZ8=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5426450/original/037517400_1764306006-Screenshot_2025-11-28_113148.png</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Teddy Bantah Sekolah Rakyat Tak Bermutu, Sebut 7 Siswa Makassar Juara Olimpiade</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:03:19 +0700</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Total sudah 43.000 anak-anak yang menimba ilmu melalui Sekolah Rakyat.</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265431/teddy-bantah-sekolah-rakyat-tak-bermutu-sebut-7-siswa-makassar-juara-olimpiade</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Su0806dau7fzoTBVeslawBuCcMM=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319321/original/089480100_1786240991-IMG_6871.jpg</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Alasan Pramono Bongkar JPO 'Love-Hate Relationship'</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:48:01 +0700</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Nantinya hanya akan ada satu JPO yang digunakan masyarakat di Rasuna Said.</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265425/alasan-pramono-bongkar-jpo-love-hate-relationship</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/CtO2BnEwrGvJEPxfm-IHuIskBZI=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319310/original/020844600_1786239794-InShot_20260809_073045119.jpg</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>JPO 'Love-Hate Relationship' di Rasuna Said Dibongkar</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:37:52 +0700</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Keputusan itu diambil setelah Pramono bersama jajaran Pemprov DKI mengecek langsung kondisi dua JPO yang lokasinya berdekatan.</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265419/jpo-love-hate-relationship-di-rasuna-said-dibongkar</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/iBV6ZzoMdpqMhCGijXn0cX-hpTs=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319305/original/076111900_1786239435-InShot_20260809_073343691.jpg</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Jorge Messi Wafat, Sosok yang Punya Pengaruh Besar dalam Karier Lionel Messi</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:59:54 +0700</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Kabar duka dari Lionel Messi, sang ayah wafat pada usia 68 tahun, Sabtu (8/8/2026). Sosok yang berpengaruh dalam karier La Pulga.</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>https://bola.kompas.com/read/2026/08/09/09574338/jorge-messi-wafat-sosok-yang-punya-pengaruh-besar-dalam-karier-lionel-messi</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/3KHTHkO2sB8NRqbV3svfqVtS-WU=/49x36:1790x1197/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/08/08/6a7740c1d94fa.jpg</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Kebakaran SPBU Cemplang Bogor Diduga akibat Korsleting Listrik Mobil</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:59:54 +0700</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>SPBU Cemplang Bogor terbakar diduga akibat korsleting listrik mobil, Minggu (9/8/2026). Satu korban luka bakar dan kerugian materil sedang dihitung, SPBU tutup sementara.</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/09/09111051/kebakaran-spbu-cemplang-bogor-diduga-akibat-korsleting-listrik-mobil</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/TqR0QFdWwFoKRAh9NTIwvYsz3x4=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/09/6a77de0216025.jpg</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Long Weekend HUT RI, 6 Wisata Sejarah di Jawa Barat untuk Napak Tilas Perjuangan</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:59:54 +0700</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Jelajahi 6 wisata edukatif di Jawa Barat yang menyimpan jejak perjuangan kemerdekaan, lengkap dengan alamat dan informasi tiket masuk.</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>https://travel.kompas.com/read/2026/08/09/083000327/long-weekend-hut-ri-6-wisata-sejarah-di-jawa-barat-untuk-napak-tilas</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/4HkrwzqLGxQ0UP7TlromdTl4Qyo=/0x5:631x426/1200x675/filters:watermark(data/photo/2026/01/30/697c81889b5f6.png,0,-0,1)/data/photo/2023/05/20/6468f17685f82.png</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I93"/>
+  <autoFilter ref="A1:I172"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 05:45 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$246</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$326</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I246"/>
+  <dimension ref="A1:I326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11996,8 +11996,3768 @@
         </is>
       </c>
     </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Kemenkum Lampung berkomitmen hadirkan pelayanan hukum yang bermanfaat</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:30:45 +0700</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Kantor Wilayah Kementerian Hukum (Kemenkum) Lampung menegaskan komitmennya untuk terus hadir melayani dan memberikan ...</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686399/kemenkum-lampung-berkomitmen-hadirkan-pelayanan-hukum-yang-bermanfaat</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/650341.jpg</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Balon udara bermotif program pemerintah hiasi langit Wonosobo</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:23:25 +0700</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Warga menyaksikan penerbangan balon udara pada Tunas Bumi Fest 2026 di Alun-alun Kota Wonosobo, Jawa Tengah, Minggu ...</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5686395/balon-udara-bermotif-program-pemerintah-hiasi-langit-wonosobo</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/penerbangan-balon-motif-program-prabowo-090826-aez-2.jpg</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Persija akan daratkan tiga pemain pada bursa transfer musim panas ini</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:15:16 +0700</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Persija Jakarta akan mendaratkan dua atau tiga pemain anyar pada bursa transfer musim panas ini untuk memenuhi ...</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686393/persija-akan-daratkan-tiga-pemain-pada-bursa-transfer-musim-panas-ini</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG-20260809-WA0020.jpg</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Jizhou di China perkaya pengalaman wisatawan dengan aktivitas air</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:10:37 +0700</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Dengan memanfaatkan sumber daya alam dan pemandangan pedesaan yang dimilikinya, Distrik Jizhou terus memperluas ...</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686391/jizhou-di-china-perkaya-pengalaman-wisatawan-dengan-aktivitas-air</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/CjkinzN000007_20260809_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>DKI siapkan Gedung Cikini untuk relokasi ASN usai kebakaran Bapenda</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:10:33 +0700</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) DKI Jakarta menyiapkan gedung di kawasan Cikini sebagai lokasi relokasi sementara ...</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686387/dki-siapkan-gedung-cikini-untuk-relokasi-asn-usai-kebakaran-bapenda</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_111043103.jpg</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Takaichi tak singgung "Amerika" di peringatan bom Hiroshima, Nagasaki</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:09:01 +0700</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Perdana Menteri (PM) Jepang Sanae Takaichi kembali tidak menyebut Amerika Serikat sebagai pihak yang bertanggung jawab ...</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686384/takaichi-tak-singgung-amerika-di-peringatan-bom-hiroshima-nagasaki</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/ilustrasi-peringatan-bom-atom-Jepang.jpg</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Pemkab Pati bantu penyerapan garam petani</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:08:09 +0700</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Pemerintah Kabupaten Pati, Jawa Tengah, berkomitmen mengoptimalkan penyerapan garam petani menyusul melimpahnya ...</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686383/pemkab-pati-bantu-penyerapan-garam-petani</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001064358.jpg</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Festival Tari Dug Dug Der Semarangan libatkan 25 ribu peserta</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:08:01 +0700</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Sejumlah penari mementaskan tari dug dug der Semarangan saat mengikuti Festival Tari Dug Dug Der di Lapangan Pancasila ...</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5686380/festival-tari-dug-dug-der-semarangan-libatkan-25-ribu-peserta</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Festival-Tari-Massal-Dug-Dug-Der-Di-Semarang-090826-mz-7.jpg</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>DKI siapkan sistem cadangan lalu lintas imbas kebakaran Bapenda</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:03:49 +0700</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) DKI Jakarta menyiapkan sistem cadangan (backup) untuk mengatur lalu lintas dan menjaga ...</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686379/dki-siapkan-sistem-cadangan-lalu-lintas-imbas-kebakaran-bapenda</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG-20260809-WA0045.jpg</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Pemkot Jaksel targetkan pengerukan saluran PHB Taman Alfa rampung September</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:02:49 +0700</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Administrasi Jakarta Selatan (Pemkot Jaksel) menargetkan pengerukan saluran air penghubung (PHB) Taman ...</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686376/pemkot-jaksel-targetkan-pengerukan-saluran-phb-taman-alfa-rampung-september</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001019550.jpg</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Hunter: Penyakit kanker Joe Biden sudah menyebar ke tulang</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:00:45 +0700</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Kanker prostat yang diderita mantan presiden Amerika Serikat Joe Biden (83) telah menyebar ke titik lain di ...</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686375/hunter-penyakit-kanker-joe-biden-sudah-menyebar-ke-tulang</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/01/02/Joe-Biden-AS.jpg</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Memacu produksi sawit untuk penuhi kebutuhan</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Kementerian Pertanian (Kementan) memacu produksi kelapa sawit nasional untuk memenuhi kebutuhan minyak sawit mentah ...</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5686195/memacu-produksi-sawit-untuk-penuhi-kebutuhan</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/20260809-Memacu-produksi-sawit-untuk-penuhi-kebutuhan.jpg</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Koarmada RI gagalkan penyelundupan 1,3 ton narkoba di perairan Kepri</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:47:48 +0700</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Komando Armada Republik Indonesia (Koarmada RI) menggagalkan upaya penyelundupan narkoba melalui jalur laut di perairan ...</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686371/koarmada-ri-gagalkan-penyelundupan-13-ton-narkoba-di-perairan-kepri</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000582734.jpg</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Baznas bersama Menko PM salurkan bantuan pemberdayaan pesantren Gresik</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:43:16 +0700</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Badan Amil Zakat Nasional (Baznas) bersama Menteri Koordinator Bidang Pemberdayaan Masyarakat (Menko PM) Muhaimin ...</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686367/baznas-bersama-menko-pm-salurkan-bantuan-pemberdayaan-pesantren-gresik</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_20260809_100455.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Pertunjukan Tari Topeng "Gesah Mak Kinang" digelar di Bandung</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:32:42 +0700</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Pertunjukan tari topeng bertema "Gesah Mak Kinang" mengangkat kesenian Topeng Cisalak, yang merupakan seni ...</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686364/pertunjukan-tari-topeng-gesah-mak-kinang-digelar-di-bandung</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/CjkinzN000025_20260806_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Sabalenka tersingkir, Swiatek ke perempat final WTA 1000 Toronto</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:31:14 +0700</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Unggulan teratas Aryna Sabalenka tersingkir dari National Bank Open 2026 setelah dikalahkan Ekaterina Alexandrova dalam ...</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686360/sabalenka-tersingkir-swiatek-ke-perempat-final-wta-1000-toronto</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/05/Sabalenka.jpg</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Pezeshkian sebut Iran siap lanjutkan jalur perdamaian jika AS bangun kepercayaan</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:23:45 +0700</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Presiden Iran Masoud Pezeshkian menyatakan Iran siap melanjutkan jalur perdamaian jika Amerika Serikat membangun ...</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686359/pezeshkian-sebut-iran-siap-lanjutkan-jalur-perdamaian-jika-as-bangun-kepercayaan</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/24/XxjpbeE000177_20260416_PEPFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Pemkab Jayawijaya pertahankan FBLB top 10 KEN</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:16:10 +0700</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Pemerintah Kabupaten (Pemkab) Jayawijaya, Papua Pegunungan memastikan mempertahankan Festival Budaya Lembah ...</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686356/pemkab-jayawijaya-pertahankan-fblb-top-10-ken</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_20260807_122741.jpg</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Kemenpar harap FBLB pertahankan eksistensi nilai budaya Lembah Baliem</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:11:49 +0700</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Kementerian Pariwisata (Kemenpar) RI mengharapkan Festival Budaya Lembah Baliem (FBLB) terus mempertahankan ...</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686352/kemenpar-harap-fblb-pertahankan-eksistensi-nilai-budaya-lembah-baliem</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/MG_7199.jpg</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Pramono Bakal Tambah 1 Peron di Stasiun KRL JIS dalam Waktu Dekat</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:29:50 +0700</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung bakal menambah 1 peron di Stasiun KRL JIS untuk meningkatkan konektivitas. Parkir di Ancol akan dikenakan tarif parkir saja.</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610754/pramono-bakal-tambah-1-peron-di-stasiun-krl-jis-dalam-waktu-dekat</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/29/gubernur-dki-jakarta-pramono-anung-menyampaikan-dukacita-atas-bocah-tewas-usai-terperosok-lubang-di-manggarai-tebet-jaksel-b-b-1782730598311_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Harapan Pramono Usai STY Latih Persija: Mudah-mudahan Musim Ini Juara</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:29:09 +0700</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Pramono Anung optimis Persija juara liga 2026/2027 di bawah pelatih Shin Tae-yong. Dia berharap dukungan warga Jakarta untuk prestasi tim.</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610753/harapan-pramono-usai-sty-latih-persija-mudah-mudahan-musim-ini-juara</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/pramono-1786253227896_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Mobil Terbakar Saat Isi BBM di SPBU Kota Bogor, Sopir Luka di Tangan</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:24:29 +0700</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Muchamad Sholihin</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Sebuah mobil Daihatsu Zebra Espass terbakar di SPBU Cemplang, Bogor. Pengemudi mengalami luka bakar. Kebakaran dipadamkan oleh tim damkar.</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610747/mobil-terbakar-saat-isi-bbm-di-spbu-kota-bogor-sopir-luka-di-tangan</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/satu-unit-mobil-daihatsu-zebra-espass-terbakar-di-area-spbu-cemplang-jalan-brigjen-saptadji-hadiprawira-kecamatan-bogor-barat--1786253051904_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Ledakan yang Renggut Ribuan Nyawa Ini Masih Misterius</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:15:07 +0700</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Rakhmad Hidayatulloh Permana</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Ledakan truk pengangkut dinamit menjadi salah satu sejarah kelam Kolombia. Namun, hingga kini penyebab pasti ledakan masih misterius.</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610639/ledakan-yang-renggut-ribuan-nyawa-ini-masih-misterius</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/ledakan-cali-kolombia-yang-masih-misterius-1786242196075_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Polisi Dalami Identitas Febrio Adiono Terkait Kematian Sutrimo</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:04:49 +0700</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Staf Kejagung, Febrio Adiono, terlibat dalam kasus kematian Sutrimo yang mencurigakan. Polisi akan ekshumasi jasad untuk menyelidiki penyebabnya.</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610736/polisi-dalami-identitas-febrio-adiono-terkait-kematian-sutrimo</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/10/kabid-humas-1778386254900_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Polisi Segera Ekshumasi Jasad Sutrimo untuk Usut Penyebab Kematian</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:46:59 +0700</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Polisi akan ekshumasi jenazah Sutrimo, pria yang ditemukan meninggal di depan klinik kecantikan. Kematian dianggap tidak wajar dan penyelidikan berlanjut.</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610711/polisi-segera-ekshumasi-jasad-sutrimo-untuk-usut-penyebab-kematian</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/08/kabid-humas-polda-metro-jaya-kombes-budi-hermanto-devi-pdetikcom-1783524812593_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>PKS Dukung Prabowo Jika Rekrut Orang Baru di Kabinet: Tak Harus dari Partai</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:26:55 +0700</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Dwi Rahmawati</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Mardani PKS dukung jika Presiden mau rekrut orang baru di kabinet. Pihaknya tak masalah jika bukan dari orang partai.</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610695/pks-dukung-prabowo-jika-rekrut-orang-baru-di-kabinet-tak-harus-dari-partai</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/10/07/mardani-ali-sera-wildandetikcom_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Saepul Pemutilasi Pria di Depok Dijerat Pasal Pembunuhan Berencana</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:22:35 +0700</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Saepul ditetapkan sebagai tersangka pembunuhan dan mutilasi pria K di Depok. Motifnya adalah merampok sepeda motor korban setelah melihat foto di media sosial.</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610682/saepul-pemutilasi-pria-di-depok-dijerat-pasal-pembunuhan-berencana</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-saepul-pelaku-mutilasi-pria-inisial-k-51-di-cipayung-kota-depok-1786188316179_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Polisi Sebut Saepul Pemutilasi Pria di Depok Gabung 5 Grup LGBT di Medsos</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:19:46 +0700</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Polisi ungkap Saepul (26) membunuh dan memutilasi K (51) setelah ditolak berhubungan. Saepul tergabung dalam lima grup LGBT di media sosial.</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610679/polisi-sebut-saepul-pemutilasi-pria-di-depok-gabung-5-grup-lgbt-di-medsos</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-saepul-pelaku-mutilasi-pria-inisial-k-51-di-cipayung-kota-depok-1786188316179_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Deposit Judol Saat Piala Dunia Tembus Rp 1,02 Triliun!</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:28:05 +0700</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>PPATK mencatat deposit judi online (judol) terkait gelaran Piala Dunia mencapai Rp 1,02 triliun untuk 6.001.352 transaksi.</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610739/deposit-judol-saat-piala-dunia-tembus-rp-1-02-triliun</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/07/20/ilustrasi-judi-online-lagi_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Harga Emas Antam Naik Setinggi Ini dalam Sepekan</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:43:18 +0700</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Harga emas Antam menguat sepanjang perdagangan sepekan terakhir.</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610707/harga-emas-antam-naik-setinggi-ini-dalam-sepekan</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/10/22/harga-emas-terjun-bebas-pasar-cikini-langsung-diserbu-pembeli-1761123863171_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Kemenko Pangan Dorong Teknologi Pirolisis untuk Olah Sampah Jadi Energi</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:41:30 +0700</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Rahmat Khairurizqi</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Kementerian Koordinator Bidang Pangan dorong teknologi pirolisis untuk pengelolaan sampah. Ini solusi untuk mengolah sampah jadi energi terbarukan di Indonesia.</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610705/kemenko-pangan-dorong-teknologi-pirolisis-untuk-olah-sampah-jadi-energi</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kemenko-pangan-dorong-teknologi-pirolisis-untuk-olah-sampah-jadi-energi-1786250430758_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Buruan ke Transmart Full Day Sale, Beli Rak Besi Dapat Diskon Segede Ini</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:00:30 +0700</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Beli rak besi di Transmart Full Day Sale dapat potongan diskon gede-gedean.</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610626/buruan-ke-transmart-full-day-sale-beli-rak-besi-dapat-diskon-segede-ini</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/transmart-full-day-sale-1786245759545_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Ercel Rulista Debut Lewat Kita Satu Genk</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:12:33 +0700</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>prih febriani</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Ercel Rulista debut dengan lagu Kita Satu Genk. Ia mengekspresikan diri dan didukung penuh orang tua. Lagu ini merayakan pertemanan dan penerimaan.</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/music/d-8610741/ercel-rulista-debut-lewat-kita-satu-genk</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/ercel-rulista-1786250008823_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Christian Sugiono Santai Lihat Anak Masuk Masa Puber</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:34:45 +0700</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Christian Sugiono santai hadapi masa puber anaknya, Juna. Ia percaya edukasi di sekolah membantu anak memahami perubahan alami saat remaja.</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610701/christian-sugiono-santai-lihat-anak-masuk-masa-puber</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/11/momen-arjuna-anak-titi-kamal-christian-sugiono-lulus-sd-intip-potret-bahagianya-1781172928869_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Soal Kemungkinan Ruben Onsu Menangkan Gugatan Hak Asuh, Praktisi Hukum Soroti Alasan dan Bukti Kuat</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:14:45 +0700</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Praktisi hukum ungkap kemungkinan Ruben Onsu memenangkan hak asuh anak melawan Sarwendah. Singgung soal alasan dan bukti yang kuat.</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865953/soal-kemungkinan-ruben-onsu-menangkan-gugatan-hak-asuh-praktisi-hukum-soroti-alasan-dan-bukti-kuat</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ZG3_PDED1CjlCCKn-J5WB8tswOA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ruben-Onsu-KPAI.jpg</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Jalur Ekstrem Gunung Piramid Makan Korban, APGI Desak Pengelolaan Profesional</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:14:43 +0700</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Dua pendaki, Maliya Finda (51) asal Surabaya dan Irfan Nazrul Laili (35) warga Desa Traktakan, Bondowoso, ditemukan meninggal dunia di Gunung Piramid.</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865952/jalur-ekstrem-gunung-piramid-makan-korban-apgi-desak-pengelolaan-profesional</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/UxYvobAAvImNWul8zOb6NExL7_w=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Jalur-Ekstrem-Gunung-Piramid-Makan-Korban-APGI-Desak-Pengelolaan-Profesional.jpg</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Sinopsis Drama China Ren Yu atau Mermaid 2026, Misteri Hilangnya Gadis dan Kasus Kriminal</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:14:10 +0700</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Drama China Ren Yu aka Mermaid 2026 mengisahkan hilangnya Su Lin yang ternyata berkaitan dengan kasus tiga mayat perempuan di sungai bawah tanah.</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865951/sinopsis-drama-china-ren-yu-atau-mermaid-2026-misteri-hilangnya-gadis-dan-kasus-kriminal</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/741UGGMgGbJJbaYqHX_Ljju216w=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Film-Bioskop-Ilustrasi.jpg</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Bergabung di Formas, Gapempi Tekankan Pentingnya Daya Saing Industri Hadapi Ekonomi Global</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:09:22 +0700</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Penguatan daya saing industri nasional dinilai penting agar Indonesia mampu menghadapi persaingan ekonomi global.</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865950/bergabung-di-formas-gapempi-tekankan-pentingnya-daya-saing-industri-hadapi-ekonomi-global</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/RKVIF3CPPMBcVdcURCUkS38Se0A=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Minarni-Panggabean-1.jpg</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Pentagon Gerak Cepat! Produksi Senjata AS Dikebut 21 Hari usai Isu Krisis Amunisi Mencuat</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:07:16 +0700</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Pentagon gerak cepat! Industri pertahanan AS diberi tenggat 21 hari untuk kebut produksi senjata usai isu krisis amunisi mencuat.</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865949/pentagon-gerak-cepat-produksi-senjata-as-dikebut-21-hari-usai-isu-krisis-amunisi-mencuat</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ZxpCvNmdZFG3Ya0U1zvSQDTzLyc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bom-militer-AS-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Pelaku Mutilasi di Depok Akui Pernah Berkata Ingin Dapat Motor dengan Cara Membunuh</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:06:17 +0700</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Saepul akui membunuh Kusnaefi demi kuasai motor Honda PCX, polisi dalami pengakuan dan kronologi mutilasi di Depok.</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865948/pelaku-mutilasi-di-depok-akui-pernah-berkata-ingin-dapat-motor-dengan-cara-membunuh</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/uZv_LaESzB4DG7o2f7QLFP7w1UY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pencarian-kaki-korban-mutilasi-di-Depok-Jawa-Barat.jpg</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Kunci Gitar Lagu Petal - Ariana Grande: I Hear Them All Say, Ooh, ooh</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:48:34 +0700</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Simak kunci gitar dan lirik lagu Petal yang dinyanyikan oleh Ariana Grande dalam artikel berikut ini.</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7865947/kunci-gitar-lagu-petal-ariana-grande-i-hear-them-all-say-ooh-ooh</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/CL9ms16FPIIxTCUp0D3p9YN4Z0w=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-musik-upgrade-fm.jpg</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Kesaksian Doktif Dinilai Menguntungkan, Tim Richard Lee Siapkan 95 Pertanyaan untuk Sidang Lanjutan</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:42:25 +0700</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Richard Lee justru menilai keterangan yang disampaikan Doktif di hadapan majelis hakim memberikan keuntungan bagi kubu mereka.</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865946/kesaksian-doktif-dinilai-menguntungkan-tim-richard-lee-siapkan-95-pertanyaan-untuk-sidang-lanjutan</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/49t7p74f0-xwxuX8XA2CXTxlPLc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kolase-Dokter-Amira-Farahnaz-alias-Doktif-Polres-Metro-Jakarta-Selatan-Richard-Lee.jpg</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Kronologi Tewasnya Sutrimo Menurut Febrio Adiono: Sempat Mengeluh Sakit, saat Disusul Sudah Pingsan</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:42:00 +0700</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Kematian Sutrimo, Karumga eks Jampidsus Febrie Adriansyah, masih menyisakan tanda tanya.</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865945/kronologi-tewasnya-sutrimo-menurut-febrio-adiono-sempat-mengeluh-sakit-saat-disusul-sudah-pingsan</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/32rVEil1UZlcOjSPVPvrSrxuK9c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Klinik-tempat-Sutrimo-ditemukan-tewas.jpg</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu I Lay My Love on You - Westlife: Just a Smile and The Rain is Gone</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:39:18 +0700</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Simak lirik dan terjemahan lagu I Lay My Love on You yang dipopulerkan oleh grup musik Westlife.</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7865944/terjemahan-lirik-lagu-i-lay-my-love-on-you-westlife-just-a-smile-and-the-rain-is-gone</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zLN77GXG_MWcQ27NDqNvGgp-QJs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-musik-ilustrasi-lirik-ilustrasi-terjemahan-lirik-lagu.jpg</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban IPS Kelas 10 SMA Kurikulum Merdeka Halaman 145 Edisi Revisi: Pengayaan</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:35:23 +0700</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Berikut ini kunci jawaban IPS kelas 10 SMA Kurikulum Merdeka Halaman 145 Edisi Revisi: Pengayaan.</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865943/kunci-jawaban-ips-kelas-10-sma-kurikulum-merdeka-halaman-145-edisi-revisi-pengayaan</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/DSga7wM08_0kQh0WIsFqhAjs6F8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Simak-kunci-jawaban-Informatika-Kelas-5-Halaman-139.jpg</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Lumba-lumba 80 Kg Mati Terdampar di Pantai Timur Pangandaran, Dievakuasi Petugas</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:33:55 +0700</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Lumba-lumba seberat 80 Kg ditemukan terdampar di Pantai Timur Pangandaran, Jawa Barat, Sabtu (8/8/2026) pagi.</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865942/lumba-lumba-80-kg-mati-terdampar-di-pantai-timur-pangandaran-dievakuasi-petugas</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/761v1mORgSW6CYvfnlbkwDeInoI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/hiu-terdampar-4.jpg</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Jakarta Kebakaran, Pramono Anung Pindahkan Tempat Kerja Ribuan ASN ke Cikini</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:33:44 +0700</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Seribu ASN yang bekerja di Gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta, usai kebakaran hebat pada Jumat (7/8/2026) malam.</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865941/gedung-bapenda-dki-jakarta-kebakaran-pramono-anung-pindahkan-tempat-kerja-ribuan-asn-ke-cikini</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/W9SHOqGhp7bj-avPCZWsw2q4wt4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/api-membara-di-gedung-bapenda-dki-jakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Iuran BPJS Kesehatan Pengurus Kopdes Merah Putih Bukan dari APBN, Bagaimana dengan Gaji?</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:29:40 +0700</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>BPJS Kesehatan menegaskan pengurus dan manajer Kopdes Merah Putih bukan berasal dari APBN, namun dengan skema potongan gaji.</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865940/iuran-bpjs-kesehatan-pengurus-kopdes-merah-putih-bukan-dari-apbn-bagaimana-dengan-gaji</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/C6L5CH9NnUo38tihcoKQQ6Irfi0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/KDKMP-Koperasi-Desa-Merah-Putih-Kopdes-Merah-Putih.jpg</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Tak Sekadar Berakting, Jerome Kurnia Ingin Terlibat Lebih Dalam di Belakang Layar</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:25:04 +0700</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Jerome Kurnia kembali dipercaya memerankan karakter Romo Thomas dalam film horor eksorsisme Kuasa Gelap: Perjanjian Darah.</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865939/tak-sekadar-berakting-jerome-kurnia-ingin-terlibat-lebih-dalam-di-belakang-layar</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/lDNppR1fWKvUMHX27AhmPdEwNbI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/jerome-kurnia-produser.jpg</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban Bahasa Indonesia Kelas 12 Halaman 31, Ayo Berlatih</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:11:22 +0700</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Berikut kunci jawaban Bahasa Indonesia kelas 12 halaman 31 Kurikulum Merdeka, Ayo Berlatih.</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865938/kunci-jawaban-bahasa-indonesia-kelas-12-halaman-31-ayo-berlatih</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/XhBRIz0w6j4a0Am_HhX9naYOyXU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/siswa-SMA-MPLS-2.jpg</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Selain di Gunung Gede Pangrango, Kebakaran Melanda Kawasan Bromo, Akses Wisata Ditutup</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:10:37 +0700</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Buntut kebakaran, seluruh akses wisata Gunung Bromo mulai Sabtu (8/8/2026) pukul 22.00 WIB hingga waktu yang belum ditentukan.</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/ramadan/7865937/selain-di-gunung-gede-pangrango-kebakaran-melanda-kawasan-bromo-akses-wisata-ditutup</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/j2S7gAqYm6hUyXDc9EsEv3NLcUc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Karhutla-Bromo-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>HP Sutrimo Tidak Diketahui, Keluarga Cuma Terima KTP hingga Uang Santunan Rp20 Juta</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:09:09 +0700</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Keluarga justru tidak menerima ponsel milik Sutrimo pasca jenazahnya diterima. Keluarga hanya menerima KTP hingga uang santunan.</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865936/hp-sutrimo-tidak-diketahui-keluarga-cuma-terima-ktp-hingga-uang-santunan-rp20-juta</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/CawjQmYsx6SChqFOdefPkSh2M4U=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kematian-Sutrimo-Dilaporkan-ke-Polisi-oleh-Keluarga.jpg</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban IPS Kelas 10 SMA Kurikulum Merdeka Halaman 140 Edisi Revisi: Aktivitas 3.3</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:07:03 +0700</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Berikut ini kunci jawaban IPS kelas 10 SMA Kurikulum Merdeka Halaman 140 Edisi Revisi: Aktivitas 3.3.</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865935/kunci-jawaban-ips-kelas-10-sma-kurikulum-merdeka-halaman-140-edisi-revisi-aktivitas-33</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/U9U0Ezm2sPloSaaCbS7kqX3m2cw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/suasana-hari-pertama-pembelajaran-tatap-muka-ptm-terbatas-di-kota-bogor-senin-18102021.jpg</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Potret Rapat DPR Kosovo Ricuh, Cekcok Berujung Lempar Telur</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:20:32 +0700</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Rapat parlemen Kosovo ricuh setelah anggota oposisi melempar telur ke Albin Kurti yang meminta tambahan waktu untuk membentuk pemerintahan.</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260809104904-7-757704/potret-rapat-dpr-kosovo-ricuh-cekcok-berujung-lempar-telur</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/09/anggota-parlemen-kosovo-time-kadriaj-melemparkan-telur-ke-arah-perdana-menteri-albin-kurti-tidak-terlihat-dalam-foto-saat-sida-1786247238587_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Video: Gak Cuma Sekedar Sikat Gigi, Perhatikan Kandungan Pasta Gigi</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:00:36 +0700</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia TV</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Gak Cuma Sekedar Sikat Gigi, Perhatikan Kandungan Ini di Pasta Gigi Kalian</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260804114058-8-756361/video-gak-cuma-sekedar-sikat-gigi-perhatikan-kandungan-pasta-gigi</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/04/gak-cuma-sekedar-sikat-gigi-perhatikan-kandungan-ini-di-pasta-gigi-kalian-1785823034585_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Produsen Makanan Thailand Pusing Gara-Gara Aturan Pemerintah RI</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:45:35 +0700</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Elga Nurmutia</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Eksportir makanan Thailand diminta meninjau sertifikasi produk sebelum 17 Oktober 2026, seiring RI memperluas ketentuan halal. Persiapkan dokumen dan standar!</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260809101235-4-757701/produsen-makanan-thailand-pusing-gara-gara-aturan-pemerintah-ri</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/03/15/stiker-halal-yang-tertempel-di-pintu-masuk-salah-satu-restoran-siap-saji-di-salemba-jakarta-jumat-1532024-badan-penyelenggara--1_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Video: Ekspansi Kapal Perang Buatan RI, Siap Ekspor ke Filipina - UEA</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:00:03 +0700</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Ekspansi Kapal Perang Made in Indonesia, Siap Ekspor ke Filipina - Uni Emirat Arab</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260803171603-8-756193/video-ekspansi-kapal-perang-buatan-ri-siap-ekspor-ke-filipina--uea</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/04/ekspansi-kapal-perang-made-in-indonesia-siap-ekspor-ke-filipina-uni-emirat-arab-1785809228719_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Blak-blakan! Hunter Biden Akui Kontroversi Pengampunan Joe Biden</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 10:45:45 +0700</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Romys Binekasri</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Hunter Biden mengakui kontroversi pengampunan hukum dari ayahnya, Joe Biden. Ia juga berbicara tentang kecanduan dan kesehatan sang ayah.</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260809082953-4-757699/blak-blakan-hunter-biden-akui-kontroversi-pengampunan-joe-biden</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2023/06/21/hunter-biden-2_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Harta Karun Langka RI, Harganya Bisa Tembus Rp18 Miliar per Ton</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 10:30:30 +0700</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Berikut jenis logam tanah jarang di Indonesia yang memiliki harga selangit.</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260809074233-4-757697/harta-karun-langka-ri-harganya-bisa-tembus-rp18-miliar-per-ton</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/08/25/neodymium-1756109326869_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Video: Tarik Investasi Asing di Tengah Gejolak, DPR Dukung Bentuk PFII</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 10:00:52 +0700</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Tarik Investasi Asing di Tengah Gejolak, DPR Dukung Pembentukan PFII</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260806152635-8-757167/video-tarik-investasi-asing-di-tengah-gejolak-dpr-dukung-bentuk-pfii</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/06/tarik-investasi-asing-di-tengah-gejolak-dpr-dukung-pembentukan-pfii-1786006125297_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Bukan 16 Juta per Bulan, Segini Gaji Manajer Kopdes Menurut Purbaya</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:45:11 +0700</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Program Koperasi Desa Merah Putih (KDMP) jadi sorotan setelah kabar gaji manajernya Rp 16 juta. Menteri Keuangan bantah dan sebut gaji lebih rendah dari UMP.</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260809073811-4-757696/bukan-16-juta-per-bulan-segini-gaji-manajer-kopdes-menurut-purbaya</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/03/menteri-keuangan-purbaya-yudhi-sadewa-saat-konferensi-pers-hasil-rapat-berskla-kssk-iii-tahun-2016-di-jakarta-senin-382026-1785751135196_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Uang Pensiun PNS Bisa Tembus Rp1 M, Ini Penjelasannya</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:15:55 +0700</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Romys Binekasri</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Kepala BKN Zudan Arif Fakrulloh membagikan tips meraih dana pensiun Rp 1 miliar bagi ASN melalui disiplin menabung dan investasi. Temukan strategi optimalnya!</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260809070955-4-757691/uang-pensiun-pns-bisa-tembus-rp1-m-ini-penjelasannya</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2018/08/17/1633dc04-d1c2-422f-aea4-b4c4a0ae2b61_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Spanyol-Italia Memanas, Turis Italia Mendadak Diperiksa</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:46:15 +0700</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Spanyol memberlakukan pemeriksaan acak bagi pelancong dari Italia di tengah perselisihan kedua negara terkait migrasi dan kontrol perbatasan.</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808193425-7-757667/spanyol-italia-memanas-turis-italia-mendadak-diperiksa</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/petugas-kepolisian-nasional-spanyol-memeriksa-dokumen-para-pelancong-yang-tiba-dari-italia-di-bandara-madrid-barajas-madrid-sp-1786192857705_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>PCPM Bank Indonesia Dibuka Hari Ini, Ini Syarat dan Linknya!</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:40:06 +0700</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>haa</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Bank Indonesia membuka pendaftaran lowongan kerja PCPM untuk lulusan S1 dan S2 hingga 14 Agustus 2026. Daftar secara online di situs resmi BI.</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260809062605-4-757687/pcpm-bank-indonesia-dibuka-hari-ini-ini-syarat-linknya</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2018/04/05/2fefffec-bee3-4f59-b957-3c879483222a_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Trump Mau Investasi Rp54,26 T di Proyek Mineral Kritis, Ini Alasannya</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:20:44 +0700</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Pemerintah AS menginvestasikan US$3 miliar untuk proyek mineral kritis dan baterai, mendukung industri dalam negeri dan ketahanan nasional, kata Trump.</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260809055044-4-757686/trump-mau-investasi-rp5426-t-di-proyek-mineral-kritis-ini-alasannya</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/04/presiden-as-donald-trump-menari-saat-menyampaikan-pidato-tentang-perekonomian-di-general-motors-proving-ground-di-milford-mich-1785832321413_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Terbakar, Pramono: Data Pajak Jakarta Aman</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 07:00:10 +0700</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda Gedung Dinas Teknis Bapenda DKI Jakarta, namun data perpajakan aman. Gubernur Pramono pastikan pelayanan publik tetap normal.</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260809053915-4-757685/gedung-bapenda-dki-terbakar-pramono-data-pajak-jakarta-aman</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/petugas-penanggulangan-kebakaran-dan-penyelamatan-gulkarmat-memasuki-gedung-badan-pendapatan-daerah-bapenda-dki-jakarta-setela-1786171326942_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Selat Hormuz Memanas, Kapal Minyak UEA Diserang Saat Melintas</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:40:11 +0700</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Perusahaan minyak ADNOC melaporkan serangan rudal di Selat Hormuz. Iran menegaskan pembukaan kembali selat tergantung pada syarat yang diajukan.</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808214611-4-757684/selat-hormuz-memanas-kapal-minyak-uea-diserang-saat-melintas</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/16/pergerakan-kapal-di-selat-hormuz-16-juli-2026-1784170047813_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Pemerintah Cari Pajak Baru, Rumah Kontrakan Bakal Dikenakan</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 06:00:30 +0700</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Pemerintah akan memperluas basis perpajakan, fokus pada wajib pajak dengan lebih dari satu properti.</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808213343-4-757683/pemerintah-cari-pajak-baru-rumah-kontrakan-bakal-dikenakan</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/09/26/ilustrasi-pajak_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Bos Danantara Bocorkan Soal Streamlining BUMN, 652 Perusahaan Dihapus</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:40:37 +0700</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>BP BUMN dan BPI Danantara mempercepat transformasi dengan memangkas 652 perusahaan pelat merah, menyisakan 250.</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260809113237-17-757713/bos-danantara-bocorkan-soal-streamlining-bumn-652-perusahaan-dihapus</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/23/kepala-bp-bumn-sekaligus-coo-danantara-indonesia-dony-oskaria-menggelar-pertemuan-bersama-direktur-utama-pt-sucofindo-rabu-227-1784802380001_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Petani Kelapa Sawit RI Menangis, Ada Bencana Depan Mata</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:15:32 +0700</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Aktivitas panen kelapa sawit di Kalimantan dan Sumatra terganggu akibat kenaikan harga bahan bakar dan kelangkaan pasokan, mengancam produksi CPO global.</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260809100832-17-757700/petani-kelapa-sawit-ri-menangis-ada-bencana-depan-mata</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/09/24/petani-sawit-1758698548293_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Prabowo Panggil Banyak Sosok untuk Calon Gubernur BI, Siapa Saja?</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 08:15:40 +0700</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Posisi Gubernur Bank Indonesia kosong setelah Perry Warjiyo. Mensesneg Prasetyo Hadi ungkap Presiden Prabowo siapkan beberapa nama pengganti.</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260809063221-17-757688/prabowo-panggil-banyak-sosok-untuk-calon-gubernur-bi-siapa-saja</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/06/pertemuan-presiden-ri-dengan-150-periset-dari-badan-riset-dan-inovasi-nasional-6-agustus-2026-1786010089825_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Ini Dia 'Sosok Pengganti' Debt Collector</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:30:30 +0700</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Teknologi AI kini digunakan dalam penagihan utang, menggantikan peran manusia. Meskipun efisien, tantangan akurasi data dan keadilan tetap ada.</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260809072730-37-757695/ini-dia-sosok-pengganti-debt-collector</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2023/11/14/ojk-atur-cara-dan-larangan-tagih-utang-pinjol_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Langkah BYD Indonesia Bangun Ekosistem Kendaraan Energi Baru Bersama Beyond Community</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:18:56 +0700</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG — Sederet bangku berwarna transparan tersusun di depan panggung utama booth BYD Indonesia di Hall 10B ICE BSD City, Tangerang. Puluhan orang berkemeja biru dongker bertuliskan Beyond Community...</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhlfk348/langkah-byd-indonesia-bangun-ekosistem-kendaraan-energi-baru-bersama-beyond-community</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260809115430-701.png</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Sebut Penghasilan Danantara Naik 400 Persen, Prabowo: Perlu Diaudit</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 11:53:28 +0700</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Lida Puspaningtyas</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Presiden Prabowo Subianto meminta peningkatan kinerja Badan Pengelola Investasi Daya Anagata Nusantara (Danantara) terus diaudit dan diverifikasi. Permintaan itu disampaikan setelah dirinya menerima laporan adanya lonjakan penghasilan...</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhk94502/sebut-penghasilan-danantara-naik-400-persen-prabowo-perlu-diaudit</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/presiden-prabowo-bersama-menteri-esdm-bahlil-lahadalia-menteri_260709213755-839.jpeg</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Punya Sertifikat Pramuka Garuda, Belum Tentu Lulus Jadi Polisi</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:18:00 +0700</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Proses seleksi anggota Polri sangat ketat dan sesuai regulasi. Sertifikat Pramuka Garuda hanya dokumen pendukung.</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265524/punya-sertifikat-pramuka-garuda-belum-tentu-lulus-jadi-polisi</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/w3EJjZLnVfPOa-oau3W-jrvVLrE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5574748/original/059217200_1777975442-IMG-20260504-WA0021.jpg</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Keluarga Minta Polisi Ungkap Penyebab Kematian Sutrimo</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:15:24 +0700</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Laporan tersebut diambil setelah pihak keluarga mempertimbangkan sejumlah informasi yang berkembang.</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265523/keluarga-minta-polisi-ungkap-penyebab-kematian-sutrimo</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/-fx7HAZbdkTLuLva3_Hw8lwALys=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9308334/original/005435400_1785137531-64336.jpg</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Ajakan Hubungan Intim di Balik Kasus Mutilasi Depok</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:06:10 +0700</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Pelaku sempat mengajak korban berhubungan sesama jenis.</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265506/ajakan-hubungan-intim-di-balik-kasus-mutilasi-depok</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/3_XSuRpVsw7mR1OINb8kGSne_JA=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9316566/original/060113700_1785945727-WhatsApp_Image_2026-08-05_at_22.56.47.jpeg</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Money</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Triwulan II 2026: Siapa Penikmat Cuan Pertumbuhan?</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:45:41 +0700</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Salah satu wajah ekonomi Indonesia yang sedang berubah: pertumbuhan tidak selalu membawa lebih banyak orang ke dalam pasar kerja.</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/08/09/124500826/triwulan-ii-2026--siapa-penikmat-cuan-pertumbuhan-</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/LCeqxCE6TPMUk1lPykkKVOU2Zww=/0x0:5000x3333/1200x675/filters:watermark(data/photo/2026/01/30/697c815e7ef28.png,0,-0,1)/data/photo/2026/08/09/6a77d5c6cf862.jpg</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Kebiasaan Flossing Gigi Bisa Perpanjang Umur, Begini Penjelasan Dokter</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:45:41 +0700</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Membersihkan sela gigi dengan benang, alias flossing, rupanya efektif mencegah penyakit mematikan dan mencapai umur panjang.</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>https://lifestyle.kompas.com/read/2026/08/09/120500420/kebiasaan-flossing-gigi-bisa-perpanjang-umur-begini-penjelasan-dokter</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/DrI40PyoKgbG-VkPHX1NvWzFKD4=/105x0:2444x1559/1200x675/filters:watermark(data/photo/2026/01/30/697c817ed68bb.png,0,-0,1)/data/photo/2026/07/03/6a47b13b355c4.jpg</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>5 Makanan Populer Era 70-an yang Kini Dilarang, Ada Soda hingga Seafood</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:45:41 +0700</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Lima makanan yang populer pada era 1970-an kini dilarang atau dibatasi karena alasan kesehatan, keamanan pangan, dan kelestarian lingkungan.</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/food/read/2026/08/09/113000075/5-makanan-populer-era-70-an-yang-kini-dilarang-ada-soda-hingga-seafood</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/hbonrSMnCfKukAGX7UKqxyThuhw=/0x0:2392x1595/1200x675/filters:watermark(data/photo/2026/01/30/697c81a417f45.png,0,-0,1)/data/photo/2026/08/03/6a70898f2278e.jpg</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I246"/>
+  <autoFilter ref="A1:I326"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 06:39 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$326</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$378</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I326"/>
+  <dimension ref="A1:I378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -15756,8 +15756,2452 @@
         </is>
       </c>
     </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Festival balon udara Asta Cita hiasi langit Wonosobo</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:31:55 +0700</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>ANTARA -Festival balon udara bertajuk Asta Cita Presiden Prabowo Subianto menghiasi langit Alun-Alun Kabupaten ...</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686409/festival-balon-udara-asta-cita-hiasi-langit-wonosobo</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AYM_FESTIVAL-BALON-UDARA-ASTA-CITA.jpg</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>TNI AL gagalkan penyelundupan 1,3 ton ketamin dari Kapal MV King Sun</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:23:57 +0700</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>TNI Angkatan Laut bersama tim gabungan menggagalkan upaya penyelundupan narkotika jenis ketamin seberat 1.298 kilogram ...</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686443/tni-al-gagalkan-penyelundupan-13-ton-ketamin-dari-kapal-mv-king-sun</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_1652.jpeg</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Lebih dari 40.000 jiwa terdampak banjir imbas tanggul jebol di Myanmar</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:20:56 +0700</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Lebih dari 40.000 orang terdampak banjir pada 30 Juli hingga 7 Agustus setelah tanggul Sungai Ngawun jebol di daerah ...</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686439/lebih-dari-40000-jiwa-terdampak-banjir-imbas-tanggul-jebol-di-myanmar</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/CjkinzN000010_20260809_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Hunian impian tertunda, kepercayaan konsumen dipertaruhkan</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:20:31 +0700</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Beberapa waktu lalu, seorang warga mencurahkan keluhannya ke media massa. Pada 2018, ia membeli dua unit apartemen ...</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686436/hunian-impian-tertunda-kepercayaan-konsumen-dipertaruhkan</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-18.15.56.jpeg</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Palestina tekankan perlindungan situs purbakala</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:14:04 +0700</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Menteri Pariwisata dan Kepurbakalaan Palestina Hani Al-Hayek menekankan pentingnya upaya nasional mengawasi dan ...</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686432/palestina-tekankan-perlindungan-situs-purbakala</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/14/309654_edited.jpegWisata-Kota-Suci-Tiga-Agama-13022026-Adm-16.jpg</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>DPKH Kaltim bina peternak membuat pakan awetan hadapi musim kemarau</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:08:08 +0700</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Dinas Peternakan dan Kesehatan Hewan (DPKH) Provinsi Kalimantan Timur membina para peternak untuk memproduksi pakan ...</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686431/dpkh-kaltim-bina-peternak-membuat-pakan-awetan-hadapi-musim-kemarau</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001896691.jpg</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Dewan Pakar BPIP nilai Pakta Pertahanan Makkah bentuk kesadaran baru</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:07:49 +0700</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Dewan Pakar Badan Pembinaan Ideologi Pancasila (BPIP) Bidang Strategi Hubungan Luar Negeri Darmansjah Djumala menilai ...</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686428/dewan-pakar-bpip-nilai-pakta-pertahanan-makkah-bentuk-kesadaran-baru</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/04/12/1000365833.jpg</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Hafidz Kaltim wakili Indonesia menuju MTQ Internasional di Maroko</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:07:32 +0700</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Lembaga Pengembangan Tilawatil Qur'an (LPTQ) Provinsi Kalimantan Timur kembali melanjutkan tradisi prestasi di ...</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686425/hafidz-kaltim-wakili-indonesia-menuju-mtq-internasional-di-maroko</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_3701.jpeg</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>PSS Sleman matangkan persiapan untuk Super League</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:03:43 +0700</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>PSS Sleman terus mematangkan persiapan skuad menuju Super League 2026/2027 dengan menjalani beberapa laga uji ...</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686424/pss-sleman-matangkan-persiapan-untuk-super-league</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/2ac020c4-a5b8-46f9-85f1-a7f4c2d4fcc4-1_all_1201.jpg</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Menlu Turki: Kesepakatan pertahanan trilateral baru tak menarget Iran</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:59:33 +0700</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Menteri Luar Negeri Turki Hakan Fidan pada Sabtu (8/8) mengatakan bahwa Perjanjian Pertahanan Bersama Makkah yang ...</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686423/menlu-turki-kesepakatan-pertahanan-trilateral-baru-tak-menarget-iran</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/CjkinzN000005_20260809_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Turki bantah pakta pertahanan trilateral langgar NATO</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:57:14 +0700</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Turki membantah klaim di media sosial yang menyebut perjanjian pertahanan trilateral dengan Arab ...</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686415/turki-bantah-pakta-pertahanan-trilateral-langgar-nato</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AYM_TURKI-BANTAH-PAKTA-PERTAHANAN-TRILATERAL.jpg</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Begini serunya lomba pukul bantal menyambut HUT ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:54:59 +0700</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Seorang peserta terjatuh ke air setelah menerima pukulan dari lawannya dalam lomba pukul bantal di Kelurahan Madyopuro, ...</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5686421/begini-serunya-lomba-pukul-bantal-menyambut-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Lomba-pukul-bantal-sambut-HUT-Kemerdekaan-RI-090826-abs-6.jpg</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>PSS Sleman kenalkan sembilan pemain baru hadapi Super League 2026/2027</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:49:50 +0700</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Klub promosi BRI Super League PSS Sleman resmi memperkenalkan sembilan pemain baru yang akan memperkuat komposisi tim ...</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686420/pss-sleman-kenalkan-sembilan-pemain-baru-hadapi-super-league-2026-2027</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/2ac020c4-a5b8-46f9-85f1-a7f4c2d4fcc4-1_all_1201.jpg</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Bupati Bogor jemput bendera pusaka tahun 1948 dari pendopo bersejarah</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:48:20 +0700</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Bupati Bogor Rudy Susmanto menjemput bendera pusaka tahun 1948 dari pendopo bersejarah di Desa Malasari, Nanggung, ...</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686419/bupati-bogor-jemput-bendera-pusaka-tahun-1948-dari-pendopo-bersejarah</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1003324894.jpg</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Ruang urgensi pengurangan metana minyak dan gas di Indonesia</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:44:53 +0700</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Ada satu jenis kerugian di industri minyak dan gas Indonesia yang tidak terlihat dari kejauhan: yaitu kebocoran ...</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686412/ruang-urgensi-pengurangan-metana-minyak-dan-gas-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/08/23/IMG-20250822-WA0008.jpg</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Kemenimipas sambut HUT RI dengan jalan santai hingga bersih-bersih TMP</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:44:09 +0700</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Kementerian Imigrasi dan Pemasyarakatan (Kemenimipas) menyambut HUT ke-81 RI dengan mengadakan jalan santai atau fun ...</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686407/kemenimipas-sambut-hut-ri-dengan-jalan-santai-hingga-bersih-bersih-tmp</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-09-at-11.53.30.jpg</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>LKBN ANTARA berkomitmen bantu penguatan promosi Mandalika</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:43:12 +0700</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Direktur Utama Perum LKBN ANTARA Benny Siga Butarbutar mengatakan media ANTARA sebagai kantor berita nasional tetap ...</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686403/lkbn-antara-berkomitmen-bantu-penguatan-promosi-mandalika</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1005752026.jpg</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Kemenbud jaga Lamin Mancong sebagai monumen harmoni budaya di Kaltim</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:40:19 +0700</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Kementerian Kebudayaan melalui Balai Pelestarian Kebudayaan (BPK) terus memperkuat upaya perlindungan Lamin Mancong di ...</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686400/kemenbud-jaga-lamin-mancong-sebagai-monumen-harmoni-budaya-di-kaltim</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001896813.jpg</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Ditpolairud Polda Metro Jaya Tetapkan Tersangka Kasus Tambang Ilegal</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:19:27 +0700</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Ditpolairud Polda Metro Jaya menetapkan RS sebagai tersangka dalam kasus tambang ilegal. RS ditahan untuk penyidikan lebih lanjut.</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610813/ditpolairud-polda-metro-jaya-tetapkan-tersangka-kasus-tambang-ilegal</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/09/05/ilustrasi-tambang-ilegal_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Wagub DKI Rano Karno Tinjau Kondisi Gedung Bapenda yang Terbakar</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:16:12 +0700</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Wagub DKI Jakarta Rano Karno meninjau Gedung Bapenda yang terbakar. Operasional dihentikan sementara, dan tempat kerja alternatif disiapkan untuk pegawai.</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610810/wagub-dki-rano-karno-tinjau-kondisi-gedung-bapenda-yang-terbakar</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/wakil-gubernur-wagub-dki-jakarta-rano-karno-meninjau-langsung-kondisi-gedung-dinas-teknis-badan-pendapatan-daerah-bapenda-dki--1786256114834_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Polisi Bongkar Peredaran Sinte di Bekasi, 2 Pelaku Ditangkap</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:02:46 +0700</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Farih Maulana Sidik</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Polres Metro Bekasi Kota membongkar kasus peredaran narkotika jenis tembakau Gorilla. Dua pelaku ditangkap, barang bukti disita untuk penyidikan lebih lanjut.</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610787/polisi-bongkar-peredaran-sinte-di-bekasi-2-pelaku-ditangkap</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/polres-metro-bekasi-kota-membongkar-kasus-peredaran-narkotika-jenis-tembakau-gorila-alias-sinte-1786255302127_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Gudang Spare Part Motor di Tangerang Kebakaran, Asap Hitam Membubung</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:01:45 +0700</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda gudang sparepart motor di Kosambi, Tangerang. Asap hitam pekat terlihat, dan 12 unit pemadam dikerahkan untuk memadamkan api.</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610786/gudang-spare-part-motor-di-tangerang-kebakaran-asap-hitam-membubung</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/10/17/ilustrasi-kebakaran_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>RI &amp;amp; UEA Bahas Rencana Genjot Perdagangan</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:30:35 +0700</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Kedua menteri membahas upaya mengoptimalkan pemanfaatan Indonesia-United Arab Emirates Comprehensive Economic Partnership Agreement (IUAE-CEPA).</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610745/ri-uea-bahas-rencana-genjot-perdagangan</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/03/05/menteri-perdagangan-mendag-budi-santoso-1772697811641_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>EX2 Jadi Volume Maker Penjualan di RI, Geely Auto Tambah Kapasitas Produksi</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:11:20 +0700</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Di Indonesia, mobil ini ditawarkan dalam dua pilihan, yaitu EX2 Pro dan EX2 Max dengan tingkat kandungan dalam negeri (TKDN) mencapai 46,5 persen.</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865975/ex2-jadi-volume-maker-penjualan-di-ri-geely-auto-tambah-kapasitas-produksi</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/2vev6ROiN1lwts7oFskgl4eiWaI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/geely-k8898.jpg</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>4 Fakta Febrio Adriono: Antar Sutrimo ke RS, Eks Ajudan Febrie Adriansyah, Pegawai di Kejagung</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:10:29 +0700</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Kejagung membenarkan sosok Febrio Adiono, pengantar Sutrimo ke rumah sakit, adalah pegawainya.</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865974/4-fakta-febrio-adriono-antar-sutrimo-ke-rs-eks-ajudan-febrie-adriansyah-pegawai-di-kejagung</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/sg7n43axcHGd8Q3T9N-U9JrHaZs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/gedung-kejaksaan-agung-ri-11.jpg</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu Jellyfish - Sunset Rollercoaster feat Michael Seyer: Please Don't Wake Me Up</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:06:24 +0700</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Terjemahan lirik lagu Jellyfish yang dinyanyikan oleh Sunset Rollercoaster. Lagu yang dirilis pada 29 Juli 2022 ini kolaborasi dengan Michael Seyer.</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7865973/terjemahan-lirik-lagu-jellyfish-sunset-rollercoaster-feat-michael-seyer-please-dont-wake-me-up</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tEq9lHSi3zC8-tIEQ99J9IcoxD8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-terjemahan-lirik-lagu.jpg</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Menilik Konter Royal Phone Ambarawa, sang Bos Baru Berusia 25 Tahun Tewas Dirampok</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:56:17 +0700</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Royal Phone Ambarawa yang disantroni perampok dikenal sebagai toko ponsel yang menawarkan harga relatif murah. Pemiliknya kini tewas.</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865972/menilik-konter-royal-phone-ambarawa-sang-bos-baru-berusia-25-tahun-tewas-dirampok</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/uSFJBKkI99SpecMW9nKrYmjZaqs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pembunuhan-bos-konter-Ambarawa.jpg</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Tips Upgrade Lampu Kendaraan: Pertimbangkan Kecerahan dan Warna Cahaya</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:55:23 +0700</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Sebelum upgrade lampu bawaan kendaraan, pastikan lampu sesuai dengan jenis reflektor atau projector kendaraan.</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865971/tips-upgrade-lampu-kendaraan-pertimbangkan-kecerahan-dan-warna-cahaya</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/PapWasvtjGFgnIlvVsf68WToYz4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-lampu-mobil-882.jpg</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Anak Lahap Makan tapi Makin Kurus, Bisa Jadi Tanda Diabetes, Kenali Gejalanya</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:51:33 +0700</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Kebiasaan harian anak bisa menjadi indikasi awal hadirnya gangguan kesehatan serius, salah satunya diabetes.</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865970/anak-lahap-makan-tapi-makin-kurus-bisa-jadi-tanda-diabetes-kenali-gejalanya</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/bqAGtaSQIa3CyEfY0aJehVagx8M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-pemeriksaan-diabetes-pada-anak.jpg</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Tim Gabungan Akan Sisir Sisa Material yang Berpotensi Picu Titik Api di Kawasan Gunung Rinjani</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:51:21 +0700</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Tim gabungan akan menyisir sisa material kebakaran hutan dan lahan (karhutla) di kawasan Gunung Rinjani.</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865969/tim-gabungan-akan-sisir-sisa-material-yang-berpotensi-picu-titik-api-di-kawasan-gunung-rinjani</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/i6c2S40nNkaJZsrhRFQzrJhqsx4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Abdul-Muhari-BNPB-3210.jpg</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Cara Feby Febiola Hilangkan Gugup Berakting di Depan Kamera Setelah Sempat 11 Tahun Vakum</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:45:22 +0700</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Feby Febiola kembali ke dunia akting, dengan menerima tawaran film 'Kuasa Gelap: Perjanjian Darah' karya Rizal Mantovani.</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865968/cara-feby-febiola-hilangkan-gugup-berakting-di-depan-kamera-setelah-sempat-11-tahun-vakum</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Z6s5raXeQFngLzHSteDX8RWxtG0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/febi-febiola-film-la.jpg</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Keluarga Sutrimo Putuskan Buat Laporan, LPSK Jemput Bola untuk Beri Perlindungan</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:45:21 +0700</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>LPSK  akan mendatangi keluarga Sutrimo, orang dekat yang juga pekerja rumah eks Jampidsus, Febrie Adriansyah.</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865967/keluarga-sutrimo-putuskan-buat-laporan-lpsk-jemput-bola-untuk-beri-perlindungan</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/kZFE6PfULAXOD752T0B7EGx5hp4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Rumah-Sutrimo-di-Banyumas-1.jpg</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Pastikan Distribusi Energi, Komisaris Pertamina Patra Niaga Cek Integrated Terminal Tanjung Uban</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:44:21 +0700</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Integrated Terminal Tanjung Uban merupakan salah satu terminal yang sangat sibuk dan menjadi tulang punggung distribusi energi di Sumatera.</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865966/pastikan-distribusi-energi-komisaris-pertamina-patra-niaga-cek-integrated-terminal-tanjung-uban</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/x6-g5ZoudwpRBVbRT54DAJqKIxg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/dewan-komisaris-pertamina-PN-riau.jpg</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>PM Takaichi Tegaskan Jepang Pertahankan Tiga Prinsip Non-Nuklir di Peringatan Bom Nagasaki</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:44:20 +0700</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>PM Jepang Sanae Takaichi menegaskan Tiga Prinsip Non-Nuklir saat peringatan 81 tahun bom Nagasaki dan menyerukan dunia bebas senjata nuklir</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865965/pm-takaichi-tegaskan-jepang-pertahankan-tiga-prinsip-non-nuklir-di-peringatan-bom-nagasaki</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/TQ2PzwG346tsMfD15thp9udbE0E=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PM-Jepang-Sanae-Takaichi122232.jpg</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Iran Semprot AS dan Sekutunya, Minta Pasukan Asing Segera Angkat Kaki dari Timur Tengah</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:43:07 +0700</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Iran semprot AS dan sekutunya! Teheran mendesak seluruh pasukan asing angkat kaki dari Timur Tengah, sebut mereka biang utama ketidakamanan kawasan.</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865964/iran-semprot-as-dan-sekutunya-minta-pasukan-asing-segera-angkat-kaki-dari-timur-tengah</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Y9NtYqyR1TOGuHgmXe4oUuy7N3Q=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/bendera-Iran-Amerika-Israel-2.jpg</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Kebakaran di Gunung Bromo, BNPB: Hot Spot di Area Pusung Ledok Bedor Masih Keluarkan Asap</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:42:28 +0700</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>BNPB  mencatat hot spot di area Pusung Ledok Bedor kawasan Gunung Bromo, Provinsi Jawa Timur, masih mengeluarkan asap.</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865963/kebakaran-di-gunung-bromo-bnpb-hot-spot-di-area-pusung-ledok-bedor-masih-keluarkan-asap</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/xoFFaiJU2PaV7uUFrp2beyWsUFQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/gunung-bromo-kebakaran-12.jpg</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Polisi Segera Ekshumasi Jasad Sutrimo untuk Ungkap Penyebab Kematian</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:40:24 +0700</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Polisi siapkan ekshumasi jasad Sutrimo, orang dekat eks Jampidsus Febrie, guna ungkap penyebab kematian yang penuh kejanggalan.</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865962/polisi-segera-ekshumasi-jasad-sutrimo-untuk-ungkap-penyebab-kematian</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/CwMUyzUp6Ng_C-qMpDr5muWU_Ls=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/klinik-Mordent-Esthetic-Clinic-TKP-Sutrimo-Tewas.jpg</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Tampil Ikonik, Aplikasi Kaca Film pada iCar V23 di GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:39:16 +0700</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Contoh aplikasi kaca film yang bisa menghasilkan nilai estetika ikonik ditampilkan di pameran otomotif GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865961/tampil-ikonik-aplikasi-kaca-film-pada-icar-v23-di-giias-2026</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/j1W10LElTiwmoRNHEP-3wCtcPu4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SUV-bergaya-retro-turistik-iCar-V23-milik-Den-Dimas.jpg</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Update Ranking BWF setelah Korea Masters 2026: Top 16 Aman, Tunggal Putri India Meledak</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:35:44 +0700</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Simak update ranking BWF 2026 khususnya dari nomor tunggal putri, setelah berakhirnya turnamen Korea Masters</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865960/update-ranking-bwf-setelah-korea-masters-2026-top-16-aman-tunggal-putri-india-meledak</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/3VsW5fSrbDjMam4qXRL5D8B9Wjo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pebulu-tangkis-tunggal-putri-India-Tanvi-Sharma.jpg</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>10 Puisi 17 Agustus untuk Meriahkan HUT ke-81 RI, Penuh Semangat dan Cinta Tanah Air</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:33:55 +0700</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Simak kumpulan contoh puisi 17 Agustus untuk memeriahkan peringatan HUT ke-81 RI, penuh semangat dan cinta tanah air.</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865959/10-puisi-17-agustus-untuk-meriahkan-hut-ke-81-ri-penuh-semangat-dan-cinta-tanah-air</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/6CGTOF-7ARmb7n2ir-zMveEcqMw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Perobekan-Bendera-Merah-Putih-Biru-di-Hotel-Yamato-Surabaya_20250921_173139.jpg</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Wilayah Priangan Jawa Barat, Senin 10 Agustus 2026: Dominan Berawan</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:33:18 +0700</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) merilis prakiraan cuaca untuk wilayah Priangan, Jawa Barat, pada besok Senin (10/8/2026).</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865958/prakiraan-cuaca-wilayah-priangan-jawa-barat-senin-10-agustus-2026-dominan-berawan</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/frSAlNJSvAYtGPzW7khFc6-RSek=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Cuaca-di-Kota-Sorong-cuaca-berawan2.jpg</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Mertua dan Menantu di Sinjai Tewas Tersengat Listrik Jerat Babi, Polisi Lakukan Penyelidikan</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:31:53 +0700</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Dua warga di Kabupaten Sinjai, Sulawesi Selatan, tersengat listrik dari jerat babi pada Sabtu (8/8/2026), pukul 21.40 Wita.</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865957/mertua-dan-menantu-di-sinjai-tewas-tersengat-listrik-jerat-babi-polisi-lakukan-penyelidikan</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/KpYwknGGnaS2f9ozUQaBrSbnft8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ilustrasi-mayat.jpg</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Polisi Bekasi Gerebek Rumah di Tambun Bekasi, Pengedar dan 2 Wanita Diringkus Saat Pesta Sabu</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:30:53 +0700</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Polsek Babelan menangkap tiga orang terkait dugaan peredaran narkotika di Bekasi. Polisi menyita Etomidate dan kristal putih diduga sabu</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865956/polisi-bekasi-gerebek-rumah-di-tambun-bekasi-pengedar-dan-2-wanita-diringkus-saat-pesta-sabu</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5bxMJP6XN6rNN38h3cy5D90tgzI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-sabu-sabu-sd.jpg</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Sepekan Terakhir, Data Perdagangan Saham Ditutup Mayoritas Positif</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:32:01 +0700</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Gita Amanda</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- PT Bursa Efek Indonesia (BEI) menyampaikan kinerja pasar saham pada sepekan terakhir bergerak positif. Indeks Harga Saham Gabungan (IHSG) tercatat berada di posisi 6.409 dengan nilai kapitalisasi...</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhotd423/sepekan-terakhir-data-perdagangan-saham-ditutup-mayoritas-positif</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/092218600-1785491445-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Kunjungan Wisata ke Dalam Negeri Naik, ke Luar Negeri Turun</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:26:04 +0700</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Lida Puspaningtyas</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Menteri Pariwisata (Menpar) Widiyanti Putri Wardhana mengatakan sektor pariwisata sepanjang semester I 2026 mencatatkan pertumbuhan positif, mulai dari kunjungan wisatawan mancanegara, perjalanan wisatawan nusantara, realisasi investasi, hingga...</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhojg502/kunjungan-wisata-ke-dalam-negeri-naik-ke-luar-negeri-turun</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260603215517-620.png</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Danantara Gelontorkan Investasi Rp44,5 Triliun untuk Kuasai Pasar Daging Asia</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:18:16 +0700</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Lida Puspaningtyas</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Danantara Indonesia menggelontorkan investasi senilai 2,5 miliar dolar AS atau sekitar Rp44,5 triliun dalam memperkuat industri peternakan Tanah Air. Hal ini tertuang dalam kemitraan strategis jangka panjang...</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjho6g502/danantara-gelontorkan-investasi-rp445-triliun-untuk-kuasai-pasar-daging-asia</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/030113600-1763569982-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya Tetapkan Tersangka Kasus Tambang Ilegal</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:24:32 +0700</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Penetapan tersangka tambang ilegal dilakukan usai penyidik mengantongi sejumlah alat bukti.</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265563/polda-metro-jaya-tetapkan-tersangka-kasus-tambang-ilegal</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/8dKNexoGjeyfeHyDFmMxqz-n7q4=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319528/original/065295800_1786256663-71099.jpg</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>JIS Tak Lagi Khawatir Kekurangan Parkir Saat Acara</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:00:01 +0700</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Tarif parkir akan disamakan dengan JIS.</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265543/jis-tak-lagi-khawatir-kekurangan-parkir-saat-acara</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/oyZxFY88v-nw-sbBYgI_yWL_IKs=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/1098919/original/037495800_1451553703-20151231-Ancol-menjadi-pilihan-warga-untuk-pergantian-tahun-Gempur-5.jpg</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Usai Mutilasi, Pelaku Jual Motor dan HP Korban Lewat Facebook</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:49:02 +0700</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Motor dan handphone tersebut dijual dengan harga murah.</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265541/usai-mutilasi-pelaku-jual-motor-dan-hp-korban-lewat-facebook</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/5zOBbNi9ZgWMlrDqEpdEmRYkEIE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9316331/original/057473700_1785921854-20260805_150500.jpg</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Hampir 2 Pekan Satpam Jatiluhur Tewas, Pelaku Belum Terungkap, Kondisi Istri Drop</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:39:35 +0700</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Hampir dua pekan kasus kematian satpam di Jatiluhur belum terungkap. Istri korban mengaku kondisi kesehatannya menurun.</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>https://bandung.kompas.com/read/2026/08/09/133700578/hampir-2-pekan-satpam-jatiluhur-tewas-pelaku-belum-terungkap-kondisi-istri</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/gEW_EXysTZwFtuHHgIQ8Q-jebd4=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/08/6a7729e6144a6.jpeg</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Lexus RX Jadi Andalan Penjualan Lexus di Indonesia</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:39:35 +0700</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Lexus RX bukan lagi sekadar model pelengkap, tapi salah satu tulang punggung Lexus Indonesia.</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>https://otomotif.kompas.com/read/2026/08/09/130200615/lexus-rx-jadi-andalan-penjualan-lexus-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/JMzRlstremdtBwfc93Yoarmjl_Q=/701x467:6307x4205/1200x675/filters:watermark(data/photo/2026/01/30/697c81750a668.png,0,-0,1)/data/photo/2026/08/09/6a77ebe405fa2.jpg</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>KPAI: Rokok Ilegal Murah Bikin Candu, Pengawasan Diperketat untuk Cegah Anak Jadi Konsumen</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:39:35 +0700</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Rokok murah menjerat anak dan remaja, memicu ketergantungan serius. KPAI peringatkan strategi pasar candu, sementara Dinkes DKI soroti ribuan remaja berisiko nikotin.</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/09/12193371/kpai-rokok-ilegal-murah-bikin-candu-pengawasan-diperketat-untuk-cegah</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/WItVzYiylYTZCzEChhtqZGdQbno=/150x100:1350x900/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2025/12/12/693c063dd1589.jpg</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I326"/>
+  <autoFilter ref="A1:I378"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 07:52 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$378</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$443</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I378"/>
+  <dimension ref="A1:I443"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -18200,8 +18200,3065 @@
         </is>
       </c>
     </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Pramono pastikan data perpajakan di Bapenda dicadangkan sistem digital</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:43:31 +0700</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>ANTARA - Gubernur DKI Jakarta Pramono Anung, di Jakarta pada Minggu (9/8) mengatakan, data perpajakan yang berada di ...</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686484/pramono-pastikan-data-perpajakan-di-bapenda-dicadangkan-sistem-digital</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PRAMONO-PASTIKAN-DATA-PERPAJAKAN-DI-BAPENDA-DICADANGKAN-SISTEM-DIGITAL.jpg</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Senat Amerika Serikat sahkan Todd Blanche sebagai Jaksa Agung</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:34:33 +0700</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>ANTARA - Senat Amerika Serikat mengesahkan Todd Blanche sebagai Jaksa Agung yang sebelumnya menjabat sebagai Wakil ...</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686473/senat-amerika-serikat-sahkan-todd-blanche-sebagai-jaksa-agung</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SENAT-AMERIKA-SERIKAT-SAHKAN-TODD-BLANCHE-SEBAGAI-JAKSA-AGUNG.jpg</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Imigrasi Maluku optimalkan layanan paspor merdeka sambut HUT RI 2026</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:33:37 +0700</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Kantor Wilayah Direktorat Jenderal Imigrasi Maluku mengoptimalkan layanan paspor bagi masyarakat melalui program Paspor ...</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686488/imigrasi-maluku-optimalkan-layanan-paspor-merdeka-sambut-hut-ri-2026</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/PASPOR.jpeg</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Apple dikabarkan akan naikkan harga iPhone 17 dalam waktu dekat</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:30:17 +0700</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Apple dikabarkan berencana menaikkan harga jajaran iPhone 17 dalam waktu dekat, setelah mempertahankan harganya sejak ...</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686485/apple-dikabarkan-akan-naikkan-harga-iphone-17-dalam-waktu-dekat</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/InShot_20250910_104619944.jpg</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Era baru, hadir sepatu lari berperforma tinggi untuk pemakaian harian</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:28:05 +0700</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Jenama olahraga dari Jerman adidas memperkenalkan sebuah era baru dengan meluncurkan sepatu lari harian yang memiliki ...</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686483/era-baru-hadir-sepatu-lari-berperforma-tinggi-untuk-pemakaian-harian</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/upscalemedia-transformed-10.jpeg</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Duel Persija vs Persib dijadwalkan digelar di GBK</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:14:53 +0700</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Duel klasik antara Persija Jakarta melawan Persib Bandung pada pekan kedua Super League 2026 ...</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686476/duel-persija-vs-persib-dijadwalkan-digelar-di-gbk</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/11/08/ketum-pssi-tinjau-kondisi-rumput-sugbk-08112024-dr-04.jpg</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Pemprov Maluku gandeng ICMI perkuat riset dan inovasi daerah</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:05:26 +0700</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi Maluku menggandeng Ikatan Cendekiawan Muslim se-Indonesia (ICMI) untuk memperkuat ekosistem riset ...</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686468/pemprov-maluku-gandeng-icmi-perkuat-riset-dan-inovasi-daerah</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/icmi.jpeg</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Presiden Persija serahkan keputusan rekrut pemain ke STY</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:02:19 +0700</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>Presiden Persija Jakarta Mohammad Prapanca menyerahkan keputusan perekrutan pemain ke pelatih Persija Jakarta Shin ...</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686464/presiden-persija-serahkan-keputusan-rekrut-pemain-ke-sty</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG-20260809-WA0034_1.jpg</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Indonesia raih dua medali pada Kejuaraan Asia Hoki Bawah Air 2026</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:56:13 +0700</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Indonesia meraih satu medali perak dan satu perunggu pada Kejuaraan Asia Hoki Bawah Air CMAS 2026 di Aquatic Centre ...</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686460/indonesia-raih-dua-medali-pada-kejuaraan-asia-hoki-bawah-air-2026</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/hoki.jpeg</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Kowani dorong UNESCO tetapkan tempe sebagai WBTb Indonesia</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:53:59 +0700</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>ANTARA - Ketua Umum Kongres Wanita Indonesia (Kowani), Nannie Hadi Tjahjanto di Jakarta, pada Minggu (9/8) mendorong ...</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686444/kowani-dorong-unesco-tetapkan-tempe-sebagai-wbtb-indonesia</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AYM_KOWANI-DORONG-UNESCO-TETAPKAN.jpg</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Pertamina Patra Niaga lestarikan warisan kuliner nusantara lewat BGCC</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:53:48 +0700</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>PT Pertamina Patra Niaga turut melestarikan warisan kuliner nusantara lewat ajang kompetisi memasak Bright Gas Cooking ...</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686459/pertamina-patraniaga-lestarikan-warisan-kuliner-nusantara-lewat-bgcc</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000406013.jpg</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Eko Yuli Irawan kembali tampil untuk kali keenam di Asian Games</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:51:10 +0700</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>Lifter senior Indonesia Eko Yuli Irawan diproyeksikan menjalani Asian Games keenam dalam karirnya setelah masuk dalam ...</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686455/eko-yuli-irawan-kembali-tampil-untuk-kali-keenam-di-asian-games</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/12/14/eko-yuli-irawan-raih-perunggu-sea-games-2025-2690158.jpg</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Rizki dan Rahmat turun di kelas berbeda pada Asian Games 2026</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:42:48 +0700</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Dua lifter andalan Indonesia Rizki Juniansyah dan Rahmat Erwin Abdullah diproyeksikan turun di kelas berbeda pada Asian ...</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686453/rizki-dan-rahmat-turun-di-kelas-berbeda-pada-asian-games-2026</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/05/1000173280.jpg</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Polisi ringkus empat perusak kabel optik di Pademangan</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:39:53 +0700</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>Unit Reskrim Polsek Pademangan berhasil menangkap empat pelaku yang diduga terlibat kasus perusakan jaringan ...</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686451/polisi-ringkus-empat-perusak-kabel-optik-di-pademangan</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/b2d55bd6-0796-49aa-b348-f23ac5240be3.jpeg</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Angkat besi siapkan delapan lifter menuju Asian Games 2026</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:38:14 +0700</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Pengurus Besar Perkumpulan Angkat Besi Seluruh Indonesia (PB PABSI) menyiapkan delapan lifter yang terdiri atas empat ...</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686447/angkat-besi-siapkan-delapan-lifter-menuju-asian-games-2026</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/05/pemusatan-latihan-angkat-besi-jelang-sea-games-2025-2661229.jpg</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Api Belum Padam, Kebakaran di Kosambi Tangerang Lahap 3 Gudang</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:39:35 +0700</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>Kebakaran gudang sparepart motor di Kosambi, Tangerang, masih berlangsung. Tiga gudang terbakar, petugas pemadam berjuang memadamkan api.</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610903/api-belum-padam-kebakaran-di-kosambi-tangerang-lahap-3-gudang</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/11/13/ilustrasi-api_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Menteri Imipas Ziarah ke TMP Taruna Tangerang Jelang HUT ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:15:56 +0700</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Muchamad Sholihin</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Menteri Imigrasi Agus Andrianto berziarah di TMP Taruna, Tangerang. Kegiatan ini dilakukan jelang HUT ke-81 RI.</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610869/menteri-imipas-ziarah-ke-tmp-taruna-tangerang-jelang-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/menteri-imipas-1786259638429_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Menteri LH Ungkap Pemilik SixNine Padel Bandung Bayar Denda Rp 100 Juta</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:41:33 +0700</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Menteri LH jatuhkan sanksi Rp 100 juta dan penanaman 1.000 pohon ke SixNine Padel. Kasus ini bermula dari penebangan 10 pohon untuk videotron.</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610835/menteri-lh-ungkap-pemilik-sixnine-padel-bandung-bayar-denda-rp-100-juta</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/penyegelan-videotron-sixnine-padel-buntut-penebangan-10-pohon-secara-ilegal-1785907225233_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Keluarga Serahkan Proses Pengusutan Penyebab Kematian Sutrimo ke Polisi</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:35:15 +0700</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Keluarga Sutrimo laporkan kematian ke polisi, curiga ada ketidakwajaran. Mereka minta kepastian hukum tanpa menunjuk terlapor tertentu.</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610832/keluarga-serahkan-proses-pengusutan-penyebab-kematian-sutrimo-ke-polisi</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/27/polisi-masih-mendalami-penyebab-tewasnya-pria-bernama-sutrimo-di-depan-klinik-kecantikan-mordent-di-jaksel-penyebab-kematian-s-1785156176528_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>14.890 Barang Tertinggal di Kereta hingga Juli, Nilainya Rp 10,8 Miliar</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:30:07 +0700</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) mencatat sebanyak 14.890 barang temuan di berbagai wilayah operasional sepanjang Januari-Juli 2026.</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610761/14-890-barang-tertinggal-di-kereta-hingga-juli-nilainya-rp-10-8-miliar</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/03/24/arus-balik-lebaran-lewat-kereta-api-1774345135238_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Pertamina Bantu UMKM Kembangkan Olahan Hasil Laut, Pakai Cara Ini</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:15:32 +0700</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Program Kampung Bahari Si Pelaut melibatkan empat kelompok yang mengembangkan budidaya ikan dan sayuran, rehabilitasi mangrove, serta pengolahan hasil perikanan</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610899/pertamina-bantu-umkm-kembangkan-olahan-hasil-laut-pakai-cara-ini</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/pertamina-patra-niaga-1786260901782_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Cuma di Transmart Full Day Sale, Alat Masak Jadi Semurah Ini</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:00:07 +0700</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Belanja kebutuhan rumah tangga lebih murah di Transmart Full Day Sale.</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610714/cuma-di-transmart-full-day-sale-alat-masak-jadi-semurah-ini</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/transmart-full-day-sale-1786250852282_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Gisela Cindy Menanti Hari Bahagia: Akan Menikahi Sahabat Terbaikku</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:19:23 +0700</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>wes</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Gisela Cindy menumpahkan kebahagiaan jelang pernikahan. Ia bahagia karena akan menikahi sahabat terbaiknya.</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610800/gisela-cindy-menanti-hari-bahagia-akan-menikahi-sahabat-terbaikku</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/gisella-cindy-1786251703656_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Anisa Rahma-Suami Naik Gunung Merbabu: Cerita Baru Pernikahan Kita</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:08:50 +0700</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Pasangan Anisa Rahma dan Anandito Dwis baru saja membuka gembok pencapaian terkait pernikahan. Mereka naik gunung bersama.</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610795/anisa-rahma-suami-naik-gunung-merbabu-cerita-baru-pernikahan-kita</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/anisa-rahma-1786251541741_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Polisi Bakal Bongkar Makam Sutrimo Usai Kematian Dinilai Janggal</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:40:06 +0700</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Penyidik dari Polda Metro Jaya bakal melakukan ekshumasi terhadap jasad Sutrimo menyusul laporan dari kerabat soal dugaan kejanggalan kematiannya.</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809132136-12-1390286/polisi-bakal-bongkar-makam-sutrimo-usai-kematian-dinilai-janggal</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2018/08/24/8a7149c5-8060-403e-9fba-e91b1608a9fb_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Daftar Daerah RI Dikepung Karhutla hingga Warga Tewas</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:10:19 +0700</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan melanda sejumlah daerah di Indonesia, termasuk Gunung Bromo dan Kalimantan.</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809125010-20-1390279/daftar-daerah-ri-dikepung-karhutla-hingga-warga-tewas</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/pemadaman-kebakaran-kawasan-hutan-di-boyolali-1785974493169_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Kebakaran Hutan Meluas di Bromo, Semua Akses Wisata Ditutup</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan dan lahan kian meluas di area Kaldera Bromo pada Minggu (9/8).</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809130011-24-1390280/kebakaran-hutan-meluas-di-bromo-semua-akses-wisata-ditutup</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/thumbnail-video-1786255374008_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Pramono Putuskan Bongkar JPO 'Love-Hate Relationship' Rasuna Said</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung memutuskan untuk membongkar JPO "Love-Hate Relationship" di kawasan Jalan HR Rasuna Said, Kuningan, Jakarta Selatan (Jaksel).</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809122801-20-1390274/pramono-putuskan-bongkar-jpo-love-hate-relationship-rasuna-said</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/12/dki-siapkan-5-mobil-klinik-hewan-keliling-di-5-wilayah-1783840775602_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Pengunjung Acara di JIS Kini Bisa Parkir di Ancol</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:30:38 +0700</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta meminta pengelola JIS dan Ancol kolaborasi dalam pengelolaan parkir untuk acara di JIS.</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809123914-20-1390275/pengunjung-acara-di-jis-kini-bisa-parkir-di-ancol</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/06/22/peresmian-stasiun-jis-dan-jpo-jisancol-1782127101693_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Koarmada RI Gagalkan Penyelundupan 1,3 Ton Narkoba di Perairan Kepri</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:00:05 +0700</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Komando Armada Republik Indonesia (Koarmada RI) menggagalkan upaya penyelundupan narkoba melalui jalur laut di perairan Tanjung Berakit, Kepulauan Riau.</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809121705-12-1390264/koarmada-ri-gagalkan-penyelundupan-13-ton-narkoba-di-perairan-kepri</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/koarmada-i-tangkap-kapal-asing-bawa-13-ton-narkotika-diperairan-bintan-kepri-1786252733952_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Polri: Pemilik Sertifikat Pramuka Garuda Tetap Harus Ikut Tes Seleksi</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 12:40:05 +0700</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Kepolisian Negara Republik Indonesia (Polri) menegaskan pemilik sertifikat Pramuka Garuda tetap harus mengikuti tes atau seleksi untuk menjadi anggota Polri.</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809120148-12-1390260/polri-pemilik-sertifikat-pramuka-garuda-tetap-harus-ikut-tes-seleksi</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/08/14/pramuka-gelar-perkemahan-nasional-untuk-anak-berkebutuhan-khususpramuka-gelar-perkemahan-nasional-untuk-anak-berkebutuhan-khus-1755177247887_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Keluarga Lapor Polisi Minta Kepastian Hukum Soal Kematian Sutrimo</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 10:30:10 +0700</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Keluarga resmi melaporkan persoalan kematian Sutrimo ke Polresta Banyumas.</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809101451-12-1390240/keluarga-lapor-polisi-minta-kepastian-hukum-soal-kematian-sutrimo</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/keluarga-sutrimo-didampingi-kuasa-hukum-membuat-laporan-ke-polresta-banyumas-1786243465746_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>KLH/BPLH Ajak Anak Muda Bedah MRT Sebagai Solusi Krisis Ekologi Kota</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 09:48:00 +0700</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>Kementerian Lingkungan Hidup gelar program KELANA untuk edukasi lingkungan bagi pelajar untuk belajar tentang transportasi berkelanjutan dan dampak ekologisnya.</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809093651-25-1390223/klh-bplh-ajak-anak-muda-bedah-mrt-sebagai-solusi-krisis-ekologi-kota</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/kementerian-lingkungan-hidup-1786241566359_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Pecah Kongsi Chia/Soh Berujung Unik, Sama-sama Runner-up di Final Pertama usai Berpisah</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:32:57 +0700</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Aaron Chia dan Soh Wooi Yik sama-sama telah mencapai final perdana bersama pasangan baru setelah dipisahkan namun kompak runner-up.</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865998/pecah-kongsi-chiasoh-berujung-unik-sama-sama-runner-up-di-final-pertama-usai-berpisah</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/LynNsIx1h_zoZE6M8En8wUU9smQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ChiaSoh-Semifinal-Malaysia-Masters-2025.jpg</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Kisah Sarah Tumiwa Berubah Karakter di Film, Dari Tetangga Manis Jadi Hantu</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:31:39 +0700</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Sarah Tumiwa pun menerima tantangan baru di industri perfilman.Dari karakter tetangga manis, Sarah harus berubah jadi hantu.</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865997/kisah-sarah-tumiwa-berubah-karakter-di-film-dari-tetangga-manis-jadi-hantu</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/UMscM6OslnChrtx97yAODcuxrYQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sarah-Tumiwa-karakter-hantu.jpg</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Isu Pacar Pelaku DPP Terlibat Pembunuhan Bos Royal Phone Ambarawa, Polisi: Tidak Terkait</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:31:19 +0700</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Polisi membantah keterlibatan kekasih pelaku DPP dalam kasus pencurian dan pembunuhan bos Royal Phone Ambarawa.</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865996/isu-pacar-pelaku-dpp-terlibat-pembunuhan-bos-royal-phone-ambarawa-polisi-tidak-terkait</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/uSFJBKkI99SpecMW9nKrYmjZaqs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pembunuhan-bos-konter-Ambarawa.jpg</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Kode Redeem FF Terbaru Hari Ini, Minggu 9 Agustus 2026: Klaim Hadiahnya secara Gratis</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:31:06 +0700</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Kumpulan kode redeem Free Fire terbaru pada hari ini, Minggu (9/8/2026) di laman reward.ff.garena.com, klaim kodenya dan dapat hadiah gratisnya.</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/techno/7865995/kode-redeem-ff-terbaru-hari-ini-minggu-9-agustus-2026-klaim-hadiahnya-secara-gratis</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Zh5QA3rKg5MvVJECnJJmunlfDqk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Potret-bermain-gim-Garena-Free-Fire-FF-untuk-kode-redeem-FF.jpg</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Momen Pertemuan STY dan Gubernur Pramono, Ambisi Bawa Persija Juara Super League 2026-2027</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:30:23 +0700</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Pramono Anung dan Shin Tae-yong kompak targetkan Persija juara Super League 2026/2027, jadi kado 500 tahun Jakarta.</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865994/momen-pertemuan-sty-dan-gubernur-pramono-ambisi-bawa-persija-juara-super-league-2026-2027</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/bfmhXMmNBm7ANgGhz13KpjWWyZI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/STY-DAN-PRAMONO.jpg</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Harga Emas Antam Hari Ini, Minggu 9 Agustus 2026: Stagnan di Angka Rp2.690.000 per Gram</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:27:27 +0700</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Harga emas pada hari ini, Minggu (9/8/2026), stagnan di level Rp 2.690.000, simak rincian harga emas terbarunya.</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865993/harga-emas-antam-hari-ini-minggu-9-agustus-2026-stagnan-di-angka-rp2690000-per-gram</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/J5yz2H6KghKOYYUDkxXa0zEptx0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Harga-Emas-Antam-Naik_20251007_212034.jpg</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Sosok Eko Sapto Purnomo, Plt Bupati Sukoharjo Naik Tangga Ikut Padamkan Api Akibat Drone Jatuh</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:23:03 +0700</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Aksi heroik Plt Bupati Sukoharjo, Eko Sapto Purnomo viral. Dalam sebuah video yang beredar, Eko naik tangga ikut memadamkan api akibat drone jatuh.</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865992/sosok-eko-sapto-purnomo-plt-bupati-sukoharjo-naik-tangga-ikut-padamkan-api-akibat-drone-jatuh</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/-y8VHSg8H55O61w1S7dUctMuTrY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Plt-Bupati-Sukoharjo-Eko-Sapto-padamkan-api.jpg</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Hadiri HUT ke-8 MBI, Bamsoet Ajak Komunitas Otomotif Perkuat Brotherhood dan Persatuan Bangsa</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:21:56 +0700</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Bambang Soesatyo (Bamsoet) mengajak seluruh komunitas otomotif di Indonesia untuk menjaga soliditas serta memperkuat persatuan dan kesatuan bangsa.</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865991/hadiri-hut-ke-8-mbi-bamsoet-ajak-komunitas-otomotif-perkuat-brotherhood-dan-persatuan-bangsa</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/bSb3q2zOVaNkOmE2EvTJwMhf0os=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/bamsoet-mbi-persatuan-bangsa.jpg</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Iran Kirim Sinyal Damai ke AS: Pezeshkian Tegaskan Dialog Tak Berarti Tunduk pada Washington</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:13:48 +0700</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Iran buka peluang kesepakatan dengan AS. Presiden Masoud Pezeshkian menegaskan diplomasi adalah strategi, bukan tanda Teheran menyerah pada Washington</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865990/iran-kirim-sinyal-damai-ke-as-pezeshkian-tegaskan-dialog-tak-berarti-tunduk-pada-washington</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/R-46RcW9veQ0KzuwqGM4_Yx11Y0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Presiden-Iran-Masoud-Pezeshkian-ketika-menghadiri-KTT-BRICS-di-Kazan-Rusia.jpg</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Sudah Akhir Pekan, Prabowo Telah Putuskan Nama Calon Gubernur BI? Ini Kata Komisi XI DPR</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:13:06 +0700</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Gubernur BI yang baru harus memiliki kapabilitas dalam menjalankan bauran kebijakan untuk mendukung pertumbuhan ekonomi nasional.</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865989/sudah-akhir-pekan-prabowo-telah-putuskan-nama-calon-gubernur-bi-ini-kata-komisi-xi-dpr</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/jg29-yqbvdfq2O1GIB27QJD1kCI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Presiden-Prabowo-Subianto-meresmikan-Bendungan-Meninting.jpg</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Menjaga Asa di Surga Bahari, Dedikasi Mantri BRI untuk Masyarakat Kepulauan Wakatobi</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:12:52 +0700</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>Di gugusan Kepulauan Wakatobi, Wa Ode Sitti Rahmatiah Jufri, seorang Mantri BRI dari Unit Wangi-Wangi, Kantor Cabang BRI Baubau.</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865988/menjaga-asa-di-surga-bahari-dedikasi-mantri-bri-untuk-masyarakat-kepulauan-wakatobi</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/LrOjRj_Ml8Bn2Jjq9WJXCcm0ecA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/menjaga-asa-pulau-wakatobi.jpg</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Polemik Kasus Yurizal, Cibiran Nakes di Medsos Dinilai Bukan Sekadar Masalah Komunikasi</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:11:20 +0700</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Polemik komentar nakes terkait kasus Yurizal dinilai sebagai persoalan empati dan psikologi sosial, bukan sekadar komunikasi.</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865987/polemik-kasus-yurizal-cibiran-nakes-di-medsos-dinilai-bukan-sekadar-masalah-komunikasi</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/mKiK7DSnd0Cxme8GVosRxLtbQdw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sosok-Yurizal-Tri-Chaerawan.jpg</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Prediksi Race MotoGP Inggris 2026: Jorge Martin Calon Juara Baru, Tradisi Silverstone Berlanjut?</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:10:51 +0700</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Jorge Martin bawa modal sempurna menuju main race MotoGP Inggris 2026 lewat raihan pole dan memenangkan sprint race di Sirkuit Silverstone.</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865986/prediksi-race-motogp-inggris-2026-jorge-martin-calon-juara-baru-tradisi-silverstone-berlanjut</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WwTcMGAR_FjpP1p85zJvliY79So=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Jorge-Martin-Juara-Dunia-MotoGP-2024_20241118_125846.jpg</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Keamanan Siber Tak Cukup Andalkan Teknologi, Manusia Jadi Faktor Utama</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:10:17 +0700</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Virna mengatakan penguatan kesadaran, pengembangan talenta, dan pembangunan pertahanan kolektif pada akhirnya diperlukan</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/techno/7865985/keamanan-siber-tak-cukup-andalkan-teknologi-manusia-jadi-faktor-utama</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/LlDex0HUPRBmKlmkAx_WRO5f-fM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/keamanansiber111111.jpg</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Kronologi Bos Royal Phone Ambarawa Tewas Dibunuh, Pelaku DPP Bertanya pada TI Mau Uang atau Tidak</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:04:08 +0700</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Pembunuhan bos Royal Phone Ambarawa bermula saat pelaku DPP menawarkan kepada TI, apakah mau uang atau tidak.</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865984/kronologi-bos-royal-phone-ambarawa-tewas-dibunuh-pelaku-dpp-bertanya-pada-ti-mau-uang-atau-tidak</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/7ZZnVepqeCk6txc4fbmLp3oj0rQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sosok-Candra-Waskito-Bos-Royal-Phone-Ambarawa-Tewas-Dirampok-Dikenal-Dermawan-Semasa-Hidup.jpg</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Industri Wisata Kebugaran Dibidik Jadi Mesin Pertumbuhan Bisnis Baru</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:02:28 +0700</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>Pengembangan wellness tourism dapat menjadi peluang bagi daerah untuk mengembangkan sektor pariwisata sekaligus menggerakkan bisnis lokal.</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865983/industri-wisata-kebugaran-dibidik-jadi-mesin-pertumbuhan-bisnis-baru</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ft9YfOIlOyXjYW2Tps25J4CMIwA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Perkumpulan-Penggiat-Wisata-Kebugaran-Indonesia-Perwakin-77.jpg</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Kenali Pengobatan 2 Tipe Diabetes pada Anak, Perubahan Gaya Hidup hingga Terapi Seumur Hidup</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:55:12 +0700</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Penanganan penyakit diabetes pada kelompok usia anak tidak sama. Pengobatan tergantung jenis diabetes yang dialami anak.</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865982/kenali-pengobatan-2-tipe-diabetes-pada-anak-perubahan-gaya-hidup-hingga-terapi-seumur-hidup</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/bqAGtaSQIa3CyEfY0aJehVagx8M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-pemeriksaan-diabetes-pada-anak.jpg</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Hasil Final Korea Masters 2026: Yoo Tae-bin Gagal Juara, Revans Lunas tapi Gelar Lepas</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:47:32 +0700</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Tunggal puta Korea, Yoo Tae-bin kembali harus puas menjadi runner-up setelah kalah dari Zhu Xuan Chen di final Korea Masters 2026.</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865981/hasil-final-korea-masters-2026-yoo-tae-bin-gagal-juara-revans-lunas-tapi-gelar-lepas</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WJiBgGsDpO3dDnN5JKdwq2mXfd0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Yoo-Tae-Bin-Badminton-Korea.jpg</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda Jakarta, Kesaksian Warga: Kita Was-was, Lokasi Dekat Pom Bensin, Takut</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:45:37 +0700</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Kebakaran yang melanda gedung Bapenda Jakarta lantai 11 hingga 16 pada (7/8/2026) malam, warga sekitar panik.</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865980/kebakaran-gedung-bapenda-jakarta-kesaksian-warga-kita-was-was-lokasi-dekat-pom-bensin-takut</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1_y4HpWTBQMj1aoqmNV2l0rqqG8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kEBAKARAN-GEDUNG-DKI32.jpg</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Atasi Backlog Perumahan, Pembangunan Hunian Subsidi di Kawasan Perkotaan Perlu Diperbanyak</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:44:04 +0700</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Pembangunan Samesta Alonia Jakarta menjadi langkah awal untuk mewujudkan pembangunan perumahan rakyat dalam skala yang lebih besar.</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865979/atasi-backlog-perumahan-pembangunan-hunian-subsidi-di-kawasan-perkotaan-perlu-diperbanyak</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/13KdPHzGQoSYCFkInxeGB4qraVw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Proses-pemesanan-hunian-subsidi-semesta.jpg</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Video: Isu Pemilihan Gubernur BI Jadi Perhatian, Ini Efeknya ke Rupiah</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:30:50 +0700</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia TV</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Isu Pemilihan Gubernur BI Jadi Perhatian Investor, Ini Efeknya ke Rupiah</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260807141912-19-757447/video-isu-pemilihan-gubernur-bi-jadi-perhatian-ini-efeknya-ke-rupiah</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/isu-pemilihan-gubernur-bi-jadi-perhatian-investor-ini-efeknya-ke-rupiah-1786089168073_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Video: Urgensi Optimalisasi KUB Demi Perkuat Likuditas dan Layanan BPD</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:00:42 +0700</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>ASBANDA Dorong Optimalisasi KUB Demi Perkuat Likuditas, SDM dan Layanan Digital</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805161843-19-756843/video-urgensi-optimalisasi-kub-demi-perkuat-likuditas-layanan-bpd</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/asbanda-dorong-optimalisasi-kub-demi-perkuat-likuditas-sdm-layanan-digital-1785922861763_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Era Baru Bioteknologi, AI Kini Mampu Rancang Virus</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:30:14 +0700</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>AI kini mampu merancang virus, membuka peluang baru dalam pengembangan obat. Namun, muncul kekhawatiran tentang keamanan dan potensi penyalahgunaan teknologi.</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260809124014-37-757718/era-baru-bioteknologi-ai-kini-mampu-rancang-virus</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/05/20/ai-artificial-intelligence-reutersdado-ruvicillustrationfile-photo-1779242747740_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>GIIAS 2026 Diproyeksikan Catat Kenaikan Jumlah Pengunjung</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:41:00 +0700</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG -- Gabungan Industri Kendaraan Bermotor Indonesia (Gaikindo) optimistis tren positif penyelenggaraan Gaikindo Indonesia International Auto Show (GIIAS) 2026 berlanjut hingga hari terakhir pameran pada Ahad (9/8/2026).
+Ketua Harian...</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhqmp348/giias-2026-diproyeksikan-catat-kenaikan-jumlah-pengunjung</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/030253400-1785559217-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Mendag: BRICS Sepakati Mayoritas Substansi Perdagangan</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Gita Amanda</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Menteri Perdagangan (Mendag) RI Budi Santoso menyampaikan para menteri perdagangan negara-negara anggota BRICS menyetujui sebagian besar substansi dari pertemuan ini, meskipun pernyataan bersama (joint statement) belum tercapai.
+Dalam...</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhpw3423/mendag-brics-sepakati-mayoritas-substansi-perdagangan</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/menteri-perdagangan-mendag-budi-santoso-di-brussels_250713151814-802.jpg</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Backlog Rumah Masih Tinggi, Perumnas Mulai Bangun Hunian Vertikal</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:57:41 +0700</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Perum Perumnas resmi memulai pembangunan hunian vertikal subsidi perkotaan Samesta Alonia Jakarta. Proyek tersebut ditujukan untuk memperluas akses hunian layak dan terjangkau bagi masyarakat berpenghasilan rendah (MBR),...</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhpt6416/backlog-rumah-masih-tinggi-perumnas-mulai-bangun-hunian-vertikal</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260809135633-752.png</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Energi</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Dewan Komisaris Pertamina Patra Niaga Tinjau Distribusi Energi dan Program Pemberdayaan Masyarakat</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:56:00 +0700</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Intan Pratiwi</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, BATAM – Dewan Komisaris PT Pertamina Patra Niaga melakukan kunjungan kerja di Kepulauan Riau, Rabu (5/8), untuk meninjau langsung kesiapan operasional perusahaan, pengamanan objek vital nasional, serta pelaksanaan program...</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhkgv522/dewan-komisaris-pertamina-patra-niaga-tinjau-distribusi-energi-dan-program-pemberdayaan-masyarakat</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/dewan-komisaris-pt-pertamina-patra-niaga-melakukan-kunjungan-kerja_260809115747-356.jpeg</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Polisi Segera Ekshumasi Jenazah Sutrimo Demi Ungkap Penyebab Kematian</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:24:11 +0700</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Sutrimo disebut sebagai Karumga di kediaman mantan Jampidsus Febrie Adriansyah.</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265598/polisi-segera-ekshumasi-jenazah-sutrimo-demi-ungkap-penyebab-kematian</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/VZHx_LLEJelDk16a18hkWPVJUFU=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9308040/original/045771500_1785126728-WhatsApp_Image_2026-07-27_at_11.27.01.jpeg</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Kejari Depok Tetapkan Tersangka Baru Kasus Pengadaan Antena RRI</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 13:44:18 +0700</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Tersangka terlibat dalam pengadaan Antena Rotable Log Periodic untuk siaran luar negeri pada tahun anggaran 2021.</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265568/kejari-depok-tetapkan-tersangka-baru-kasus-pengadaan-antena-rri</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/jkod3Wzf0fS3-RPkxx9YEu3y_8E=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319536/original/085503800_1786257793-IMG-20260809-WA0009.jpg</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Kemarau Panjang Buat Waduk Bojongsari Indramayu Surut, Sungai Cimanuk Lama juga Mengering</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:52:04 +0700</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Kemarau panjang sebabkan Waduk Bojongsari Indramayu nyaris kering, dan Sungai Cimanuk lama mengering. Warga manfaatkan sisa air untuk memancing.</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/09/144346078/kemarau-panjang-buat-waduk-bojongsari-indramayu-surut-sungai-cimanuk-lama</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/AMp0kv-OAuSck1OSSFDDi7yqzaQ=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/09/6a781bf671bf5.jpeg</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>Cahaya</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Doa Tahajud Farrah, Santri Medan yang Lolos Beasiswa S1-S2 dan Al-Azhar Kairo</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:52:04 +0700</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Farrah mendapatkan beasiswa Program Akselerasi S1 dan S2 Bahasa Arab di UIN Sunan Ampel Surabaya dan Al-Azhar Kairo.</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>https://cahaya.kompas.com/aktual/26H09141500490/doa-tahajud-farrah-santri-medan-yang-lolos-beasiswa-s1-s2-dan-al-azhar-kairo</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/kS_tBZACJgj_3-5U7Pc8f00nHqU=/265x80:1071x618/1200x675/data/photo/2026/08/09/6a7825045f2a6.jpeg</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Sudaryono Tugaskan Pejabat BGN Berkantor di Daerah, Masuk Jakarta Harus Izin Dulu</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:52:04 +0700</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Kepala BGN Sudaryono menjelaskan bahwa kebijakan tersebut diperlukan karena lokasi pelaksanaan MBG tersebar di berbagai daerah.</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/09/13452691/sudaryono-tugaskan-pejabat-bgn-berkantor-di-daerah-masuk-jakarta-harus-izin</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/KomEhJDnwiNPmp2vAKeSQfDZ_eg=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/07/6a75b912399bd.jpeg</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I378"/>
+  <autoFilter ref="A1:I443"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 08:32 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$443</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$487</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I443"/>
+  <dimension ref="A1:I487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -21257,8 +21257,2076 @@
         </is>
       </c>
     </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Cuaca ekstrem ubah tren liburan musim panas di Prancis</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:23:00 +0700</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>ANTARA - Kondisi cuaca ekstrem mulai mengubah pola liburan musim panas masyarakat Prancis sehingga banyak wisatawan ...</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686527/cuaca-ekstrem-ubah-tren-liburan-musim-panas-di-prancis</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/CUACA-EKSTREM-UBAH-TREN-LIBURAN-MUSIM-PANAS-DI-PRANCIS.jpg</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>DLH Bandung Barat terjunkan tim telusuri pencemaran Sungai Cihaur</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:20:34 +0700</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Dinas Lingkungan Hidup (DLH) Kabupaten Bandung Barat, Jawa Barat, segera menerjunkan tim untuk menelusuri dugaan ...</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686532/dlh-bandung-barat-terjunkan-tim-telusuri-pencemaran-sungai-cihaur</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/488488.jpg</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Call Center 1500813 DKI layani derek hingga kendaraan jenazah gratis</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:13:56 +0700</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi DKI Jakarta menyediakan layanan derek hingga pemandu kendaraan jenazah gratis ...</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686529/call-center-1500813-dki-layani-derek-hingga-kendaraan-jenazah-gratis</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_143721478.jpg</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Pelti dorong kehadiran lebih banyak petenis di Liga Tenis Indonesia</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:12:17 +0700</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>Pengurus Pusat Persatuan Tenis Seluruh Indonesia (PP Pelti) berharap lebih banyak petenis nasional ambil bagian pada ...</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686523/pelti-dorong-kehadiran-lebih-banyak-petenis-di-liga-tenis-indonesia</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_4213.jpeg</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Apple dikabarkan akan luncurkan tiga produk "Ultra" hingga awal 2027</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:10:12 +0700</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>Apple dikabarkan akan meluncurkan hingga tiga produk "Ultra" terbaru mulai akhir 2026 hingga awal ...</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686520/apple-dikabarkan-akan-luncurkan-tiga-produk-ultra-hingga-awal-2027</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/InShot_20260805_145658063.jpg</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Robot humanoid makin banyak digunakan di Shenzhen, kini mulai terintegrasi dalam kehidupan sehari-hari</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:09:49 +0700</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Sebuah robot humanoid membuat es krim untuk pengunjung di sebuah taman di Shenzhen, Guangdong, China, Senin (3/8/2026). ...</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5686516/robot-humanoid-makin-banyak-digunakan-di-shenzhen-kini-mulai-terintegrasi-dalam-kehidupan-sehari-hari</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Robot-Humanoid-Terintegrasi-Di-Shenzhen-090826-LX-4.jpg</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>RI-Iran sepakat perkuat kemitraan teknologi baru, ketahanan pangan</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:07:23 +0700</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>Indonesia dan Iran sepakat memperluas kerja sama sains dan akademis di bidang teknologi baru, termasuk penelitian ...</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686512/ri-iran-sepakat-perkuat-kemitraan-teknologi-baru-ketahanan-pangan</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/23/WhatsApp-Image-2026-07-22-at-15.04.10.jpeg</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Juarai Liga Tenis Indonesia Seri 1, Lucky Candra tatap Asian Games</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:00:06 +0700</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Petenis putra Indonesia Lucky Candra Kurniawan menatap Asian Games 2026 setelah menjuarai nomor tunggal putra ...</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686508/juarai-liga-tenis-indonesia-seri-1-lucky-candra-tatap-asian-games</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_4212.jpeg</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Semifinal Piala AFF 2026</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>Empat tim terbaik melangkah ke semifinal Piala AFF 2026 usai babak penyisihan grup berakhir pada Sabtu (8/8). ...</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5686471/semifinal-piala-aff-2026</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/20260809-Semifinal-Piala-AFF-2026_1.jpg</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Polisi kejar dua pelaku perusakan kabel optik di Pademangan Jakut</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:59:34 +0700</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>Polsek Pademangan masih mengejar dua pelaku perusakan kabel optik di Jalan Pademangan Timur Gang Melati, Jakarta ...</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686505/polisi-kejar-dua-pelaku-perusakan-kabel-optik-di-pademangan-jakut</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_4582.jpeg</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Gerindra: Rapor "oke" Prabowo ke pemerintahannya bukan klaim sepihak</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:59:26 +0700</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Juru Bicara Partai Gerindra Sugiat Santoso menilai pernyataan Presiden Prabowo Subianto yang menyebut kinerja dua tahun ...</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686504/gerindra-rapor-oke-prabowo-ke-pemerintahannya-bukan-klaim-sepihak</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/22/raker-komisi-xiii-dpr-dengan-ksp-2798755.jpg</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>SPPG wajib cantumkan batas waktu konsumsi di ompreng MBG pekan depan</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:57:26 +0700</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>Badan Gizi Nasional (BGN) mewajibkan Satuan Pelayanan Pemenuhan Gizi (SPPG) untuk mencantumkan batas waktu konsumsi ...</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686501/sppg-wajib-cantumkan-batas-waktu-konsumsi-di-ompreng-mbg-pekan-depan</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG-20260809-WA0009_edit_2244477823466886.jpg</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Bulog perkuat Gerakan Pangan Murah di Alor guna stabilkan harga</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:53:34 +0700</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>Perum Bulog memperkuat pelaksanaan Gerakan Pangan Murah (GPM) di Kabupaten Alor, Nusa Tenggara Timur (NTT) guna menjaga ...</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686499/bulog-perkuat-gerakan-pangan-murah-di-alor-guna-stabilkan-harga</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/02C2574B-3D54-49DD-8048-40377485E0F9.jpeg</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>BPJPH perkuat aturan-sanksi soal penyelenggaraan jaminan produk halal</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:52:47 +0700</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>Badan Penyelenggara Jaminan Produk Halal (BPJPH) memperkuat aturan melalui Peraturan BPJPH Nomor 2 Tahun 2026 tentang ...</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686495/bpjph-perkuat-aturan-sanksi-soal-penyelenggaraan-jaminan-produk-halal</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000172109.jpg</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Satgas PRR Aceh Kemendagri tinjau sawah terdampak bencana Aceh Barat</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:51:29 +0700</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>ANTARA - Tim Satgas Percepatan Rehabilitasi dan Rekonstruksi (PRR) Aceh Kemendagri meninjau lokasi persawahan terdampak ...</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686480/satgas-prr-aceh-kemendagri-tinjau-sawah-terdampak-bencana-aceh-barat</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AYM_SATGAS-PRR-ACEH-KEMENDAGRI-TINJAU_1.jpg</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Seskab Teddy disambut Puisi dari Jalanan Menuju Harapan saat tinjau SR</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:51:17 +0700</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>Suara riuh tepuk tangan menggema di Gedung Politeknik Penerbangan Indonesia Curug, Banten. Di hadapan Sekretaris ...</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686493/seskab-teddy-disambut-puisi-dari-jalanan-menuju-harapan-saat-tinjau-sr</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000177274.jpg</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Di hadapan Seskab Teddy, orang tua siswa SR berlinang air mata haru</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:47:37 +0700</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>Ruang makan Gedung Politeknik Penerbangan Indonesia Curug, Banten mendadak dipenuhi suara tawa bahagia dan isak haru. ...</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686491/di-hadapan-seskab-teddy-orang-tua-siswa-sr-berlinang-air-mata-haru</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000177269_1.jpg</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Seskab: Anak putus sekolah berani bermimpi besar di Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:44:29 +0700</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Sekretaris Kabinet Letkol Teddy Indra Wijaya mendorong anak-anak yang sempat putus sekolah maupun belum pernah ...</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686489/seskab-anak-putus-sekolah-berani-bermimpi-besar-di-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000177254_1.jpg</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Kebakaran Lahan di Bromo Capai 520 Hektare, 3 Helikopter Diterjunkan</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:21:52 +0700</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>M Rofiq</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>Petugas berjuang memadamkan kebakaran di Gunung Bromo yang meluas hingga 520 hektare. Tiga helikopter dikerahkan untuk membantu pemadaman.</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610958/kebakaran-lahan-di-bromo-capai-520-hektare-3-helikopter-diterjunkan</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kobaran-api-membakar-kawasan-tnbts-luas-kebakaran-capai-176-hektare-1786243979974_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Program Bedah Rumah Ortu Siswa Sekolah Rakyat Mulai Berjalan di Madura</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:16:51 +0700</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Rahmat Khairurizqi</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>Program bedah rumah orang tua siswa Sekolah Rakyat di Sumenep dimulai. Kolaborasi Kemensos dan Kementerian PKP renovasi 10 ribu unit rumah tidak layak huni.</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610952/program-bedah-rumah-ortu-siswa-sekolah-rakyat-mulai-berjalan-di-madura</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/program-bedah-rumah-ortu-siswa-sekolah-rakyat-mulai-berjalan-di-madura-1786263282323_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Keji! Ayah Cabuli Anak Kandung Iming-imingi Uang Rp 200 Ribu di Depok</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:49:36 +0700</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>Seorang pria ditangkap di Depok karena mencabuli anak kandungnya. Pelaku iming-imingi korban dengan uang Rp 200 ribu.</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610922/keji-ayah-cabuli-anak-kandung-iming-imingi-uang-rp-200-ribu-di-depok</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2015/06/24/aa654593-18dd-45c4-8548-2ae955b419a7_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Alami Gangguan, KRL Bogor-Jakarta Cuma Pakai Satu Jalur di Bojong Gede</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:49:20 +0700</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Farih Maulana Sidik</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>KRL Bogor-Jakarta mengalami keterlambatan akibat gangguan operasional di Stasiun Bojong Gede. KCI mohon maaf dan imbau pengguna untuk mengikuti arahan petugas.</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610921/alami-gangguan-krl-bogor-jakarta-cuma-pakai-satu-jalur-di-bojong-gede</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2018/12/14/d95637d0-4b01-4219-b36e-4e6aaa2935a9_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Sarung Bantal Sofa Diobral di Transmart Full Day Sale</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:00:22 +0700</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>Transmart Full Day Sale kembali hadir pada Minggu (9/8/2026).</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610724/sarung-bantal-sofa-diobral-di-transmart-full-day-sale</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/transmart-full-day-sale-1786251089527_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Laut Hitam Memanas, Turki Desak Rusia-Ukraina Hentikan Serangan ke Kapal Sipil</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:21:45 +0700</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Situasi di Laut Hitam makin panas, Turki mendesak Rusia dan Ukraina untuk menghentikan serangan terhadap kapal sipil.</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866012/laut-hitam-memanas-turki-desak-rusia-ukraina-hentikan-serangan-ke-kapal-sipil</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/uLOIDvtlV0XVuuOhiFXAfSQhrW8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Menlu-Hakan-Fidan-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Depok Besok, Senin 10 Agustus 2026, BMKG: Cerah dari Pagi hingga Malam</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:18:47 +0700</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Simak prakiraan cuaca Senin (10/8/2026), di Depok menurut informasi BMKG besok cuaca cerah pada pagi hingga malam hari.</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866011/prakiraan-cuaca-depok-besok-senin-10-agustus-2026-bmkg-cerah-dari-pagi-hingga-malam</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rkI_12LEXO3BCzMn96LIvnKjTas=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/jalan-ir-h-juanda-yang-jadi-satu-lokasi-rawan-begal-di-depok.jpg</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Misi Tak Kunjung Usai, Perang Iran Seret USS Abraham Lincoln, Ribuan Tentara Kelelahan di Laut</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:12:35 +0700</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>259 hari di laut, USS Abraham Lincoln jadi sorotan. Laporan soal kelelahan awak mencuat, namun Angkatan Laut AS menegaskan kapal tetap siap tempur.</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866010/misi-tak-kunjung-usai-perang-iran-seret-uss-abraham-lincoln-ribuan-tentara-kelelahan-di-laut</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/mA2w8drd_0XOz6rPtbEpDOoAiuE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kapal-induk-kelas-Nimitz-USS-Abraham-Lincoln-CVN-72.jpg</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Bramantyo Suwondo Ajak Warga Magelang Jaga Lingkungan Lewat Gerakan Langit Biru Indonesia ASRI</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:11:46 +0700</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>Anggota DPR RI dari Fraksi Partai Demokrat Bramantyo Suwondo mengajak masyarakat peduli lingkungan lewat kegiatan kerja bakti dan penanaman pohon.</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866009/bramantyo-suwondo-ajak-warga-magelang-jaga-lingkungan-lewat-gerakan-langit-biru-indonesia-asri</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/UAPch0mLSKJDjdZRc8o4_yctDDk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/partai-demokrat-hut-langit-biru.jpg</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Andika Kangen Band Tak Bisa Manggung di Sounds Project Vol.9, Pajang Poster Minta Maaf di Ranjang RS</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:09:35 +0700</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Andika Kangen Band bagikan kondisinya yang tengah terbaring sakit. Ia pun minta maaf tak bisa manggung di The Sounds Project.</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866008/andika-kangen-band-tak-bisa-manggung-di-sounds-project-vol9-pajang-poster-minta-maaf-di-ranjang-rs</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/UFF_cl7cXk60Kt4dm7CkIjJVX1o=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/adnika-kangen-band-sakit.jpg</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Daftar 16 Pemain Timnas Futsal Indonesia yang Ikut Uji Coba ke Spanyol: Evan Absen, Israr Standby</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:06:13 +0700</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>Timnas futsal Indonesia membawa 16 pemain untuk menjalani pemusatan latihan dan rangkaian uji coba di Spanyol pada akhir Agustus ini.</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866007/daftar-16-pemain-timnas-futsal-indonesia-yang-ikut-uji-coba-ke-spanyol-evan-absen-israr-standby</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/XMHmNImszCLLWEFh13QSIOyMJEI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Indonesia-Gagal-Raih-Juara-AFC-Futsal-Asian-Cup-2026_20260208_110254.jpg</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Apakah ASI dan Susu Formula Bisa Sebabkan Karies Gigi Anak?</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:59:12 +0700</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Dokter Gigi Klinik APIC, drg. Nadya Cita Bella menjelaskan orang tua perlu membersihkan mulut anak setelah minum susu dan sebelum tidur.</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866006/apakah-asi-dan-susu-formula-bisa-sebabkan-karies-gigi-anak</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/kyJa-U78i1cGRMMF5skXv16Vuz0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kesehatan-Gigi-Anak-Panti-Asuhan_20250822_204519.jpg</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Semarak HUT ke-81 RI di Papua, Upacara Bendera di Bawah Laut hingga Hiburan Rakyat</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:58:09 +0700</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>Papua menyambut HUT ke-81 RI dengan upacara bawah laut, pembagian 2.000 bendera, serta beragam layanan publik untuk masyarakat</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866005/semarak-hut-ke-81-ri-di-papua-upacara-bendera-di-bawah-laut-hingga-hiburan-rakyat</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iItXS-tN5XPrNVBphpozJUHVwEE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/papua12223233.jpg</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Ayu Ting Ting Bongkar Isi Chat dengan Kevin Gusnadi, Terungkap Panggilan Sayang</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:55:27 +0700</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Penyanyi dangdut Ayu Ting Ting membocorkan isi chat pribadinya dengan sang kekasih, Kevin Gusnadi. Terungkap panggilan sayang keduanya, yaitu "Bebe".</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866004/ayu-ting-ting-bongkar-isi-chat-dengan-kevin-gusnadi-terungkap-panggilan-sayang</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/D0cXy9JcPlAHdV_RnN7CvyZC44A=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ayu-Ting-Ting-3-27052026.jpg</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Soroti Dampak Konflik Ruben Onsu dan Sarwendah, Komnas Anak Singgung Kondisi Psikis: Miris</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:54:35 +0700</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>Komnas Anak menyoroti dampak terhadap anak buntut konflik Ruben Onsu dan Sarwendah. Singgung kondisi psikis.</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866003/soroti-dampak-konflik-ruben-onsu-dan-sarwendah-komnas-anak-singgung-kondisi-psikis-miris</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/GHpt62tuig514FSTblvdMr1GGQc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ruben-Onsu-ketemu-anak22.jpg</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban IPS Kelas 7 SMP Halaman 178 Kurikulum Merdeka Lembar Aktivitas 21 Transaksi Online</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:53:19 +0700</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Soal dan Kunci Jawaban IPS kelas 7 SMP halaman 178, siswa diminta untuk menjawab soal Lembar Aktivitas 21.</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7866002/kunci-jawaban-ips-kelas-7-smp-halaman-178-kurikulum-merdeka-lembar-aktivitas-21-transaksi-online</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ZJH5U9Whl4bTaiBOyK_OIX-A_aE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SISWA-SMP-UJIAN-03.jpg</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Sebelum Membunuh Kunaefi, Saepul Pelaku Mutilasi Curhat Ingin Punya Motor, Tergiur PCX Milik Korban</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:52:17 +0700</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>Pelaku mutilasi di Depok, Saepullah, sempat curhat ingin punya motor dengan cara membunuh.</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866001/sebelum-membunuh-kunaefi-saepul-pelaku-mutilasi-curhat-ingin-punya-motor-tergiur-pcx-milik-korban</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/OjMG3FJ-39duihokZY4K15I_9Os=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pelaku-Mutilasi-di-Depok-Saepullah-12.jpg</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Feby Febiola Pikir Panjang Terima Tawaran Film, Domisili di Luar Jakarta Jadi Pertimbangan</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:47:03 +0700</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>Feby Febiola bersiap untuk kembali meramaikan industri perfilman. Tapi, ia tak mau sembarangan dalam menerima tawaran film.</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866000/feby-febiola-pikir-panjang-terima-tawaran-film-domisili-di-luar-jakarta-jadi-pertimbangan</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/LF0DQo9fIwhbt12KobtZKYehsNA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Feby-febiolamm.jpg</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Indonesia Bawa 12 Pebasket Putri ke Turnamen Jerman, Tantang Wakil Australia, Hungaria, dan Spanyol</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:46:06 +0700</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>12 pebasket putri muda Indonesia siap berlaga di Berlin pada adidas x Alba Next Up Tournament U19.</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865999/indonesia-bawa-12-pebasket-putri-ke-turnamen-jerman-tantang-wakil-australia-hungaria-dan-spanyol</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tUQ8R0_jXSSeXWxwmUC5420MSOc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Imma-Do-Great-Basketball-memboyong-12-pebasket-putri-muda-Indonesia-ke-Berlin.jpg</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Bank Jakarta dan Persija Perluas Kolaborasi ke Layanan Digital</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Bank Jakarta dan Persija Jakarta memperkuat kerja sama untuk musim kompetisi 2026-2027 melalui pengembangan layanan perbankan, program bersama, dan transformasi digital. Kolaborasi tersebut ditandai dengan kick-off “United...</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhrjg416/bank-jakarta-dan-persija-perluas-kolaborasi-ke-layanan-digital</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260809143206-928.png</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Ruang Berkarya Buka Peluang Ekonomi bagi Penyandang Disabilitas</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:12:25 +0700</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Akses penyandang disabilitas terhadap pekerjaan masih terbatas. Data Kementerian Ketenagakerjaan mencatat tingkat partisipasi angkatan kerja dari sekitar 17 juta penyandang disabilitas usia produktif hanya mencapai 20,14 persen...</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjht8c416/ruang-berkarya-buka-peluang-ekonomi-bagi-penyandang-disabilitas</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260809150938-430.png</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Iran Tegaskan tidak akan Buka Selat Hormuz hingga AS Penuhi Syarat</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:03:00 +0700</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Gita Amanda</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TEHERAN -- Iran tidak akan membuka Selat Hormuz sampai Amerika Serikat memenuhi sejumlah syarat, termasuk mengakhiri ancaman terhadap Teheran, kata Sekretaris Dewan Keamanan Nasional Tertinggi (SNSC) Iran Mohammad Bagher Zolghadr,...</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhqo3423/iran-tegaskan-tidak-akan-buka-selat-hormuz-hingga-as-penuhi-syarat</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/warga-iran-berjalan-di-depan-lukisan-raksasa-mengilustrasikan-kapal_260421112547-400.jpg</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Kado HUT RI dari Pemprov DKI, Tarif Transportasi Cuma Rp 1</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Layanan Transjakarta, MRT, dan LRT Jakarta berlaku untuk kebijakan ini.</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265615/kado-hut-ri-dari-pemprov-dki-tarif-transportasi-cuma-rp-1</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/WI1ID511-w7yN8rvJ69EA8_2kkg=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/4308949/original/005498300_1675159370-Tarif_integrasi_transportasi_umum_di_jakarta_masih_di_kaji_pemprov_DKI-ANGGA_3.jpg</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Ribuan Warga Bogor Bentangkan Bendera Merah Putih Raksasa</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 14:57:49 +0700</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>Ribuan warga memadati sepanjang Jalan Kota Bogor, Jawa Barat, Minggu, 9 Agustus 2026, saat kirab bendera Merah Putih dalam Festival Merah Putih 2026. Kirab dimulai pukul 06.00 WIB dari Tugu Kujang melintasi Jalan Otista, Juanda, dan Sudirman hingga berakhir di Pusdikzi, Bogor Tengah. Sebanyak lima rangkaian kain Merah Putih dengan panjang mencapai 100 meter dibentangkan dalam parade. Kegiatan ini digelar untuk menyemarakkan HUT ke-81 RI sekaligus memperkuat semangat nasionalisme.</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/photo/read/8265617/ribuan-warga-bogor-bentangkan-bendera-merah-putih-raksasa</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/ZljpE79IL1nHE0VEWo6fhwxiDM4=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319620/original/035314700_1786262233-ben1.jpg</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>PDIP Banten Punya Cara Baru Dekati Generasi Muda</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:26:25 +0700</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>Strategi baru PDIP Banten untuk merangkul generasi muda diwujudkan melalui pembentukan tim sepak bola.</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265644/pdip-banten-punya-cara-baru-dekati-generasi-muda</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/KHN17mlG7mblWKxHFvbySyCVIkc=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319655/original/039888400_1786263968-5f514824-d73e-40ae-9960-9ca40623e9ee.jpg</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Sumur Bor di Aceh Timur Semburkan Air Setinggi 40 Meter, Ditemukan Gas Mudah Terbakar</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:32:46 +0700</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Sumur bor di Aceh Timur menyemburkan air setinggi 40 meter. Selain itu juga ditemukan gas yang mudah terbakar.</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/09/153231478/sumur-bor-di-aceh-timur-semburkan-air-setinggi-40-meter-ditemukan-gas-mudah</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/EyBdjsYLt_IPGUg5PRZsgEaJyyg=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/09/6a78317b6136d.jpg</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I443"/>
+  <autoFilter ref="A1:I487"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 10:27 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$573</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$616</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I573"/>
+  <dimension ref="A1:I616"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -27367,8 +27367,2031 @@
         </is>
       </c>
     </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Stok Beras Berlimpah, BULOG Perkuat Gerakan Pangan Murah di Alor</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:20:28 +0700</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>Alor (ANTARA) — Perum BULOG memastikan ketersediaan stok beras di Kabupaten Alor, Nusa Tenggara Timur, dalam ...</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686645/stok-beras-berlimpah-bulog-perkuat-gerakan-pangan-murah-di-alor</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/cache/1200x800/no-image.jpg</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Kemnaker: Integrasi data tingkatkan kualitas layanan ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:20:01 +0700</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Kementerian Ketenagakerjaan (Kemnaker) mengatakan penguatan integrasi data lintas instansi berperan penting untuk ...</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686641/kemnaker-integrasi-data-tingkatkan-kualitas-layanan-ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/caa71fb4-a612-4423-9aa0-94826a3f2e39.jpeg</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>KBRI Kuala Lumpur buka layanan penggantian paspor akhir pekan</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:14:12 +0700</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>Kedutaan Besar Republik Indonesia (KBRI) Kuala Lumpur memberi kemudahan bagi warga negara Indonesia di Malaysia yang ...</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686637/kbri-kuala-lumpur-buka-layanan-penggantian-paspor-akhir-pekan</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001046023.jpg</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>BPBD Cianjur turunkan 25 petugas bantu pemadaman di Gunung Gede</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:13:28 +0700</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>Badan Penanggulangan Bencana Daerah Kabupaten Cianjur, Jawa Barat, menurunkan 25 orang petugas dan relawan guna ...</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686635/bpbd-cianjur-turunkan-25-petugas-bantu-pemadaman-di-gunung-gede</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/bepe-deh.jpeg</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>16 pemain timnas futsal Indonesia segera TC di Spanyol</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:12:10 +0700</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>Federasi Futsal Indonsia (FFI) mengumumkan 16 pemain masuk skuad timnas futsal Indonesia untuk melakukan pemusatan ...</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686633/16-pemain-timnas-futsal-indonesia-segera-tc-di-spanyol</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/28/IMG-20260728-WA0213.jpg</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Kuasa hukum sebut Rudy Tanoe minta diperiksa KPK pada 11 Agustus</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:08:26 +0700</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Kuasa hukum Rudijanto Tanoesoedibjo alias Rudy Tanoe, Ricky HP Sitohang, mengatakan kliennya meminta Komisi ...</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686629/kuasa-hukum-sebut-rudy-tanoe-minta-diperiksa-kpk-pada-11-agustus</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/12/14/Screenshot_20231214_140224_Video-Player.jpg</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Ford perkenalkan pikap listrik Fathom, dijual mulai Rp500 jutaan</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:02:09 +0700</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>Ford resmi memperkenalkan pikap listrik terbarunya bernama Fathom yang akan menjadi model pertama yang menggunakan ...</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5686625/ford-perkenalkan-pikap-listrik-fathom-dijual-mulai-rp500-jutaan</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Fathom.jpg</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>DKP DIY optimalkan lahan milik kalurahan untuk budi daya lele dan nila</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:55:55 +0700</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>Dinas Kelautan dan Perikanan (DKP) Daerah Istimewa Yogyakarta (DIY) mengoptimalkan lahan atau tanah milik ...</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686623/dkp-diy-optimalkan-lahan-milik-kalurahan-untuk-budi-daya-lele-dan-nila</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_20260809_155954.jpg</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Indonesia-Iran perkuat kerja sama budaya lewat film dan sastra</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:50:42 +0700</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>Pemerintah Indonesia dan Iran memperkuat kerja sama kebudayaan melalui sejumlah bidang, termasuk perfilman, sastra, ...</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686619/indonesia-iran-perkuat-kerja-sama-budaya-lewat-film-dan-sastra</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-09-at-15.50.48.jpeg</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>DKI luncurkan Pelopor KITA perkuat budaya keselamatan lalu lintas</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:47:56 +0700</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Dinas Perhubungan (Dishub) DKI Jakarta meluncurkan program Pelopor KITA, Keselamatan Lalu Lintas dan Angkutan Jakarta ...</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686615/dki-luncurkan-pelopor-kita-perkuat-budaya-keselamatan-lalu-lintas</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_160340895.jpg</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Indonesia menyerah 1-3 kepada Filipina dalam Leg 2 SEA V Cup</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:40:12 +0700</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>Timnas bola voli putri Indonesia ditaklukkan Filipina 1-3 (13-25, 25-23, 19-25, 31-33) pada pertandingan ketiga Leg 2 ...</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686612/indonesia-menyerah-1-3-kepada-filipina-dalam-leg-2-sea-v-cup</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/06/11/Voli-putri.jpg</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Dua bulan kesulitan air bersih, warga Gurabunga andalkan mata air Ake Goa</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:40:12 +0700</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>Warga mengisi air bersih ke dalam jerigen yang diambil dari sumber mata air Ake Goa di Kelurahan Gurabunga, Tidore, ...</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5686608/dua-bulan-kesulitan-air-bersih-warga-gurabunga-andalkan-mata-air-ake-goa</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Warga-Bergantung-Sumber-Air-Ake-Goa-Di-Tidore-090826-ans-3.jpg</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Gaungkan Tempe Goes to UNESCO, Kowani gelar fun walk 10.000 langkah</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:37:40 +0700</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>Kongres Wanita Indonesia (Kowani) mengadakan fun walk 10.000 langkah sehat dalam rangka menggaungkan gerakan Tempe ...</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686607/gaungkan-tempe-goes-to-unesco-kowani-gelar-fun-walk-10000-langkah</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-09-at-09.28.55.jpg</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Masyarakat Hukum Adat Wehea menanti penetapan</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:36:02 +0700</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>Di antara rimbunnya pepohonan yang menjulang tinggi di enam desa yang terhampar di Kecamatan Muara Wahau, Kutai ...</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686604/masyarakat-hukum-adat-wehea-menanti-penetapan</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/MHA-Wehea-37.jpeg</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Perlukah mencuci semua buah dan sayur sebelum dimakan?</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:36:02 +0700</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>Buah dan sayuran segar sebaiknya tetap dicuci sebelum dikonsumsi untuk membantu menghilangkan kotoran, pestisida, dan ...</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686603/perlukah-mencuci-semua-buah-dan-sayur-sebelum-dimakan</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/08/13/Pameran-Agrinex-28032014-pus-31.jpg</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Ribuan warga Bogor kirab bendera Merah Putih sepanjang 500 meter</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:32:25 +0700</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>Ribuan warga mengikuti kirab bendera Merah Putih raksasa sepanjang 500 meter dalam rangkaian Festival Merah Putih (FMP) ...</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686601/ribuan-warga-bogor-kirab-bendera-merah-putih-sepanjang-500-meter</t>
+        </is>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1003325683.jpg</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Top! Capaian Dekarbonisasi Pertamina di Semester I 2026 Tembus 118%</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:07:19 +0700</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Rahmat Khairurizqi</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>Pertamina berhasil melampaui target dekarbonisasi dengan pengurangan emisi 118% di 2026. Komitmen ESG dan bisnis rendah karbon terus dikembangkan.</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8611072/top-capaian-dekarbonisasi-pertamina-di-semester-i-2026-tembus-118</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/pertamina-1786269972998.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Ekonomi RI Bisa Tumbuh Tinggi, tapi Ada Syaratnya</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:00:13 +0700</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>Ekonom Senior Indef Didik J Rachbini mengungkapkan penyebab pertumbuhan ekonomi Indonesia hanya berada di kisaran 5%.</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8611028/ekonomi-ri-bisa-tumbuh-tinggi-tapi-ada-syaratnya</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/05/27/bangkit-dari-pandemi-ekonomi-ri-kuartal-ii-2021-diramal-tembus-7-3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Kasus Temuan 996 Senjata di Sekolah Swasta Pondok Pinang, IWD Diduga Ingin Ambil Alih Yayasan</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:11:13 +0700</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>Satu senjata api dan ratusan airsoft gun ditemukan di sebuah sekolah swasta di Kebayoran lama.</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866050/kasus-temuan-996-senjata-di-sekolah-swasta-pondok-pinang-iwd-diduga-ingin-ambil-alih-yayasan</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/enu60eSCVJ1ALLFEmi5pFfeMTg4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/996-senjata-di-sebuah-sekolah-kawasan-Pondok-Pinang-32010.jpg</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Keisya Levronka dan Razan Zu Ungkap Keseruan Syuting Film 'Dan Bandung'</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:10:31 +0700</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Keisya Levronka dan Razan Zu menceritakan keseruan saat syuting film Dan Bandung. Menurut Keisya, Kota Bandung memiliki suasana yang menenangkan.</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866049/keisya-levronka-dan-razan-zu-ungkap-keseruan-syuting-film-dan-bandung</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/UHZ9-t3bj-vfurIaaRIbrZpYIRY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Keisya-Levronka-1-29072025.jpg</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Samsung Rilis ISOCELL HPC, Sensor Kamera 200 MP dengan HDR 16-bit</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:08:28 +0700</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>Samsung memperkenalkan ISOCELL HPC yaitu sensor kamera 200 MP dengan HDR 16-bit dan Zoom HDR hingga 4x. Berikut penjelasan spesifikasinya.</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/techno/7866048/samsung-rilis-isocell-hpc-sensor-kamera-200-mp-dengan-hdr-16-bit</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ZOC4LyBmgETx7UFuChOm9u-acsw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SENSOR-BARU-SAMSUNG-3453453.jpg</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>DPR Tunggu Surpres Calon Gubernur BI, Fit and Proper Test Diharap Digelar di Masa Sidang Mendatang</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:52:28 +0700</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>setelah surpres tersebut masuk nantinya, maka DPR melalui Komisi XI akan melakukan fit and proper test atau uji kelayakan</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7866047/dpr-tunggu-surpres-calon-gubernur-bi-fit-and-proper-test-diharap-digelar-di-masa-sidang-mendatang</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/O_cWjD8PKOltHmJKejl9Vf6Z2_U=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Logo-Bank-Indonesia-di-gedung-Bank-Indonesia.jpg</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Inovasi Hasil Laut Dorong Ekonomi dan Kelestarian Pesisir Kampung Tua Terih Batam</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:50:07 +0700</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>Program ini meningkatkan pendapatan kelompok sekaligus mengurangi sampah dan mendukung rehabilitasi mangrove.</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7866046/inovasi-hasil-laut-dorong-ekonomi-dan-kelestarian-pesisir-kampung-tua-terih-batam</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/a4qs5LTdLZBVuExVX9JeDeXT0TE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kampung-Bahari-Si-Pelaut.jpg</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Rekap Hasil Final Korea Masters 2026: 3 Sejarah Lahir, 5 Sektor Punya Juara Baru</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:43:37 +0700</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>Final Korea Masters 2026 melahirkan 3 sejarah baru sekaligus memastikan lima sektor memiliki juara berbeda pada turnamen Super 300 di Asan.</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866045/rekap-hasil-final-korea-masters-2026-3-sejarah-lahir-5-sektor-punya-juara-baru</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/mTgQQN2z3RBUhH0D74fVWlhu1cE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/YutaMaya-Juara-Korea-Masters-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>PCNU Tangsel Resmi Dilantik, Ini Tujuh Arah Khidmat 2026-2031</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:42:14 +0700</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>PCNU Tangsel 2026-2031 resmi dilantik, Gus Mas’ud tekankan khidmat NU: penguatan jamiyah, pemberdayaan jamaah, dan ekonomi mandiri.</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866044/pcnu-tangsel-resmi-dilantik-ini-tujuh-arah-khidmat-2026-2031</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/HJCOcQcTeCWDlhv2_Pg71J3-eVE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pelantikan-PCNU-Tangsel-Periode-2026-2031.jpg</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Revisi UU Pemilu Belum Punya Draf dan Naskah Akademik, Pakar Soroti Lambannya Pembahasan</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:37:01 +0700</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>Revisi UU Pemilu yang telah masuk Program Legislasi Nasional (Prolegnas) Prioritas 2025 dan 2026 hingga kini belum juga memiliki naskah akademik.</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866043/revisi-uu-pemilu-belum-punya-draf-dan-naskah-akademik-pakar-soroti-lambannya-pembahasan</t>
+        </is>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/2PQ-9K1jB9Nr3MuycLoORz7UPyE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pakar-hukum-pemilu-Titi-Anggraini-3102938.jpg</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Raih 5 Emas, 4 Perak, 17 Perunggu, Indonesia Juara Umum 8th Asian Taekwondo Open Championships 2026</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:34:10 +0700</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>Atlet Indonesia menjadi juara umum 8th Asian Taekwondo Indonesia Open Championships 2026 yang digelar di Jakarta.</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866042/raih-5-emas-4-perak-17-perunggu-indonesia-juara-umum-8th-asian-taekwondo-open-championships-2026</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/6EPdxqRi3FKq_7-PczKBVFPC-Cg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kejuaraan-takewondo-ws.jpg</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Megawati Hadiri Peluncuran Buku Autobiografi Erros Djarot, Ada Anies Baswedan hingga Menkop Ferry</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:29:58 +0700</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>Ketua Umum DPP PDI Perjuangan (PDIP), Megawati Soekarnoputri menghadiri acara peluncuran buku Autobiografi Erros Djarot volume 2 dan 3.</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866041/megawati-hadiri-peluncuran-buku-autobiografi-erros-djarot-ada-anies-baswedan-hingga-menkop-ferry</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5gAc5qnmxo78QKWzrv7ABMkfjFg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Megawati-Soekarnoputri-menghadiri-acara-peluncuran-buku-Autobiografi-Erros-Djarot.jpg</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Spek Xiaomi Redmi Note 17 vs Redmi Note 17 Pro, Pilih yang Mana?</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:27:58 +0700</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>Xiaomi China resmi memperkenalkan Redmi Note 17 vs Redmi Note 17 Pro. Dua varian ini kemungkinan akan dirilis di Indonesia. Berikut speknya.</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/techno/7866040/spek-xiaomi-redmi-note-17-vs-redmi-note-17-pro-pilih-yang-mana</t>
+        </is>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/olMgHSXWRE5ZrYHWW6ONj2P1guc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/REDMI-NOTE-17-PRO-34534534.jpg</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>S-400 Rusia Dikabarkan Sempat Tembak Jatuh 24 Jet Tempur Ukraina, 10 MiG-29 Hancur dalam Sehari</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:25:55 +0700</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>Informasi mengenai operasi tersebut terungkap dalam publikasi jurnal militer Rusia Voyennaya Mysl atau Military Thought.</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866039/s-400-rusia-dikabarkan-sempat-tembak-jatuh-24-jet-tempur-ukraina-10-mig-29-hancur-dalam-sehari</t>
+        </is>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/NQ9AWrMHJGPyM6lP2PdDzS1K3Zw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sistem-pertahanan-udara-Rusia-S-300-dan-S-400.jpg</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Cirebon Senin, 10 Agustus 2026: Waspada, Suhu Matahari Tembus 35 Derajat</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:24:30 +0700</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>Menurut pantauan BMKG Jawa Barat  prakiraan cuaca untuk wilayah Cirebon pada Senin (10/8/2026) cerah dengan potensi terik matahari yang menyengat.</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7866038/prakiraan-cuaca-cirebon-senin-10-agustus-2026-waspada-suhu-matahari-tembus-35-derajat</t>
+        </is>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5NsvRAfKVVqlNUGVnYRGovtF7v4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-cerah-berawan-8.jpg</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Kumpulan Puisi Bertema Kemerdekaan 2026, Cocok untuk Dibacakan saat Perayaan HUT Ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:24:09 +0700</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>Hari Kemerdekaan akan segera tiba, berikut contoh kumpulan teks puisi bertema Hari Kemerdekaan Indonesia, untuk memeriahkan HUT ke-81 RI.</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866037/kumpulan-puisi-bertema-kemerdekaan-2026-cocok-untuk-dibacakan-saat-perayaan-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rOHHaL3nFdAXtANu847n5YbI8lQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pembagian-Bendera-Merah-Putih_20250808_150014.jpg</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>5 Ciri Warga Kelas Bawah, Cek Ada di Kamu?</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:00:02 +0700</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto soroti penurunan kemiskinan ekstrem di WEF Davos. Artikel ini membahas lima indikator ekonomi kelas bawah dan menengah.</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260809153202-17-757732/5-ciri-warga-kelas-bawah-cek-ada-di-kamu</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/06/02/suasana-aktivitas-warga-pada-permukiman-kumuh-yang-berdekatan-dengan-rel-kereta-di-jakarta-senin-262025-cnbc-indonesiafaisal-r-1748854425015_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Riwayat Kredit Jelek? Ini Cara Bersihkan Nama di SLIK OJK</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>Skor kredit dalam SLIK OJK penting saat mengajukan pinjaman. Pelajari cara memperbaiki catatan kredit buruk dan pentingnya pembaruan data.</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260809152900-17-757731/riwayat-kredit-jelek-ini-cara-bersihkan-nama-di-slik-ojk</t>
+        </is>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2020/02/06/408afd32-323a-4fe1-b91b-aa3022b4b547_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>New Daihatsu Sigra 1.2R Hadir dengan Sejumlah Penyegaran</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:09:04 +0700</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, 
+TANGERANG -- Daihatsu memperkenalkan penyegaran Astra Daihatsu Sigra varian 1.2R pada ajang Gaikindo Indonesia International Auto Show (GIIAS) 2026 di ICE BSD City, Tangerang. Pembaruan mencakup sejumlah bagian eksterior,...</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhyv4348/new-daihatsu-sigra-12r-hadir-dengan-sejumlah-penyegaran</t>
+        </is>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260729232442-602.png</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>Energi</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Tingkatkan Layanan, Pertamina Resmikan Integrasi Informasi Publik</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:52:48 +0700</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>Ferry kisihandi</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- PT Pertamina (Persero) resmi meluncurkan Integrasi Layanan Informasi Publik sebagai semangat baru dalam menghadirkan layanan informasi yang informatif. 
+Peluncuran ini mencerminkan komitmen Pertamina sebagai perusahaan yang...</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjhy40472/tingkatkan-layanan-pertamina-resmikan-integrasi-informasi-publik</t>
+        </is>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/pertamina-meluncurkan-integrasi-layanan-informasi-publik-yang-menjadi-cermin_260809165134-517.jpeg</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>DPRD Bandung Petakan Risiko Proyek RSUD dan Gedung Inspektorat, Cegah Molor hingga Anggaran Membengkak</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:23:37 +0700</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>DPRD Bandung memetakan risiko hukum, teknis, hingga anggaran proyek RSUD dan Gedung Inspektorat agar pembangunan berjalan sesuai target.</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265702/dprd-bandung-petakan-risiko-proyek-rsud-dan-gedung-inspektorat-cegah-molor-hingga-anggaran-membengkak</t>
+        </is>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/idH9FwrPo2yJPCCPYo80X89EqWA=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319714/original/090819300_1786271016-9ab54bb3-9640-492b-b913-56b1036d7f7c__1_.jpeg</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Megawati Hadiri Peluncuran Buku Erros Djarot, Ada Menkop sampai Anies</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:17:09 +0700</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Tokoh politik dan seniman turut meramaikan acara tersebut.</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265698/megawati-hadiri-peluncuran-buku-erros-djarot-ada-menkop-sampai-anies</t>
+        </is>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/5jdeogdvVllKSJm43QV9hJYO5lQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319703/original/014102400_1786270609-93aae30a-3030-410e-96a6-5cda6e195d96.jpg</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Kekeringan Ancam 12 Kecamatan di Kabupaten Tangerang</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:07:26 +0700</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>Memiliki curah hujan yang sangat rendah, sebanyak 12 wilayah di Kabupaten Tangerang masuk dalam kategori waspada kekeringan.</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265696/kekeringan-ancam-12-kecamatan-di-kabupaten-tangerang</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/mjPdIrRvElAsO8GtlqwxKuGVneE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/4565724/original/045442100_1693995926-20230906-Kekeringan_di_Sawah-ANG_7.jpg</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>KPK Geledah 15 Lokasi di Kasus Bupati Pemalang, Ini Hasilnya</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:42:42 +0700</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>KPK mengamankan sejumlah barang bukti saat penggeledahan terkait kasus Bupati Pemalang nonaktif Anom Widiyantoro.</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265685/kpk-geledah-15-lokasi-di-kasus-bupati-pemalang-ini-hasilnya</t>
+        </is>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/N33opNKiRzfdpkapW0QV5UgcMEU=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9310910/original/007198200_1785380863-pem5.jpg</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Komnas PA Tunjuk 5 Figur Anak Jadi Duta Anti-bullying, Ada Farel Prayoga</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:27:56 +0700</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>Komnas PA menobatkan 5 figur anak, termasuk penyanyi Farel Prayoga dan influencer cilik, sebagai Duta Anak Anti-Bullying 2026. Mereka akan kampanye anti-perundungan.</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/09/17274871/komnas-pa-tunjuk-5-figur-anak-jadi-duta-anti-bullying-ada-farel-prayoga</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/H8csFFxNBBDoCeGejHDBPpbMWDY=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/09/6a78506aef334.jpg</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>Edukasi</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>KPAI Soroti Masih Adanya Masalah Tata Kelola MBG, Ini Rekomendasinya</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:27:56 +0700</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>Komisi Perlindungan Anak Indonesia (KPAI) masih melihat ada permasalahan krisis tata kelola di program Makan Bergizi Gratis (MBG).</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/edu/read/2026/08/09/164637971/kpai-soroti-masih-adanya-masalah-tata-kelola-mbg-ini-rekomendasinya</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/i3phhwWRZgzddtFWs_8GLlOR4_I=/113x0:1080x645/1200x675/filters:watermark(data/photo/2026/01/30/697c819b2dbec.png,0,-0,1)/data/photo/2026/06/20/6a362c78137f0.jpg</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>Edukasi</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Waspada Stroke di Kamar Mandi, Pakar Neurologi Unesa Ungkap Penyebab dan Cara Mencegahnya</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:27:56 +0700</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Berdasarkan pengalaman lebih dari satu dekade menangani pasien, ia menemukan pola yang berulang ketika menerima pasien stroke di IGD.</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>https://edukasi.kompas.com/read/2026/08/09/161117771/waspada-stroke-di-kamar-mandi-pakar-neurologi-unesa-ungkap-penyebab-dan-cara</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/WlYlO2owCLbMCslCEzuoAQ3DItE=/2x0:1000x665/1200x675/filters:watermark(data/photo/2026/01/30/697c819b2dbec.png,0,-0,1)/data/photo/2022/06/26/62b84da354aea.jpg</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I573"/>
+  <autoFilter ref="A1:I616"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 11:23 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$616</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$662</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I616"/>
+  <dimension ref="A1:I662"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -29390,8 +29390,2170 @@
         </is>
       </c>
     </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>JMP kecam hoaks kerusuhan di Jakarta, ingatkan bahaya provokasi</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:14:30 +0700</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Jurnalis Mitra Polri (JMP) mengecam penyebaran hoaks dan narasi provokatif terkait isu kerusuhan di Jakarta yang ...</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686684/jmp-kecam-hoaks-kerusuhan-di-jakarta-ingatkan-bahaya-provokasi</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Aksi-28-Agustus-2025-280825-RIV-3.jpg</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Resmi dilantik, ini tujuh arah khidmat PCNU Tangsel periode 2026-2031</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:10:42 +0700</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>Pengurus Cabang Nahdlatul Ulama (PCNU) Kota Tangerang Selatan periode 2026-2031 menetapkan tujuh arah khidmat mencakup ...</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686680/resmi-dilantik-ini-tujuh-arah-khidmat-pcnu-tangsel-periode-2026-2031</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-09-at-3.51.40-PM.jpeg</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Fans Messi berikan penghormatan untuk mendiang sang ayah</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:08:28 +0700</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>ANTARA - Para penggemar pesepak bola Lionel Messi dan warga Kota Rosario, Argentina, pada Minggu (9/*8), memberikan ...</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686555/fans-messi-berikan-penghormatan-untuk-mendiang-sang-ayah</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/FANS-MESSI-BERIKAN-PENGHORMATAN-UNTUK-MENDIANG-SANG-AYAH.jpg</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Kemenimipas dorong semangat kepedulian lewat donor darah HUT RI</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:05:35 +0700</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>Kementerian Imigrasi dan Pemasyarakatan mendorong semangat kepedulian melalui kegiatan donor darah menyambut Hari Ulang ...</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686679/kemenimipas-dorong-semangat-kepedulian-lewat-donor-darah-hut-ri</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG-20260809-WA0007.jpg</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Jaecoo J5 EV catat penjualan 3.200 unit pada Juli 2026</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:01:29 +0700</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>Mobil listrik Jaecoo J5 EV mencatat penjualan sebanyak 3.200 unit pada Juli 2026, meningkat sekitar 4,9 persen ...</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5686676/jaecoo-j5-ev-catat-penjualan-3200-unit-pada-juli-2026</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/26/1000921601.jpg</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Luas panen padi Indonesia 2026 capai 9,46 juta hektare, naik dari tahun lalu</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:55:51 +0700</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Foto udara pekerja memanen padi menggunakan mesin pertanian modern (Combine Harvester) di area persawahan kawasan ...</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5686672/luas-panen-padi-indonesia-2026-capai-946-juta-hektare-naik-dari-tahun-lalu</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Luas-Panen-Padi-Januari-September-2026-Meningkat-090826-Um-2.jpg</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Volkswagen siapkan model pikap baru untuk pasar Amerika Serikat</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:48:41 +0700</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Volkswagen tengah menyiapkan pikap baru sebagai strategi perusahaan memperkuat posisinya di pasar otomotif Amerika ...</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5686669/volkswagen-siapkan-model-pikap-baru-untuk-pasar-amerika-serikat</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/AM001343PIC-vw-amarok-Aventura-center-stage-lp-5.jpg</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Penduduk Penajam tembus 206 ribu kursi DPRD bisa bertambah</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:44:36 +0700</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Pertumbuhan penduduk Kabupaten Penajam Paser Utara, Kalimantan Timur, berpotensi meningkatkan jumlah kursi DPRD ...</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686668/penduduk-penajam-tembus-206-ribu-kursi-dprd-bisa-bertambah</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_20250307_162218.jpg</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Indonesia jamu Rumania pada Piala Davis  Grup II Dunia 2026</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:35:47 +0700</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Indonesia akan menjamu Rumania pada Piala Davis Grup II Dunia 2026 yang dijadwalkan berlangsung pada 18-20 September ...</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686665/indonesia-jamu-rumania-pada-piala-davis-grup-ii-dunia-2026</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/08/Tim-tenis-Indonesia-lolos-Grup-II-Dunia-Piala-Davis-2026-080226-sth-09.jpg</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Pram: Transjakarta kelola transporasi laut Kepulauan Seribu mulai 2027</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:31:35 +0700</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Gubenur DKI Jakarta Pramono Anung menyebut pengelolaan transportasi laut hingga mencakup wilayah Kepulauan Seribu yang ...</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686664/pram-transjakarta-kelola-transporasi-laut-kepulauan-seribu-mulai-2027</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_163639468.jpg</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>NEXT ingatkan nasabah perlu cermati konsekuensi bunga simpanan tinggi</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:31:26 +0700</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>NEXT Indonesia Center mengingatkan masyarakat untuk mencermati ulang konsekuensi bunga simpanan yang tinggi atau berada ...</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686660/next-ingatkan-nasabah-perlu-cermati-konsekuensi-bunga-simpanan-tinggi</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/30/IMG_20260430_102209.jpg</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Menhut sebut "water bombing" dioptimalkan padamkan api di lereng Bromo</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:29:59 +0700</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Menteri Kehutanan (Menhut) Raja Juli Antoni menyatakan keberadaan helikopter water bombing atau pengebom air ...</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686657/menhut-sebut-water-bombing-dioptimalkan-padamkan-api-di-lereng-bromo</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001409951.jpg</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Jangan sepelekan saraf terjepit, bisa berujung kelumpuhan</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:27:17 +0700</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>ANTARA - Saraf terjepit tak selalu sekadar menimbulkan nyeri dan kesemutan. Jika tekanan pada saraf atau sumsum tulang ...</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686535/jangan-sepelekan-saraf-terjepit-bisa-berujung-kelumpuhan</t>
+        </is>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Thumbnai-BiSa-Saraf-Kejepit-01_5.jpg</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Kolaborasi Bank Jakarta-Persija perkuat simbol dan kebanggaan warga</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:25:00 +0700</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) DKI Jakarta mendukung penuh kolaborasi Bank Jakarta dan Persija sebagai sinergi dua ...</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686655/kolaborasi-bank-jakarta-persija-perkuat-simbol-dan-kebanggaan-warga</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_164830830.jpg</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Puluhan ribu warga Semarang meriahkan festival tari Dug Dug Der</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:24:51 +0700</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>ANTARA - Sebanyak puluhan ribu orang meramaikan festival tari Dug Dug Der Semarangan di Lapangan Pancasila, Kawasan ...</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686599/puluhan-ribu-warga-semarang-meriahkan-festival-tari-dug-dug-der</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PULUHAN-RIBU-WARGA-SEMARANG-MERIAHKAN-FESTIVAL-TARI-DUG-DUG-DER.jpg</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Telur retak masih aman dimakan? Ini penjelasan ahli</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:24:30 +0700</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Telur dengan cangkang retak tidak selalu harus dibuang, tetapi keamanan telur bergantung pada kapan retakan terjadi dan ...</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686651/telur-retak-masih-aman-dimakan-ini-penjelasan-ahli</t>
+        </is>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/IMG_20230523_111545-1.jpg</t>
+        </is>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Satgas Yonif 511/DY gelar makan bergizi ke-22 di Lanny Jaya</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:23:39 +0700</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Satgas Pamtas Yonif 511/DY menggelar program makan bergizi bagi 150 warga Kampung Tima, Distrik Balingga, Kabupaten ...</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686647/satgas-yonif-511-dy-gelar-makan-bergizi-ke-22-di-lanny-jaya</t>
+        </is>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-08-at-14.22.02.jpeg</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Yayasan Ungkap Awal Mula Ditemukan Ratusan Senjata di Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:16:34 +0700</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Pemilik yayasan sekolah swasta di Jakarta Selatan mengungkap penemuan ratusan senjata. Terdapat konflik internal terkait kepemilikan dan izin senjata tersebut.</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611155/yayasan-ungkap-awal-mula-ditemukan-ratusan-senjata-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/pendiri-yayasan-sekolah-swasta-di-jaksel-yang-ditemukan-senjata-adrialdetikcom-1786266610236_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Kebakaran Gudang di Tangerang Mulai Pendinginan Usai 6 Jam Terbakar</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:00:16 +0700</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Kebakaran di pergudangan Kosambi, Tangerang, melibatkan tiga gudang. Saat ini, petugas sedang proses pendinginan.</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611140/kebakaran-gudang-di-tangerang-mulai-pendinginan-usai-6-jam-terbakar</t>
+        </is>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/10/17/ilustrasi-kebakaran_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Dari Tali Baja ke Jembatan Perintis, Asa Warga Desa Sikundo Segera Terwujud</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:22:19 +0700</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Chayyara Zulghifary</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Pembangunan Jembatan Gantung Perintis Garuda di Desa Sikundo diharapkan selesai Agustus 2026, memudahkan akses warga dan menghidupkan kembali aktivitas ekonomi.</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611092/dari-tali-baja-ke-jembatan-perintis-asa-warga-desa-sikundo-segera-terwujud</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/dari-tali-baja-ke-jembatan-perintis-asa-warga-desa-sikundo-segera-terwujud-1786270876960.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Pertamina Resmikan Integrasi Layanan Informasi Publik, Ini Tujuannya</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:16:12 +0700</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Annisa Sekar Melati</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Pertamina meluncurkan Integrasi Layanan Informasi Publik untuk meningkatkan keterbukaan dan kualitas layanan.</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611087/pertamina-resmikan-integrasi-layanan-informasi-publik-ini-tujuannya</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/pertamina-resmikan-integrasi-layanan-informasi-publik-1786270550016.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Ditangkap Polisi, Jukir Liar di Tambora Paksa Pemotor Bayar Parkir Rp 5.000</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:15:52 +0700</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Polisi tangkap juru parkir liar di Tambora yang memaksa pemotor bayar Rp 5.000. Pelaku positif narkoba dan menggunakan karcis kedaluwarsa.</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611086/ditangkap-polisi-jukir-liar-di-tambora-paksa-pemotor-bayar-parkir-rp-5-000</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/07/25/ilustrasi-penangkapan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Hari Anak Nasional, Komnas Anak Soroti Fenomena Bullying Sejak Kelas 1 SD</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:11:30 +0700</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Adhfar</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Komnas Anak DKI Jakarta memperingati Hari Anak Nasional 2026 dengan diskusi untuk menekan bullying. Lima anak terpilih sebagai Duta Anak Anti-bullying.</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611074/hari-anak-nasional-komnas-anak-soroti-fenomena-bullying-sejak-kelas-1-sd</t>
+        </is>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/komisi-nasional-perlindungan-anak-komnas-anak-dki-jakarta-memperingati-hari-anak-nasional-2026-1786270267101_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Komnas Anak soal Temuan Senjata di Sekolah Jaksel: Harusnya Jadi Tempat Aman</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:04:30 +0700</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Adhfar Aulia Syuhada</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Komnas Anak soroti temuan ratusan senjata di sekolah swasta Jaksel. Mereka mendesak agar sekolah jadi tempat aman dan mendukung penyelidikan polisi.</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611066/komnas-anak-soal-temuan-senjata-di-sekolah-jaksel-harusnya-jadi-tempat-aman</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/ruangan-mantan-kepala-yayasan-ditemukannya-senjata-di-sekolah-swasta-jaksel-taufiqdetikcom-1786104460641_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Jukir Liar yang Ajak Duel-Paksa Pemotor Bayar di Tambora Positif Narkoba</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:46:58 +0700</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Polisi menangkap juru parkir liar 'Bang Jago' di Jakarta Barat yang memaksa tarif parkir dan mengajak duel pengendara. Pelaku juga positif narkoba.</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611053/jukir-liar-yang-ajak-duel-paksa-pemotor-bayar-di-tambora-positif-narkoba</t>
+        </is>
+      </c>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2015/11/06/6da17d61-730f-4c82-8d3a-363b30d553a8_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Yayasan Sekolah Jaksel Bantah Polemik Penemuan Senjata karena Konflik Pendiri</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:40:26 +0700</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Yayasan sekolah swasta di Jakarta Selatan bantah konflik antarpendiri terkait penemuan senjata. Kuasa hukum menegaskan fokus pada pendidikan anak.</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611035/yayasan-sekolah-jaksel-bantah-polemik-penemuan-senjata-karena-konflik-pendiri</t>
+        </is>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/alvon-kurnia-parma-pengacara-yayasan-sekolah-di-jaksel-tempat-temuan-senjata-saat-konferensi-pers-1786267194234_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Kemenhub Ungkap 56% Perjalanan Bus AKAP Melakukan Pelanggaran</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:00:43 +0700</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>Lebih dari separuh perjalanan bus AKAP yang berangkat dari terminal tipe A terindikasi melakukan pelanggaran.</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8611123/kemenhub-ungkap-56-perjalanan-bus-akap-melakukan-pelanggaran</t>
+        </is>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/07/28/operasional-terminal-cicaheum-bandung-bakal-dihentikan-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Menyulap Sampah Plastik Menjadi Paving Blok</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:00:32 +0700</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Rafida Fauzia</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Sampah plastik tertolak diolah menjadi paving blok di Jakarta. Dalam sehari, satu ton sampah plastik dapat menghasilkan 500 meter persegi paving.</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8610407/menyulap-sampah-plastik-menjadi-paving-blok</t>
+        </is>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/menyulap-sampah-plastik-menjadi-paving-blok-1786209238331.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Perbankan Wajib Transformasi Biar Nasabah Makin Nyaman</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:42:31 +0700</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Sylke Febrina Laucereno</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Inovasi layanan dan teknologi jadi kunci untuk inklusi keuangan.</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8611153/perbankan-wajib-transformasi-biar-nasabah-makin-nyaman</t>
+        </is>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/12/24/ilustrasi-bank-digital_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Pemerintah Diminta Lakukan Hal Ini buat Geber Pertumbuhan Ekonomi Digital</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:57:59 +0700</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Sylke Febrina Laucereno</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>Pemerintah diminta membangun ekosistem digital yang melibatkan platform global untuk mendukung pertumbuhan ekonomi digital.</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8611100/pemerintah-diminta-lakukan-hal-ini-buat-geber-pertumbuhan-ekonomi-digital</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/03/28/ilustrasi-transaksi-digital-1774668306314_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>5 Lowongan Kerja British Council Indonesia, Posisi Manajer hingga Kepala Bidang</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:00:50 +0700</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>British Council Indonesia membuka lowongan kerja untuk 5 posisi di antaranya Manajer hingga Kepala Bidang. Berikut informasi lengkapnya.</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866060/5-lowongan-kerja-british-council-indonesia-posisi-manajer-hingga-kepala-bidang</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hPbiJwwRUgJWdQQUS4Itj8Hqzrg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/LOWONGAN-KERJA-3453454353.jpg</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Demi Rawat Ibu Sakit, Aldi Taher Berencana Jual Rumah Agar Lebih Dekat</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:59:16 +0700</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>Aldi Taher tengah berusaha memberikan perhatian lebih kepada kedua orangtuanya, terutama sang ibu yang masih menjalani proses pemulihan</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866059/demi-rawat-ibu-sakit-aldi-taher-berencana-jual-rumah-agar-lebih-dekat</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ZqOxiGFA4_9uMfWNTtQvWNAVab8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/aldi-taher-triad.jpg</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Banyumas, Senin 10 Agustus 2026: Seluruh Kecamatan Berawan</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:50:40 +0700</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Pada hari Senin, 10 Agustus 2026, daerah Kabupaten Banyumas, Jawa Tengah, diprediksi akan berawan.</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866058/prakiraan-cuaca-banyumas-senin-10-agustus-2026-seluruh-kecamatan-berawan</t>
+        </is>
+      </c>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5NsvRAfKVVqlNUGVnYRGovtF7v4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-cerah-berawan-8.jpg</t>
+        </is>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Pengalaman Pengunjung GIIAS 2026 Setelah Test Drive Grand Vitara Facelift 2026</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:46:37 +0700</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>Suzuki Grand Vitara menjadi model SUV yang banyak diminati pengunjung GIIAS 2026 untuk dijajal performanya di area test drive.</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7866057/pengalaman-pengunjung-giias-2026-setelah-test-drive-grand-vitara-facelift-2026</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/yyN3AZ6dbpSNeWbEiMwJO_ihk-s=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/suzuki-vitara-930.jpg</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Jadwal Acara TV Senin, 10 Agustus 2026: Lapor Pak! TRANS 7 dan Cipung Abubu Mentari TV</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:39:08 +0700</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Simak jadwal acara TV besok Senin 10 Agustus 2026 terdapat tayangan Lapor Pak! TRANS 7 dan Cipung Abubu Mentari TV.</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866056/jadwal-acara-tv-senin-10-agustus-2026-lapor-pak-trans-7-dan-cipung-abubu-mentari-tv</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/H5aLayjCy83MjA-P9TOjSo-_9Qw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ILUSTRASI-TELEVISI-3.jpg</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Pria Bunuh Teman Kencan di Kamar Indekos Pinrang Sulsel, Berawal Dari Pelaku Kurang Bawa Uang</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:34:15 +0700</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Wanita berinisial IN tewas dibunuh teman kencan di kamar indekos Kabupaten Pinrang, Sulawesi Selatan (Sulsel). berikut kronologi dan motifnya</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866055/pria-bunuh-teman-kencan-di-kamar-indekos-pinrang-sulsel-berawal-dari-pelaku-kurang-bawa-uang</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0vnfr07ygtSQr0kVzLyuJpOqNYY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ilustrasi-pembunuhan-wae-lah.jpg</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Rekrutmen PCPM Bank Indonesia Angkatan 41 Dibuka, Lolos Jadi Asisten Manajer BI</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:31:58 +0700</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Rekrutmen PCPM Bank Indonesia Angkatan 41 dibuka hingga 14 Agustus 2026. Pelamar yang lolos akan menjadi Asisten Manajer BI melalui pelatihan.</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866054/rekrutmen-pcpm-bank-indonesia-angkatan-41-dibuka-lolos-jadi-asisten-manajer-bi</t>
+        </is>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Alq4sHcRpPrD7j1TcXqnXvkqIFc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/LOWONGAN-KERJA-BI-34534534.jpg</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Saor Siagian Desak Polisi Bekerja Tanpa Beban Psikologis Usut Kematian Sutrimo, Singgung Tantangan</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:31:53 +0700</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Kepolisian diminta melakukan ekshumasi atau pengangkatan jenazah Sutrimo untuk menemukan penyebab kematiannya.</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866053/saor-siagian-desak-polisi-bekerja-tanpa-beban-psikologis-usut-kematian-sutrimo-singgung-tantangan</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ooGbxXPeqJD9m-KyAxapZgHY_PQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/praktisi-hukum-dan-pegiat-antikorupsi-saor-siagian-yy.jpg</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Live Race MotoGP Inggris 2026 Jam 19.00 WIB: Jorge Martin Bidik Kemenangan, Ducati Kejar Aprilia</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:27:48 +0700</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>Pantau live hasil MotoGP Inggris 2026 malam ini mulai pukul 19.00 WIB dengan pasukan Aprilia lebih diunggulkan ketimbang Ducati.</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866052/live-race-motogp-inggris-2026-jam-1900-wib-jorge-martin-bidik-kemenangan-ducati-kejar-aprilia</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/QWRdNYbbfG5s6YXga5PrKpnEFfo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sprint-Race-MotoGP-Amerika-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Misteri Kematian Sutrimo: Disebut Punya Riwayat Diabetes Akut, Bisakah Sebabkan Kematian Mendadak?</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:24:31 +0700</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>Dokter Novianto Adi beri penjelasan apakah penyakit diabetes yang diderita Eks Karumga Febrie Adriansyah, Sutrimo bisa sebabkan kematian mendadak.</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866051/misteri-kematian-sutrimo-disebut-punya-riwayat-diabetes-akut-bisakah-sebabkan-kematian-mendadak</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/TYMpag4Kl-8VDabiqGKaGE9RBw8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Olah-TKP-Kasus-Tewasnya-Karumga-Sutrimo_1.jpg</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Usaha Ultra Mikro Perempuan Perkuat Ekonomi Masyarakat Pesisir</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:39:51 +0700</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Penguatan ekonomi masyarakat pesisir tidak cukup hanya dengan membuka akses permodalan. Pendampingan usaha, peningkatan nilai tambah produk, penguatan kapasitas perempuan, hingga akses pendidikan turut menentukan kemampuan keluarga...</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tji049416/usaha-ultra-mikro-perempuan-perkuat-ekonomi-masyarakat-pesisir</t>
+        </is>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260809173843-885.png</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Kasus 996 Senjata di Sekolah, Kuasa Hukum Bantah Ada Ekskul Menembak</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:08:54 +0700</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>Kuasa Hukum Yayasan Harapan Ibu Pondok Pinang membantah adanya konflik kepentingan antara para pendiri yayasan.</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265719/kasus-996-senjata-di-sekolah-kuasa-hukum-bantah-ada-ekskul-menembak</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/YAVOExu6fnI0Yew1ROoX836YmpQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319668/original/013460500_1786264819-71184.jpg</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Pendiri Yayasan Ngaku Sedih Ada Temuan Senjata Api di Sekolah</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:04:43 +0700</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Yan Sofyan Syafe'i, salah satu pendiri Yayasan Harapan Ibu Pondok Pinang Jaksel mengaku sedih ada temuan ratusan senjata api di sekolah.</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265713/pendiri-yayasan-ngaku-sedih-ada-temuan-senjata-api-di-sekolah</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/NehaaytFpLPd5KPabLwDKmp3Fps=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319721/original/068224600_1786273459-71222.jpg</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Ramaikan di GIIAS 2026, Kia PV5 Usung Konsep Satu Platform Banyak Fungsi</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:23:12 +0700</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>PT Kia Sales Indonesia kembali memamerkan Kia PV5 Concept ke Indonesia, kali ini pada ajang Gaikindo Indonesia International Auto Show (GIIAS) 2026.</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>https://otomotif.kompas.com/read/2026/08/09/182100515/ramaikan-di-giias-2026-kia-pv5-usung-konsep-satu-platform-banyak-fungsi</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/5Nc5xjQBCDH69HrzU7vBXkWySEw=/341x318:4000x2757/1200x675/filters:watermark(data/photo/2026/01/30/697c81750a668.png,0,-0,1)/data/photo/2026/08/09/6a7839c79f9ca.jpg</t>
+        </is>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Penjualan Mobil Juli 2026 Naik, Gaikindo Masih Optimistis</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:23:12 +0700</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>Penjualan mobil nasional Juli 2026 mencapai 81.115 unit, naik dari bulan sebelumnya. Gaikindo berharap tren positif berlanjut hingga akhir tahun.</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>https://otomotif.kompas.com/read/2026/08/09/174100015/penjualan-mobil-juli-2026-naik-gaikindo-masih-optimistis</t>
+        </is>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/ryJCwNn9dBXWtJ5h-c1pxn1-QWA=/0x106:1554x1141/1200x675/filters:watermark(data/photo/2026/01/30/697c81750a668.png,0,-0,1)/data/photo/2026/08/09/6a78512b9a206.jpeg</t>
+        </is>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Alasan Konsumen Pilih Wuling Aira EV, Beli Tunai dan Tak Mau Inden</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:23:12 +0700</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Tak mau menunggu inden, konsumen membeli Wuling Aira EV secara tunai di GIIAS 2026 dan bisa langsung dibawa pulang.</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>https://otomotif.kompas.com/read/2026/08/09/170100515/alasan-konsumen-pilih-wuling-aira-ev-beli-tunai-dan-tak-mau-inden</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/1OhI1QLiTYAqeSF9c-BuJTmrCY8=/0x85:1280x938/1200x675/filters:watermark(data/photo/2026/01/30/697c81750a668.png,0,-0,1)/data/photo/2026/08/09/6a7832d737c41.jpeg</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I616"/>
+  <autoFilter ref="A1:I662"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 12:27 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$662</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$705</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I662"/>
+  <dimension ref="A1:I705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -31552,8 +31552,2029 @@
         </is>
       </c>
     </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Kolaborasi PLN dan Rappo berdayakan warga lewat furnitur daur ulang</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:22:25 +0700</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>PT PLN Unit Induk Distribusi Sulawesi Selatan, Sulawesi Tenggara dan Sulawesi Barat (UID Sulselrabar) berkolaborasi ...</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686745/kolaborasi-pln-dan-rappo-berdayakan-warga-lewat-furnitur-daur-ulang</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/20260809_151255.jpg</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Jesus Vivas: 11.000 imigran Maroko masih bertahan di Ceuta</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:19:33 +0700</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>Wali Kota Ceuta Juan Jesus Vivas mengatakan jumlah imigran asal Maroko yang masih berada di wilayah ...</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686744/jesus-vivas-11000-imigran-maroko-masih-bertahan-di-ceuta</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/AA-20260731-42116094-42116080-MIGRANTS_ARRIVE_ON_SHORE_AFTER_ATTEMPTING_SEA_CROSSING_TO_CEUTA_FROM_MOROCCO.jpg</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Tak dapat undangan upacara HUT RI? Pemerintah siapkan Pesta Rakyat</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:17:21 +0700</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>Kementerian Sekretariat Negara menutup pendaftaran undangan Upacara Peringatan HUT Ke-81 Kemerdekaan Republik Indonesia ...</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686743/tak-dapat-undangan-upacara-hut-ri-pemerintah-siapkan-pesta-rakyat</t>
+        </is>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000402640.jpg</t>
+        </is>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Van Gastel soroti fisik pemain PSIM setelah uji coba lawan UAD FC</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:14:02 +0700</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>Pelatih kepala PSIM Yogyakarta Jean-Paul van Gastel menyoroti fisik pemain-pemainnya setelah  melawan UAD FC ...</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686740/van-gastel-soroti-fisik-pemain-psim-setelah-uji-coba-lawan-uad-fc</t>
+        </is>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/22/Gastel.jpg</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Pemprov Sulsel siapkan 300 unit  pompa air hadapi dampak El Nino</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:09:35 +0700</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi Sulawesi Selatan menyiapkan 300 unit pompa air sebagai langkah mitigasi menghadapi musim kemarau ...</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686739/pemprov-sulsel-siapkan-300-unit-pompa-air-hadapi-dampak-el-nino</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001583660.jpg</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Marvin Loria pemain terakhir yang didatangkan PSIM musim ini</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:09:06 +0700</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>PSIM Yogyakarta menyebut Marvin Loria menjadi pemain anyar terakhir yang didatangkan untuk menyambut musim ...</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686735/marvin-loria-pemain-terakhir-yang-didatangkan-psim-musim-ini</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_7486.jpeg</t>
+        </is>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Pramono siapkan JIS jadi kandang utama Persija Jakarta</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:06:11 +0700</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung menegaskan komitmen Pemerintah Provinsi DKI Jakarta untuk menjadikan Jakarta ...</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686732/pramono-siapkan-jis-jadi-kandang-utama-persija-jakarta</t>
+        </is>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_183036571.jpg</t>
+        </is>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>STKIP Pasundan juara Liga Universitas regional Bandung</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:04:59 +0700</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>STKIP Pasundan keluar sebagai juara regional Bandung kompetisi sepak bola Liga Universitas Coca-Cola 2026 setelah ...</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686728/stkip-pasundan-juara-liga-universitas-regional-bandung</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/85b63009-573e-4ced-8163-0c5e56c689de.jpeg</t>
+        </is>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>PT TPS catat arus peti kemas pada Juli tumbuh 11,79 persen</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:01:09 +0700</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>PT Terminal Petikemas Surabaya (TPS) mencatat pertumbuhan arus peti kemas sebesar 11,79 persen pada Juli 2026 ...</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686725/pt-tps-catat-arus-peti-kemas-pada-juli-tumbuh-1179-persen</t>
+        </is>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Kegiatan-bongkar-muat-di-CY-TPS.jpg</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Jaecoo J7 di Australia ditarik karena masalah kabel kelistrikan</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:58:13 +0700</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>Sebanyak 171 unit SUV keluarga Jaecoo J7 tahun produksi 2025 hingga 2026 di Australia ditarik kembali (recall) karena ...</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5686721/jaecoo-j7-di-australia-ditarik-karena-masalah-kabel-kelistrikan</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/02/15/IMG_6009.jpg</t>
+        </is>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Anggota DPR dorong Kota Magelang jadi contoh toleransi beragama</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:48:00 +0700</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>Anggota Komisi VIII DPR RI Wibowo Prasetyo menilai Kota Magelang memiliki potensi besar untuk menjadi contoh dalam ...</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686717/anggota-dpr-dorong-kota-magelang-jadi-contoh-toleransi-beragama</t>
+        </is>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/kentongan-wali.jpg</t>
+        </is>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Ribuan warga Makassar serbu pangkalan TNI AL demi naik kapal perang</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:45:14 +0700</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>Ribuan warga Makassar dan sekitarnya memadati Markas Komando Daerah Angkatan Laut (Kodaeral) VI untuk melihat dan ...</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686713/ribuan-warga-makassar-serbu-pangkalan-tni-al-demi-naik-kapal-perang</t>
+        </is>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/ImgResizer_Crop_IMG-20260809-WA0007.jpg</t>
+        </is>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Honda Super-One mobil listrik mungil nan lincah</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>Honda meluncurkan mobil listrik Super-ONE untuk pasar Indonesia dengan jumlah terbatas. Mobil mungil ...</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/infografik/5686711/honda-super-one-mobil-listrik-mungil-nan-lincah</t>
+        </is>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/20260809-Honda-Super-One-mobil-listrik-mungil-nan-lincah.jpg</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>LKBN Antara komitmen perkuat citra ikon wisata KEK Mandalika</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:42:08 +0700</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>ANTARA - Lembaga Kantor Berita Nasional (LKBN) ANTARA berkomitmen memperkuat citra Kawasan Ekonomi Khusus (KEK) ...</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686709/lkbn-antara-komitmen-perkuat-citra-ikon-wisata-kek-mandalika</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/LKBN-ANTARA-KOMITMEN-PERKUAT.jpg</t>
+        </is>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Candaan Bill Maher soal Ariana Grande tuai reaksi penonton</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:36:14 +0700</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Komedian Bill Maher melontarkan lelucon mengenai berat badan penyanyi Ariana Grande dalam program "Real ...</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686708/candaan-bill-maher-soal-ariana-grande-tuai-reaksi-penonton</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Untitled-design-62.jpg</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Topan Dolphin mendekat, China aktifkan peringatan merah tertinggi di Shanghai</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:33:35 +0700</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>Warga memegang erat payung yang terbalik akibat tiupan angin saat hujan di Huangpu, Shanghai, China, Minggu (9/8/2026). ...</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5686705/topan-dolphin-mendekat-china-aktifkan-peringatan-merah-tertinggi-di-shanghai</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Peringatan-Merah-Topan-Dolphin-090826-WX-1.jpg</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Lomba ketangkasan lansia sambut hari Kemerdekaan</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:33:01 +0700</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>ANTARA - Sekolah lanjut usia (lansia) Kalimasada di Kalurahan Donoharjo, Sleman, D.I. Yogyakarta menggelar lomba ...</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686693/lomba-ketangkasan-lansia-sambut-hari-kemerdekaan</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/LOMBA-KETANGKASAN-LANSIA.jpg</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>TNGGP catat 150 petugas gabungan masih berupaya padamkan api</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:27:24 +0700</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>Balai Besar Taman Nasional Gunung Gede Pangrango mencatat sekitar 150 petugas gabungan dan relawan masih berupaya ...</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686701/tnggp-catat-150-petugas-gabungan-masih-berupaya-padamkan-api</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/api-gede.jpg</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Melihat benteng bersejarah di selatan Pulau Bangka</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:27:06 +0700</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>ANTARA - Di ujung paling selatan Pulau Bangka, Kabupaten Bangka Selatan, Provinsi Kepulauan Bangka Belitung, berdiri ...</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686685/melihat-benteng-bersejarah-di-selatan-pulau-bangka</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/MELIHAT-BENTENG-BERSEJARAH-DI-SELATAN-PULAU-BANGKA.jpg</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>KAI Daop 6 tangani 1.075 barang tertinggal senilai Rp1,16 miliar</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:26:41 +0700</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) Daerah Operasi (Daop) 6 Yogyakarta telah menangani 1.075 barang milik penumpang yang ...</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686697/kai-daop-6-tangani-1075-barang-tertinggal-senilai-rp116-miliar</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000044649.jpg</t>
+        </is>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Menhut serahkan penyelidikan penyebab karhutla di Bromo kepada aparat</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:23:46 +0700</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Menteri Kehutanan (Menhut) Raja Juli Antoni mempercayakan proses penyelidikan penyebab kebakaran hutan dan lahan ...</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686696/menhut-serahkan-penyelidikan-penyebab-karhutla-di-bromo-kepada-aparat</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001410029.jpg</t>
+        </is>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Bea Cukai Semarang Gagalkan Peredaran 3,2 Juta Batang Rokok Ilegal</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:14:24 +0700</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Farih Maulana Sidik</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Bea dan Cukai Semarang gagalkan penyelundupan 3,28 juta batang rokok ilegal senilai Rp 4,87 miliar. Dua sopir ditangkap untuk penyelidikan lebih lanjut.</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611217/bea-cukai-semarang-gagalkan-peredaran-3-2-juta-batang-rokok-ilegal</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2016/08/30/9950fe5a-950e-41f3-9b92-db2c7d0dbb2e_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Polisi Masih Cari Kaki Korban Mutilasi Saepul: Jika Warga Tahu Harap Lapor</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:09:05 +0700</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Polisi mencari potongan kaki korban mutilasi di Kali Licin, Depok. Saepul, pelaku, ditangkap setelah membunuh dan memutilasi pria K.</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611211/polisi-masih-cari-kaki-korban-mutilasi-saepul-jika-warga-tahu-harap-lapor</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/anjing-pelacak-k9-dasa-dikerahkan-mencari-kaki-pria-berinisial-k-51-korban-mutilasi-di-depok-devidetikcom-1786088609041_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Pramono: TransJakarta Kelola Transportasi ke Pulau Seribu Tahun Depan</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:57:50 +0700</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung rencanakan pengalihan pengelolaan transportasi Kepulauan Seribu ke TransJakarta untuk kemudahan akses warga.</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611203/pramono-transjakarta-kelola-transportasi-ke-pulau-seribu-tahun-depan</t>
+        </is>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/dari-call-center-hingga-rute-ancol-pemprov-dki-tambah-layanan-transportasi-publik-1786248603240_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Harga Cabai Rawit Kian Pedas, Nyaris Rp 60 Ribu/Kg</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:00:15 +0700</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>Komoditas pangan yang mengalami kenaikan harga di antaranya beras, cabai, daging sapi dan daging ayam.</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8611182/harga-cabai-rawit-kian-pedas-nyaris-rp-60-ribu-kg</t>
+        </is>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/02/20/cabai-rawit-merah-mengalir-ke-pasar-induk-kramat-jati-1771573533198_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Barang-barang Ini Banyak Dibeli Masyarakat Lewat Toko Online</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:57:53 +0700</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Sylke Febrina Laucereno</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>Belanja online di Indonesia semakin populer, dengan banyak produk ringan di bawah 300 gram.</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8611165/barang-barang-ini-banyak-dibeli-masyarakat-lewat-toko-online</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/02/24/ilustrasi-belanja-online-1771906901925_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Memburu Keadilan Pemilu Substantif</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:21:48 +0700</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>The Jeblogs lewat “Bersandarlah” ingatkan jeda reflektif penting dalam perjuangan hukum pemilu, bukan tanda menyerah</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/tribunners/7866074/memburu-keadilan-pemilu-substantif</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/gWBANuKd6-xhyn9huInUQurUb3Y=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/FOTO-BENNY-SABDO-27-OKT.jpg</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Iran Tegaskan Tak Akan Buka Selat Hormuz, Minta AS Penuhi Syarat-Syarat Termasuk Kompensasi Perang</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:12:50 +0700</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>Iran tidak akan membuka Selat Hormuz sampai Amerika Serikat memenuhi syarat-syarat yang ditetapkan Teheran.</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866073/iran-tegaskan-tak-akan-buka-selat-hormuz-minta-as-penuhi-syarat-syarat-termasuk-kompensasi-perang</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/wAvXfO-jSsPZyuSmmQpiICiEJbE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Peta-Selat-Hormuz-Iran-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Tersebarnya Foto Sutrimo dengan Mulut Berbusa Picu Spekulasi Keracunan, Ahli Forensik Beri Tanggapan</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:04:17 +0700</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>Tanggapi kondisi mulut berbusa Eks Karumga Febrie Adriansyah, Sutrimo, dr Novianto memberikan pandangannya dari sudut pandang kedokteran forensik.</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866072/tersebarnya-foto-sutrimo-dengan-mulut-berbusa-picu-spekulasi-keracunan-ahli-forensik-beri-tanggapan</t>
+        </is>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/CwMUyzUp6Ng_C-qMpDr5muWU_Ls=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/klinik-Mordent-Esthetic-Clinic-TKP-Sutrimo-Tewas.jpg</t>
+        </is>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Pascatemuan Senjata di Sekolah, Yayasan Minta Perlindungan KPAI dan DPR, PJJ Berlaku Sepekan</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:57:32 +0700</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>YHI-PP minta perlindungan KPAI dan DPR usai temuan 995 senjata di sekolah Jaksel, PJJ diberlakukan sepekan demi keamanan.</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866071/pascatemuan-senjata-di-sekolah-yayasan-minta-perlindungan-kpai-dan-dpr-pjj-berlaku-sepekan</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/enu60eSCVJ1ALLFEmi5pFfeMTg4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/996-senjata-di-sebuah-sekolah-kawasan-Pondok-Pinang-32010.jpg</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>5 Teks Doa Malam Tirakatan 17 Agustus 2026 yang Penuh Harapan</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:57:11 +0700</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>Malam tirakatan adalah tradisi berkumpul untuk menyambut 17 Agustus 2026, biasanya diisi dengan doa bersama, renungan, dan ungkapan syukur.</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866070/5-teks-doa-malam-tirakatan-17-agustus-2026-yang-penuh-harapan</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/30PrYRKYXHE-Y9KEpnuKDG_mhQw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pawai-dan-lomba-17-agustusan-di-kabupaten-bandung_20220817_202718.jpg</t>
+        </is>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu Go Go Juice - Sabrina Carpenter: How's You's Been? What's Up?</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:57:11 +0700</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>Inilah lirik lagu dan terjemahan Go Go Juice yang dipopulerkan oleh penyanyi Sabrina Carpenter. Lagu ini dirilis pada 29 Agustus 2025.</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7866069/terjemahan-lirik-lagu-go-go-juice-sabrina-carpenter-hows-yous-been-whats-up</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zLN77GXG_MWcQ27NDqNvGgp-QJs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-musik-ilustrasi-lirik-ilustrasi-terjemahan-lirik-lagu.jpg</t>
+        </is>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Pengertian tentang Hepatitis B, Lengkap dengan Gejala dan Cara Mencegahnya</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:52:43 +0700</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>Hepatitis B merupakan penyakit yang disebabkan oleh virus dan menyerang organ hati, simak gejala hingga cara mencegahnya berikut ini.</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866068/pengertian-tentang-hepatitis-b-lengkap-dengan-gejala-dan-cara-mencegahnya</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/yvYBk7Mj-zTlRR51mwpwa8LWo7E=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Cek-kesehatan-gratis-di-Colomadu-Tohudan.jpg</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Klasemen Akhir SEA V Cup 2026 Putri Leg 2: Thailand Sempurna, Vietnam Juru Kunci, Indonesia Ketiga</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:49:22 +0700</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>Thailand menjadi juara SEA V Cup 2026 secara keseluruhan. Filipina mencatat sejarah dengan finis sebagai runner-up di leg kedua.</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866067/klasemen-akhir-sea-v-cup-2026-putri-leg-2-thailand-sempurna-vietnam-juru-kunci-indonesia-ketiga</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/LAwHs6XeRlKtxkdALLGPxJSPCrQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pemain-Timnas-Voli-Putri-Indonesia-berselebrasi-setelah-mencetak.jpg</t>
+        </is>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Terkait Pernyataan Kapolri, Boni Hargens Sebut Bukti Perkuat Pemerintah Prabowo-Gibran</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:37:39 +0700</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>Analis politik nilai pernyataan Kapolricerminkan komitmen terhadap dua hal fundamental yang krusial bagi stabilitas Indonesia</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866066/terkait-pernyataan-kapolri-boni-hargens-sebut-bukti-perkuat-pemerintah-prabowo-gibran</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tscjQfqgmuZy04dhWQ4vPfreYx0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Analis-Politik-dan-Hukum-Boni-Hargens-nihhhh.jpg</t>
+        </is>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Keisya Levronka Ungkap Alasan Terima Tawaran Main Film 'Dan Bandung', Singgung Karya Pidi Baiq</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:32:49 +0700</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>Artis Keisya Levronka mengungkap alasan terima tawaran bermain di film Dan Bandung. Ia mengaku menikmati karya-karya Pidi Baiq.</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866065/keisya-levronka-ungkap-alasan-terima-tawaran-main-film-dan-bandung-singgung-karya-pidi-baiq</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/UHZ9-t3bj-vfurIaaRIbrZpYIRY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Keisya-Levronka-1-29072025.jpg</t>
+        </is>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Aldi Taher Bersyukur Rezekinya Kini Lancar, Keuntungan Bisnis Dipakai untuk Obati Sang Ibu</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:29:53 +0700</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>Aldi Taher tengah menikmati kemudahan rezeki dari berbagai aktivitasnya, mulai dari pekerjaan di dunia hiburan hingga bisnis kuliner.</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866064/aldi-taher-bersyukur-rezekinya-kini-lancar-keuntungan-bisnis-dipakai-untuk-obati-sang-ibu</t>
+        </is>
+      </c>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/qw7Aqz6M7NjSWq8i2Vs2PTdk0r4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/aldi-taher-batiks.jpg</t>
+        </is>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Houthi Yaman Klaim Serang Kilang Minyak Aramco Arab Saudi, Pelabuhan di Laut Merah Juga Jadi Target</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:23:07 +0700</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>Juru bicara militer Houthi, Yahya Saree, mengatakan mereka menargetkan kilang Aramco di kota Jazan dengan drone.</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866063/houthi-yaman-klaim-serang-kilang-minyak-aramco-arab-saudi-pelabuhan-di-laut-merah-juga-jadi-target</t>
+        </is>
+      </c>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/JzTnWUfEK8Wa8q8CYPM37Kiggnk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Helikopter-Saudi-Aramco-jatuh.jpg</t>
+        </is>
+      </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Kejagung Pastikan Penyidikan Kasus Korupsi MBG Berjalan, Total 80 Saksi Telah Diperiksa</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:21:21 +0700</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>Kejagung memastikan bahwa penyidikan kasus korupsi tata kelola program makan bergizi gratis (MBG) tetap berjalan.</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G701" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866062/kejagung-pastikan-penyidikan-kasus-korupsi-mbg-berjalan-total-80-saksi-telah-diperiksa</t>
+        </is>
+      </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hzeNF5ybN0y8HQGmZckBriAu-Hg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kejagung-RI-Anang-Supriatna-saat-dite.jpg</t>
+        </is>
+      </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>YLBHI Desak Polisi Setop Proses Pidana 2 Warga Terkait Unggahan Soal Pidato Presiden</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:09:24 +0700</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>YLBHI mendesak Polda Jawa Barat menghentikan proses pidana terhadap dua warga Cimahi, AYP dan AF.</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866061/ylbhi-desak-polisi-setop-proses-pidana-2-warga-terkait-unggahan-soal-pidato-presiden</t>
+        </is>
+      </c>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hJdfjlJcGTo0MawecnpbkvHPrxc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Foto-Ketua-Umum-Yayasan-Lembaga-Bantuan-Hukum-Indonesia-YLBHI-Muhammad-Isnur.jpg</t>
+        </is>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>995 Senjata Ditemukan di Sekolah, Komnas Anak Akan Datangi Sekolah Harapan Ibu</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:27:15 +0700</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>Komnas PA DKI Jakarta akan kunjungi Sekolah Harapan Ibu menyusul temuan 995 senjata, narkoba, &amp; CD porno. Fokus: kondisi psikologis murid &amp; kelancaran belajar.</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/09/19234141/995-senjata-ditemukan-di-sekolah-komnas-anak-akan-datangi-sekolah-harapan</t>
+        </is>
+      </c>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/UPul14Yixs49yFZccXz1gxdQn1k=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/09/6a7858b5824a0.jpg</t>
+        </is>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Pemadaman Kebakaran Bromo Disebut Tidak Bisa Gunakan Mofifikasi Cuaca</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:27:15 +0700</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>Karhutla di TNBTS tak kunjung padam. Modifikasi cuaca mustahil 10 hari ke depan, kata Menhut Raja Juli Antoni.</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/08/09/183112978/pemadaman-kebakaran-bromo-disebut-tidak-bisa-gunakan-mofifikasi-cuaca</t>
+        </is>
+      </c>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/9GryLNiz-EzimcmyZYzCqKpskl8=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/09/6a785a29286d0.jpg</t>
+        </is>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Nongkrong Berujung Maut, Pria di Bandar Lampung Tewas Ditusuk Teman</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:27:15 +0700</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>Seorang pria tewas ditusuk di dada setelah perkelahian yang diduga dipicu minuman keras di Bandar Lampung.</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/09/180203878/nongkrong-berujung-maut-pria-di-bandar-lampung-tewas-ditusuk-teman</t>
+        </is>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/T5-FnLqHWPZrTpsT5oqS9uwtwto=/0x0:360x240/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/05/19/6a0c46a8cea0f.webp</t>
+        </is>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I662"/>
+  <autoFilter ref="A1:I705"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 13:44 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$705</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$765</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I705"/>
+  <dimension ref="A1:I765"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -33573,8 +33573,2828 @@
         </is>
       </c>
     </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Gulkarmat padamkan kebakaran gudang sekolah di Penjaringan Jakut</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:38:56 +0700</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>Suku Dinas Penanggulangan Kebakaran dan Penyelamatan (Gulkarmat) Jakarta Utara mengerahkan 70 personel untuk memadamkan ...</t>
+        </is>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G706" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686825/gulkarmat-padamkan-kebakaran-gudang-sekolah-di-penjaringan-jakut</t>
+        </is>
+      </c>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_4686.jpeg</t>
+        </is>
+      </c>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Air Terjun Tancak jadi destinasi favorit pendaki pemula di Jember</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:33:47 +0700</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>ANTARA - Air Terjun Tancak di lereng selatan Pegunungan Hyang Argopuro, Kabupaten Jember, menjadi salah satu destinasi ...</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G707" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686772/air-terjun-tancak-jadi-destinasi-favorit-pendaki-pemula-di-jember</t>
+        </is>
+      </c>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AIR-TERJUN-TANCAK-JADI-DESTINASI-FAVORIT.jpg</t>
+        </is>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Ahmad Sahroni traktir warga Kebon Bawang Jakut dengan produk UMKM</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:32:42 +0700</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Komisi III DPR RI Ahmad Sahroni melalui Ahmad Sahroni Center (ASC) mentraktir warga di sepanjang Jalan ...</t>
+        </is>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686823/ahmad-sahroni-traktir-warga-kebon-bawang-jakut-dengan-produk-umkm</t>
+        </is>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/bf82958d-63c9-4be0-bd79-7009953b0608.jpeg</t>
+        </is>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>PTFI dorong kepedulian lingkungan lewat gotong royong desa di Gresik</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:32:07 +0700</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>PT Freeport Indonesia (PTFI) mendorong kepedulian masyarakat terhadap kebersihan dan kelestarian lingkungan melalui ...</t>
+        </is>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G709" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686821/ptfi-dorong-kepedulian-lingkungan-lewat-gotong-royong-desa-di-gresik</t>
+        </is>
+      </c>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-09-at-20.21.05.jpeg</t>
+        </is>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>390 orang terisolasi longsor di Nagano diselamatkan dengan jembatan</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:31:53 +0700</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>Kepolisian Prefektur Nagano, Jepang, mengatakan jembatan darurat telah didirikan untuk dilewati oleh sekitar 390 orang ...</t>
+        </is>
+      </c>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G710" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686819/390-orang-terisolasi-longsor-di-nagano-diselamatkan-dengan-jembatan</t>
+        </is>
+      </c>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/03/15/WhatsApp-Image-2023-03-15-at-19.25.01.jpeg</t>
+        </is>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Kebakaran Gunung Bromo meluas, 520 Hektare lahan terbakar</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:28:07 +0700</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>ANTARA - Kebakaran hutan di kawasan Taman Nasional Bromo Tengger Semeru terus meluas. Hingga Minggu (9/8), luas lahan ...</t>
+        </is>
+      </c>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G711" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686791/kebakaran-gunung-bromo-meluas-520-hektare-lahan-terbakar</t>
+        </is>
+      </c>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KEBAKARAN-GUNUNG-BROMO-MELUAS-520-HEKTARE-LAHAN-TERBAKAR.jpg</t>
+        </is>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>MV Cape San Juan bawa alutsista Super Garuda Shield tiba di Lampung</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:27:33 +0700</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>Pelabuhan Panjang di Lampung menjadi lokasi sandar MV Cape San Juan yang membawa sejumlah alat utama sistem senjata ...</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686816/mv-cape-san-juan-bawa-alutsista-super-garuda-shield-tiba-di-lampung</t>
+        </is>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG-20260809-WA0000.jpg</t>
+        </is>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Menilik kebangkitan industri China dari perspektif yang lebih luas</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:25:13 +0700</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>Seiring China terus meningkatkan basis manufaktur dan memperluas produksi di berbagai sektor, mulai dari kendaraan ...</t>
+        </is>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686813/menilik-kebangkitan-industri-china-dari-perspektif-yang-lebih-luas</t>
+        </is>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/CjkinzN000009_20260809_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>KAI Layani 10 Juta Pelanggan Commuter Line Area VIII Surabaya hingga Juli 2026</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:22:44 +0700</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>Memasuki akhir pekan, kereta api lokal menjadi salah satu pilihan masyarakat Jawa Timur untuk bepergian antarkota, ...</t>
+        </is>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686809/kai-layani-10-juta-pelanggan-commuter-line-area-viii-surabaya-hingga-juli-2026</t>
+        </is>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/KAI-Line-Area-VIII-Surabaya.jpg</t>
+        </is>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Mengapa dunia kini memandang China secara lebih positif?</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:20:33 +0700</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>Tiga tahun lalu, hasil jajak pendapat di Kanada menunjukkan kesenjangan tingkat persepsi positif yang sangat lebar ...</t>
+        </is>
+      </c>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G715" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686807/mengapa-dunia-kini-memandang-china-secara-lebih-positif</t>
+        </is>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/CjkinzN000012_20260807_CBMFN0A002.jpg</t>
+        </is>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya juarai E-Sports Kapolri Cup 2026</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:20:18 +0700</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya menjuarai Kejuaraan Mobile Legends E-Sports Kapolri Cup 2026 setelah mengalahkan Polda Sumatera Utara ...</t>
+        </is>
+      </c>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686803/polda-metro-jaya-juarai-e-sports-kapolri-cup-2026</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000131522.jpg</t>
+        </is>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Pemerintah terus perkuat KDMP gerakkan ekonomi desa</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:18:55 +0700</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>Pemerintah terus memperkuat Koperasi Merah Putih sebagai penggerak ekonomi desa dan ditargetkan pada 16 Agustus 2026 ...</t>
+        </is>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G717" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686800/pemerintah-terus-perkuat-kdmp-gerakkan-ekonomi-desa</t>
+        </is>
+      </c>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/IMG_20260801_172518.jpg</t>
+        </is>
+      </c>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Seribu porsi nasi goreng rendang Kota Padang bantu korban banjir</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:18:32 +0700</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kota Padang Provinsi Sumatera Barat menggelar kegiatan memasak nasi goreng rendang sebanyak 1.000 ...</t>
+        </is>
+      </c>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686784/seribu-porsi-nasi-goreng-rendang-kota-padang-bantu-korban-banjir</t>
+        </is>
+      </c>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SERIBU-PORSI-NASI-GORENG-RENDANG-KOTA-PADANG-BANTU-KORBAN-BANJIR.jpg</t>
+        </is>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>Pakistan sebut Perjanjian Mekkah murni terkait pertahanan</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:18:02 +0700</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>Menteri Luar Negeri Pakistan Ishaq Dar mengatakan bahwa perjanjian pertahanan trilateral Mekkah yang ...</t>
+        </is>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G719" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686799/pakistan-sebut-perjanjian-mekkah-murni-terkait-pertahanan</t>
+        </is>
+      </c>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Bendera-Pakistan-Saudi-Turkiye.jpg</t>
+        </is>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Data SIC: Ekonomi China tunjukkan peningkatan stabil pada Juli</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:17:14 +0700</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>Data frekuensi tinggi dari Pusat Informasi Negara (State Information Center/SIC) China pada Sabtu (8/8) ...</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686795/data-sic-ekonomi-china-tunjukkan-peningkatan-stabil-pada-juli</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2021/12/19/Xinhua-News-Agency.jpg</t>
+        </is>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Unjuk kekuatan tempur trimatra, siap jaga kedaulatan negara</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:17:01 +0700</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>ANTARA - Tentara Nasional Indonesia menggelar latihan operasi TNI terintegrasi 2026 bertajuk "Perisai Trisula ...</t>
+        </is>
+      </c>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686373/unjuk-kekuatan-tempur-trimatra-siap-jaga-kedaulatan-negara</t>
+        </is>
+      </c>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PERANTARA-9agustus_1.jpg</t>
+        </is>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Cara agar latihan kekuatan tidak membosankan dan tetap konsisten</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:15:02 +0700</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>Latihan kekuatan atau strength training penting untuk membantu menjaga kekuatan dan kemandirian tubuh seiring ...</t>
+        </is>
+      </c>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686793/cara-agar-latihan-kekuatan-tidak-membosankan-dan-tetap-konsisten</t>
+        </is>
+      </c>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/17/IMG_5595.jpg</t>
+        </is>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Kota Hefei padukan tren wisata baru dengan berbagai pasar tematik</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:12:04 +0700</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>Hefei di Provinsi Anhui, China timur, telah menyelenggarakan serangkaian pasar tematik dengan memanfaatkan sumber daya ...</t>
+        </is>
+      </c>
+      <c r="F723" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G723" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686788/kota-hefei-padukan-tren-wisata-baru-dengan-berbagai-pasar-tematik</t>
+        </is>
+      </c>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/CjkinzN000012_20260808_CBMFN0A002_2.v1.jpg</t>
+        </is>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Menhut ajak masyarakat bantu pemerintah cegah karhutla</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:10:29 +0700</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>Menteri Kehutanan (Menhut) Raja Juli Antoni mengajak masyarakat turut berpartisipasi membantu pemerintah mencegah ...</t>
+        </is>
+      </c>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686787/menhut-ajak-masyarakat-bantu-pemerintah-cegah-karhutla</t>
+        </is>
+      </c>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001410201.jpg</t>
+        </is>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>TNI AL perketat pengamanan seusai gagalkan penyelundupan ketamine</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:06:21 +0700</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>ANTARA - TNI Angkatan Laut memperketat pengamanan seusai mengagalkan upaya penyelundupan 65 karung ketamine seberat 1.3 ...</t>
+        </is>
+      </c>
+      <c r="F725" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686689/tni-al-perketat-pengamanan-seusai-gagalkan-penyelundupan-ketamine</t>
+        </is>
+      </c>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/TNI-AL-PERKETAT-PENGAMANAN-SEUSAI-GAGALKAN-PENYELUNDUPAN-KETAMINE_1.jpg</t>
+        </is>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Puluhan penyelam gelar upacara bendera di bawah laut Jayapura</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:04:16 +0700</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>ANTARA - Direktorat Polisi Air dan Udara Polda Papua bersama komunitas selam Jayapura menggelar upacara pengibaran ...</t>
+        </is>
+      </c>
+      <c r="F726" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686775/puluhan-penyelam-gelar-upacara-bendera-di-bawah-laut-jayapura</t>
+        </is>
+      </c>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PULUHAN-PENYELAM-GELAR-UPACARA-BENDERA.jpg</t>
+        </is>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Mitigasi banjir, BPJN Aceh bangun saluran beton tampung air</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:57:44 +0700</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>ANTARA - Balai Pelaksanaan Jalan Nasional (BPJN) Aceh membangun box culvert atau saluran beton penampungan air di ...</t>
+        </is>
+      </c>
+      <c r="F727" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686751/mitigasi-banjir-bpjn-aceh-bangun-saluran-beton-tampung-air</t>
+        </is>
+      </c>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/MITIGASI-BANJIR-BPJN-ACEH.jpg</t>
+        </is>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Dua pesawat nyaris tabrakan di Bandara Sydney, satu awak terluka</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:54:27 +0700</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>Seorang awak kabin terluka ketika pesawat Jetstar Airways dan Qatar Airways nyaris bertabrakan di landasan pacu Bandara ...</t>
+        </is>
+      </c>
+      <c r="F728" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686783/dua-pesawat-nyaris-tabrakan-di-bandara-sydney-satu-awak-terluka</t>
+        </is>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/CjkinzN000013_20260809_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Komisaris Pertamina Patra Niaga pastikan distribusi BBM di Kepri aman</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:54:09 +0700</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>Dewan Komisaris PT Pertamina Patra Niaga memastikan distribusi bahan bakar minyak (BBM) di wilayah Kepulauan Riau dalam ...</t>
+        </is>
+      </c>
+      <c r="F729" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686780/komisaris-pertamina-patraniaga-pastikan-distribusi-bbm-di-kepri-aman</t>
+        </is>
+      </c>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000406267.jpg</t>
+        </is>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Gajah sumatra ditemukan mati di perkebunan sawit</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:51:14 +0700</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>Satu individu gajah sumatra (elephas maximus sumatranus) ditemukan mati di areal perkebunan sawit di Kampung Kaloy, ...</t>
+        </is>
+      </c>
+      <c r="F730" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686776/gajah-sumatra-ditemukan-mati-di-perkebunan-sawit</t>
+        </is>
+      </c>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/gajah-mati-aceh-tamiang.jpg</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>British Columbia Kanada tetapkan status darurat karhutla</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:45:51 +0700</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi British Columbia di Kanada bagian barat menetapkan status darurat tingkat provinsi seiring ...</t>
+        </is>
+      </c>
+      <c r="F731" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G731" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686771/british-columbia-kanada-tetapkan-status-darurat-karhutla</t>
+        </is>
+      </c>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/CjkinzN000008_20260809_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>PLN dorong ekosistem kendaraan listrik lewat EVplore di Museum SBY-Ani</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:45:48 +0700</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>PT PLN (Persero) mendorong pertumbuhan ekosistem kendaraan listrik di sektor pariwisata dengan menghadirkan Program ...</t>
+        </is>
+      </c>
+      <c r="F732" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686767/pln-dorong-ekosistem-kendaraan-listrik-lewat-evplore-di-museum-sby-ani</t>
+        </is>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-07-at-07.43.51.jpeg</t>
+        </is>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>North West miliki banyak tindik di tangan, dokter ingatkan risikonya</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:41:04 +0700</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>Dokter kulit mengingatkan risiko kesehatan yang dapat muncul akibat tindik pada tangan, setelah North West, putri ...</t>
+        </is>
+      </c>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686763/north-west-miliki-banyak-tindik-di-tangan-dokter-ingatkan-risikonya</t>
+        </is>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/Untitled-design-71.jpg</t>
+        </is>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Injourney perkuat standar layanan berkualitas desa wisata di Lombok</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:39:45 +0700</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>InJourney Tourism Development Corporation (ITDC) melaksanakan pelatihan bagi warga desa wisata di Lombok Tengah, Nusa ...</t>
+        </is>
+      </c>
+      <c r="F734" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686759/injourney-perkuat-standar-layanan-berkualitas-desa-wisata-di-lombok</t>
+        </is>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1005753478.jpg</t>
+        </is>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>TNBTS catat area terdampak kebakaran di Bromo mencapai 520 hektare</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:38:07 +0700</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>Balai Besar Taman Nasional Bromo Tengger Semeru (TNBTS) mencatat luas area di kawasan Gunung Bromo yang terdampak ...</t>
+        </is>
+      </c>
+      <c r="F735" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686755/tnbts-catat-area-terdampak-kebakaran-di-bromo-mencapai-520-hektare</t>
+        </is>
+      </c>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001410105.jpg</t>
+        </is>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Mario Suryo Aji finis ke-22 di Moto2 GP Inggris 2026</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:37:36 +0700</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>Pembalap Indonesia Mario Suryo Aji finis di posisi ke-22 dengan  dengan selisih 21,323 detik dari Filip Salac yang ...</t>
+        </is>
+      </c>
+      <c r="F736" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686752/mario-suryo-aji-finis-ke-22-di-moto2-gp-inggris-2026</t>
+        </is>
+      </c>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/21/Latihan-pembalap-nasional-Moto2-dan-Moto3-di-Mandalika-210726-AS-8.jpg</t>
+        </is>
+      </c>
+      <c r="I736" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Megawati hadiri peluncuran buku otobiografi Erros Djarot</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:32:06 +0700</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>Presiden Kelima Republik Indonesia sekaligus Ketua Umum DPP PDI Perjuangan (PDIP), Megawati Soekarnoputri menghadiri ...</t>
+        </is>
+      </c>
+      <c r="F737" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686748/megawati-hadiri-peluncuran-buku-otobiografi-erros-djarot</t>
+        </is>
+      </c>
+      <c r="H737" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000582806.jpg</t>
+        </is>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>SGN sebut upaya akselerasi hasilkan rendemen 8 persen di pabrik gula</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:29:46 +0700</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>Direktur Utama PT Sinergi Gula Nusantara (SGN) Mahmudi menyebutkan upaya akselerasi di berbagai lini operasional telah ...</t>
+        </is>
+      </c>
+      <c r="F738" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686747/sgn-sebut-upaya-akselerasi-hasilkan-rendemen-8-persen-di-pabrik-gula</t>
+        </is>
+      </c>
+      <c r="H738" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-09-at-11.54.35.jpeg</t>
+        </is>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Gubernur DKI siapkan JIS sebagai kandang utama Persija Jakarta</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:06:11 +0700</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung menegaskan komitmen Pemerintah Provinsi DKI Jakarta untuk menjadikan Jakarta ...</t>
+        </is>
+      </c>
+      <c r="F739" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686732/gubernur-dki-siapkan-jis-sebagai-kandang-utama-persija-jakarta</t>
+        </is>
+      </c>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/07/27/peluncuran-tim-persija-jakarta-2584185.jpg</t>
+        </is>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Awal Mula Kebakaran Bromo yang Meluas hingga Kini Ditutup Total</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:15:40 +0700</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan di Gunung Bromo meluas hingga 520 hektare. Mengharuskan penutupan total di kawasan wisata.</t>
+        </is>
+      </c>
+      <c r="F740" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611274/awal-mula-kebakaran-bromo-yang-meluas-hingga-kini-ditutup-total</t>
+        </is>
+      </c>
+      <c r="H740" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kebakaran-bromo-makin-meluas-1786196152369_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I740" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>KPK Sita Dokumen dan Barang Elektronik dari 3 Lokasi di Bengkulu</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:42:52 +0700</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>KPK melakukan penggeledahan di Bengkulu terkait kasus dugaan korupsi Bupati Rejang Lebong, M Fikri Thobari, menyita dokumen dan barang elektronik.</t>
+        </is>
+      </c>
+      <c r="F741" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G741" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611242/kpk-sita-dokumen-dan-barang-elektronik-dari-3-lokasi-di-bengkulu</t>
+        </is>
+      </c>
+      <c r="H741" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/03/02/gedung-baru-kpk-2_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Sumenep Siapkan Lahan 7,1 Hektare untuk Sekolah Rakyat Permanen</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:41:07 +0700</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>Rahmat Khairurizqi</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>Pemkab Sumenep siapkan lahan 7,1 hektare untuk pembangunan Sekolah Rakyat permanen. Lokasi strategis di Desa Gunggung, mendukung akses pendidikan gratis.</t>
+        </is>
+      </c>
+      <c r="F742" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611241/sumenep-siapkan-lahan-7-1-hektare-untuk-sekolah-rakyat-permanen</t>
+        </is>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/sumenep-siapkan-lahan-71-hektare-untuk-sekolah-rakyat-permanen-1786279247370.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>KPK Geledah 15 Lokasi di Kasus Pemerasan Bupati Pemalang, Sita CCTV Hotel</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:27:58 +0700</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>KPK menggeledah 15 lokasi terkait kasus pemerasan Bupati Pemalang, Anom Widiyantoro. Barang bukti termasuk dokumen dan CCTV hotel disita.</t>
+        </is>
+      </c>
+      <c r="F743" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G743" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611233/kpk-geledah-15-lokasi-di-kasus-pemerasan-bupati-pemalang-sita-cctv-hotel</t>
+        </is>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/03/02/gedung-baru-kpk-8_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Momen Korban Tegur Jukir Liar di Tambora: Tadi Katanya Nggak Takut Polisi</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:19:27 +0700</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>Jukir liar di Jakarta Barat ditangkap setelah memaksa pemotor bayar parkir dan mengancam. Pelaku sempat menantang dan mengatakan tak takut polisi.</t>
+        </is>
+      </c>
+      <c r="F744" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611220/momen-korban-tegur-jukir-liar-di-tambora-tadi-katanya-nggak-takut-polisi</t>
+        </is>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/jukir-liar-memaksa-tarif-hingga-ajak-duel-pemotor-di-jalan-jembatan-lima-tambora-jakarta-barat-1786273386183.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Bandara Husein Sastranegara Layani Pesawat Jet Mulai 14 Agustus</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:53:12 +0700</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>Bandara Husein Sastranegara Bandung melayani penerbangan pesawat jet berbadan sedang (narrow body) mulai 14 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8611222/bandara-husein-sastranegara-layani-pesawat-jet-mulai-14-agustus</t>
+        </is>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/persiapan-bandara-husein-sastranegara-jelang-pengoperasian-1786077660151_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban IPS Kelas 7 Halaman 80 Kurikulum Merdeka Edisi Revisi: Aktivitas 3</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:24:06 +0700</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>Berikut ini kunci jawaban mata pelajaran IPS Kelas 7 Halaman 80 Kurikulum Merdeka terdapat tugas Aktivitas 3 pada Tema 2.</t>
+        </is>
+      </c>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7866090/kunci-jawaban-ips-kelas-7-halaman-80-kurikulum-merdeka-edisi-revisi-aktivitas-3</t>
+        </is>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/FBmkDqYmlx5UM0pD7_3NuyX3Hwc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SISWA-SMP-BELAJAR-10.jpg</t>
+        </is>
+      </c>
+      <c r="I746" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Debut Drama Rispo di Film Ketok Mejik Dilirik Pasar Internasional Meski Belum Tayang di Indonesia</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:20:29 +0700</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>Film Ketok Mejik debut Ananta Rispo, incar pasar India dengan genre drama komedi, tayang di bioskop Indonesia 13 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866089/debut-drama-rispo-di-film-ketok-mejik-dilirik-pasar-internasional-meski-belum-tayang-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/UWXZEYDONY5rpVvURw98YS0KuUI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Komika-Ananta-Rispo-ungkap-debut-akting-full-drama-tanpa-komedi.jpg</t>
+        </is>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Tingkatkan Layanan dan Keterbukaan, Pertamina Resmikan Integrasi Informasi Publik</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:17:56 +0700</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>Pertamina secara resmi meluncurkan Integrasi Layanan Informasi Publik sebagai semangat baru dalam menghadirkan layanan informasi yang informatif.</t>
+        </is>
+      </c>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pertamina/7866088/tingkatkan-layanan-dan-keterbukaan-pertamina-resmikan-integrasi-informasi-publik</t>
+        </is>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/157fS6seVPzrvj99uVfLglWu6ts=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/penguatan-layanan-publik-pertamina.jpg</t>
+        </is>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Fakta Baru Kasus Mutilasi di Depok, Korban Tampar Pipi Pelaku Tolak Berhubungan</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:16:48 +0700</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>Polisi mengungkap fakta baru di balik kasus pembunuhan disertai mutilasi yang terjadi di Depok, Jawa Barat. Pelaku cekcok karena korban menolak</t>
+        </is>
+      </c>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866087/fakta-baru-kasus-mutilasi-di-depok-korban-tampar-pipi-pelaku-tolak-berhubungan</t>
+        </is>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/c9LhuIk5HWXCwHJ66xPrhQQyYpo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pelaku-pembunuhan-disertai-mutilasi.jpg</t>
+        </is>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Raih LEPRID bersama 25 Ribu Warga, Wali Kota Agustina Dedikasikan Penghargaan bagi Warga Semarang</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:12:14 +0700</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>Sekitar 25 ribu peserta dari berbagai unsur masyarakat mengikuti Festival Tari Dug Dug Der Semarangan.</t>
+        </is>
+      </c>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866086/raih-leprid-bersama-25-ribu-warga-wali-kota-agustina-dedikasikan-penghargaan-bagi-warga-semarang</t>
+        </is>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/jlmkkvgTpJ8AJ-LsB6V261ocGtk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/tari-dug-dug-der-semarang.jpg</t>
+        </is>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban IPS Kelas 7 Halaman 74 Kurikulum Merdeka Edisi Revisi: Aktivitas 2</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:10:10 +0700</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>Berikut ini kunci jawaban mata pelajaran IPS Kelas 7 Halaman 74 Kurikulum Merdeka terdapat tugas Aktivitas 2 pada Tema 2.</t>
+        </is>
+      </c>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7866085/kunci-jawaban-ips-kelas-7-halaman-74-kurikulum-merdeka-edisi-revisi-aktivitas-2</t>
+        </is>
+      </c>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/I26CNXmBVbp-YSqMKF_baAJSXHw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SISWA-SMP-BELAJAR-11.jpg</t>
+        </is>
+      </c>
+      <c r="I751" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Mendag Budi Santoso Bawa Isu UMKM hingga Penguatan Rantai Nilai Global ke BRICS</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:04:53 +0700</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>Pentingnya sistem perdagangan berbasis aturan bagi penguatan UMKM kembali ditegaskan oleh Menteri Perdagangan RI Budi Santoso.</t>
+        </is>
+      </c>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866084/mendag-budi-santoso-bawa-isu-umkm-hingga-penguatan-rantai-nilai-global-ke-brics</t>
+        </is>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/l-TMKp3E6aQWxuJa2HGpil31Ce0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pertemuan-tingkat-menteri-brics.jpg</t>
+        </is>
+      </c>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Babak Baru Kasus Kematian Sutrimo: Keluarga Lapor Polisi, Kasus Akan Dilimpahkan ke Polda Metro Jaya</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:58:33 +0700</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>Keluarga Sutrimo melaporkan dugaan kematian tak wajar eks Karumga Febrie Adriansyah ke Polresta Banyumas. Selanjutnya akan dilimpahkan ke Polda Metro</t>
+        </is>
+      </c>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866083/babak-baru-kasus-kematian-sutrimo-keluarga-lapor-polisi-kasus-akan-dilimpahkan-ke-polda-metro-jaya</t>
+        </is>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/CawjQmYsx6SChqFOdefPkSh2M4U=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kematian-Sutrimo-Dilaporkan-ke-Polisi-oleh-Keluarga.jpg</t>
+        </is>
+      </c>
+      <c r="I753" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Hasil Akhir MotoGP Inggris 2026: Raul Fernandez Juara, Aprilia Sapu Bersih Podium</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:58:26 +0700</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>Raul Fernandez dominan memenangkan MotoGP Inggris 2026 sekaligus membawa Aprilia mencetak podium lockout bersama Martin dan Bezzecchi.</t>
+        </is>
+      </c>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866082/hasil-akhir-motogp-inggris-2026-raul-fernandez-juara-aprilia-sapu-bersih-podium</t>
+        </is>
+      </c>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/DjHHQVKqu4ElEJ25jxIRLTW3Re4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/raul-fernandez-motogp-jerman-2024.jpg</t>
+        </is>
+      </c>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban IPS Kelas 7 Halaman 71 Kurikulum Merdeka Edisi Revisi: Aktivitas 1</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:53:58 +0700</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>Berikut ini kunci jawaban mata pelajaran IPS Kelas 7 Halaman 71 Kurikulum Merdeka terdapat tugas Aktivitas 1 pada Tema 2.</t>
+        </is>
+      </c>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7866081/kunci-jawaban-ips-kelas-7-halaman-71-kurikulum-merdeka-edisi-revisi-aktivitas-1</t>
+        </is>
+      </c>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Nj0pDBHbMVc2FfzH_Vier8Az45c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SISWA-SMP-UJIAN-01.jpg</t>
+        </is>
+      </c>
+      <c r="I755" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Polres Banyumas Segera Limpahkan Laporan Keluarga Sutrimo ke Polda Metro Jaya</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:51:37 +0700</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>Kasus kematian Sutrimo memasuki babak baru setelah keluarganya membuat laporan ke Polres Banyumas, Jawa Tengah</t>
+        </is>
+      </c>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G756" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866080/polres-banyumas-segera-limpahkan-laporan-keluarga-sutrimo-ke-polda-metro-jaya</t>
+        </is>
+      </c>
+      <c r="H756" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/_zCzt3il7XRR0CQjdvD629edaIw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kombes-Pol-Petrus-Silalahi-32.jpg</t>
+        </is>
+      </c>
+      <c r="I756" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Netanyahu Tolak Rencana AS untuk Gaza, Bersumpah Tak Akan Tarik Pasukan sampai Hamas Lucuti Senjata</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:51:11 +0700</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>Benjamin Netanyahu bersumpah tidak akan ada penarikan militer sampai Hamas benar-benar dilucuti senjatanya.</t>
+        </is>
+      </c>
+      <c r="F757" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G757" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866079/netanyahu-tolak-rencana-as-untuk-gaza-bersumpah-tak-akan-tarik-pasukan-sampai-hamas-lucuti-senjata</t>
+        </is>
+      </c>
+      <c r="H757" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/S2Pm4Qx_SFfKrqW4fB4w1BHDuTE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Benjamin-Netanyahu-menyampaikan-pidato-di-Majelis-Umum-PBB.jpg</t>
+        </is>
+      </c>
+      <c r="I757" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Tren Bedah Estetik Meningkat, Dokter Ingatkan Selektif Memilih Fasilitas dan Tenaga Medis</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:48:19 +0700</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr">
+        <is>
+          <t>Minat bedah estetik di Indonesia meningkat, dokter ingatkan keselamatan pasien dan pemahaman risiko harus jadi prioritas utama.</t>
+        </is>
+      </c>
+      <c r="F758" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866078/tren-bedah-estetik-meningkat-dokter-ingatkan-selektif-memilih-fasilitas-dan-tenaga-medis</t>
+        </is>
+      </c>
+      <c r="H758" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/V4a8mH5UEx469LMXoFT2-9lKSVk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Semakin-meningkatnya-tren-bedah-estetik-membuat-dokter-mengingatkan-untuk-selektif.jpg</t>
+        </is>
+      </c>
+      <c r="I758" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Doa agar Dijauhkan dari Amal yang Sia-Sia dan Mohon Ibadah Diterima</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:43:05 +0700</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr">
+        <is>
+          <t>Muslim sebaiknya meningkatkan ibadahnya dan berdoa agar selama amalnya diterima Allah SWT. Berikut doa yang dapat dibaca.</t>
+        </is>
+      </c>
+      <c r="F759" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G759" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/lifestyle/7866077/doa-agar-dijauhkan-dari-amal-yang-sia-sia-dan-mohon-ibadah-diterima</t>
+        </is>
+      </c>
+      <c r="H759" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/n4YUMFOUJmVFifiHpDXxewIS1hw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/DOA-AGAR-AMAL-DITERIMA-45R443.jpg</t>
+        </is>
+      </c>
+      <c r="I759" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Layanan Aftersales Isuzu Fokus Maksimalkan Uptime Armada</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:41:01 +0700</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>Isuzu menerapkan strategi solusi proaktif agar potensi gangguan kendaraan dapat dicegah sejak dini.</t>
+        </is>
+      </c>
+      <c r="F760" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G760" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7866076/layanan-aftersales-isuzu-fokus-maksimalkan-uptime-armada</t>
+        </is>
+      </c>
+      <c r="H760" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/VUxWAmtujHKiSEhGSmxoP6XjkQI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/isuzu-aftersales-strategi.jpg</t>
+        </is>
+      </c>
+      <c r="I760" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Ranking FIVB usai SEA V League 2026 Leg 2: Filipina Salip Indonesia, Thailand Ajek, Vietnam Anjlok</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:24:23 +0700</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>Ranking FIVB Timnas Indonesia mengalami penurunan setelah menutup SEA V Cup 2026 leg kedua dengan kekalahan, Minggu (9/8/2026).</t>
+        </is>
+      </c>
+      <c r="F761" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G761" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866075/ranking-fivb-usai-sea-v-league-2026-leg-2-filipina-salip-indonesia-thailand-ajek-vietnam-anjlok</t>
+        </is>
+      </c>
+      <c r="H761" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/2E_jcZDmBcSfFTurSe_jufhP824=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ranking-FIV-Timnas-voli-putri-Indonesia-9-Agustus.jpg</t>
+        </is>
+      </c>
+      <c r="I761" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Ponsel Bekas Disusupi Spyware, Rp 445 Juta Uang Korban Ludes</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:00:01 +0700</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E762" t="inlineStr">
+        <is>
+          <t>Seorang manajer keuangan di Florida kehilangan US$25.000 akibat penipuan berkedok ancaman tugas juri.</t>
+        </is>
+      </c>
+      <c r="F762" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G762" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260809182901-37-757742/ponsel-bekas-disusupi-spyware-rp-445-juta-uang-korban-ludes</t>
+        </is>
+      </c>
+      <c r="H762" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2021/04/01/infografis-waspada-ini-tanda-tanda-hp-kamu-disadap-hacker_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I762" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>DPO Kasus Penembakan Kuala Kencana hingga Mile 69 Ditangkap</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:49:13 +0700</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E763" t="inlineStr">
+        <is>
+          <t>Polisi melakukan penindakan terhadap seorang pria yang masuk dalam DPO sejumlah kasus penembakan di Papua.</t>
+        </is>
+      </c>
+      <c r="F763" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G763" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265744/dpo-kasus-penembakan-kuala-kencana-hingga-mile-69-ditangkap</t>
+        </is>
+      </c>
+      <c r="H763" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/17vKsT7Hl4qvLcz2Ln_HgtGrIxQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319751/original/053062700_1786279748-Satgas.jpg</t>
+        </is>
+      </c>
+      <c r="I763" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>Suami Tewas di Waduk Jatiluhur, Istri Sumarna Bersiap Cari Kerja, Ada Keinginan yang Belum Terwujud</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:44:12 +0700</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr">
+        <is>
+          <t>Istri Sumarna bersiap mencari kerja setelah suaminya tewas di Waduk Jatiluhur, sementara keinginan renovasi rumah belum terwujud.</t>
+        </is>
+      </c>
+      <c r="F764" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G764" t="inlineStr">
+        <is>
+          <t>https://bandung.kompas.com/read/2026/08/09/204100278/suami-tewas-di-waduk-jatiluhur-istri-sumarna-bersiap-cari-kerja-ada</t>
+        </is>
+      </c>
+      <c r="H764" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/gEW_EXysTZwFtuHHgIQ8Q-jebd4=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/08/6a7729e6144a6.jpeg</t>
+        </is>
+      </c>
+      <c r="I764" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Pemprov DKI Bidik Birokrasi Tanpa Noda, Zona Integritas Diperluas hingga Kelurahan</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:44:12 +0700</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E765" t="inlineStr">
+        <is>
+          <t>Pemprov DKI targetkan Zona Integritas di semua perangkat demi 'Birokrasi Tanpa Noda'. Namun, tantangan pungli &amp; perlunya transformasi digital jadi sorotan.</t>
+        </is>
+      </c>
+      <c r="F765" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G765" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/09/20014971/pemprov-dki-bidik-birokrasi-tanpa-noda-zona-integritas-diperluas-hingga</t>
+        </is>
+      </c>
+      <c r="H765" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/Q5zhfSuEN1ytOzFRkeEx54o0MTk=/0x1:1000x668/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2017/09/05/1495323480.jpg</t>
+        </is>
+      </c>
+      <c r="I765" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I705"/>
+  <autoFilter ref="A1:I765"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 14:28 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$765</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$801</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I765"/>
+  <dimension ref="A1:I801"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -36393,8 +36393,1700 @@
         </is>
       </c>
     </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Polres Lamongan selidiki kebakaran puluhan kios di kawasan Babat</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:18:43 +0700</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr">
+        <is>
+          <t>Kepolisian Resor (Polres) Lamongan menyelidiki kebakaran yang menghanguskan puluhan kios pedagang kaki lima di ...</t>
+        </is>
+      </c>
+      <c r="F766" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G766" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686865/polres-lamongan-selidiki-kebakaran-puluhan-kios-di-kawasan-babat</t>
+        </is>
+      </c>
+      <c r="H766" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-09-at-19.16.56.jpeg</t>
+        </is>
+      </c>
+      <c r="I766" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Wagub Jatim: Penanganan karhutla TNBTS butuh keterlibatan banyak pihak</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:12:19 +0700</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E767" t="inlineStr">
+        <is>
+          <t>Wakil Gubernur Jawa Timur Emil Elestianto Dardak mengatakan penanganan kebakaran hutan dan lahan (karhutla) di kawasan ...</t>
+        </is>
+      </c>
+      <c r="F767" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G767" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686863/wagub-jatim-penanganan-karhutla-tnbts-butuh-keterlibatan-banyak-pihak</t>
+        </is>
+      </c>
+      <c r="H767" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-09-at-16.37.37-1024x576.jpeg</t>
+        </is>
+      </c>
+      <c r="I767" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Apakah gula aren aman untuk diabetes? Ini fakta yang perlu diketahui</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:09:34 +0700</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E768" t="inlineStr">
+        <is>
+          <t>Gula aren semakin populer sebagai pemanis alami untuk berbagai makanan dan minuman. Rasanya yang khas membuat gula ini ...</t>
+        </is>
+      </c>
+      <c r="F768" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G768" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686860/apakah-gula-aren-aman-untuk-diabetes-ini-fakta-yang-perlu-diketahui</t>
+        </is>
+      </c>
+      <c r="H768" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/05/perajin-gula-aren-di-pulau-kabaena-2800203.jpg</t>
+        </is>
+      </c>
+      <c r="I768" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Jangan lari! Ini yang harus dilakukan saat bertemu harimau</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:03:36 +0700</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E769" t="inlineStr">
+        <is>
+          <t>Harimau merupakan salah satu predator puncak di alam liar yang memiliki kekuatan, kecepatan, dan naluri berburu yang ...</t>
+        </is>
+      </c>
+      <c r="F769" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G769" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686857/jangan-lari-ini-yang-harus-dilakukan-saat-bertemu-harimau</t>
+        </is>
+      </c>
+      <c r="H769" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/04/Kelahiran-anak-harimau-Sumatera-di-TSI-II-Prigen-040626-um-9A.jpg</t>
+        </is>
+      </c>
+      <c r="I769" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Basarnas akhiri monitoring KMP Mutiara Sentosa II</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:00:56 +0700</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>Badan SAR Nasional (Basarnas) mengakhiri monitoring aktif KMP Mutiara Sentosa II setelah empat hari melakukan ...</t>
+        </is>
+      </c>
+      <c r="F770" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G770" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686855/basarnas-akhiri-monitoring-kmp-mutiara-sentosa-ii</t>
+        </is>
+      </c>
+      <c r="H770" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/290226.jpg</t>
+        </is>
+      </c>
+      <c r="I770" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Polda Sumut sita 169,6 kg ganja dan tangkap tiga orang</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:00:49 +0700</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>Direktorat Reserse Narkoba Polda Sumatera Utara mengungkap peredaran 169,6 kilogram ganja dan menangkap tiga orang ...</t>
+        </is>
+      </c>
+      <c r="F771" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G771" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686853/polda-sumut-sita-1696-kg-ganja-dan-tangkap-tiga-orang</t>
+        </is>
+      </c>
+      <c r="H771" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001217102.jpg</t>
+        </is>
+      </c>
+      <c r="I771" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>Gigitan kutu kasur seperti apa? Kenali ciri dan cara mengatasinya</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:58:15 +0700</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>Gigitan kutu kasur atau bed bug dapat menyebabkan rasa gatal, kemerahan, hingga gangguan tidur pada sebagian orang. ...</t>
+        </is>
+      </c>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G772" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686849/gigitan-kutu-kasur-seperti-apa-kenali-ciri-dan-cara-mengatasinya</t>
+        </is>
+      </c>
+      <c r="H772" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/peningkatan-okupansi-hotel-usai-libur-sekolah-2834148.jpg</t>
+        </is>
+      </c>
+      <c r="I772" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>Bank Jakarta jadi energi Persija raih gelar juara Liga Indonesia</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:57:53 +0700</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>Kolaborasi Bank Jakarta dan Persija Jakarta kembali diperkuat untuk menjadi tambahan energi bagi klub dengan sebutan ...</t>
+        </is>
+      </c>
+      <c r="F773" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G773" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686848/bank-jakarta-jadi-energi-persija-raih-gelar-juara-liga-indonesia</t>
+        </is>
+      </c>
+      <c r="H773" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_191027536.jpg</t>
+        </is>
+      </c>
+      <c r="I773" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>Deplu AS lapor ke Kongres soal kirim senjata dari Turkiye ke Ukraina</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:55:25 +0700</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>Departemen Luar Negeri Amerika Serikat telah melaporkan ke Kongres AS mengenai rencana pengalihan sistem persenjataan ...</t>
+        </is>
+      </c>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G774" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686847/deplu-as-lapor-ke-kongres-soal-kirim-senjata-dari-turkiye-ke-ukraina</t>
+        </is>
+      </c>
+      <c r="H774" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/10/17/XxjpbeE000227_20251017_PEPFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I774" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Barantin pastikan pelayanan karantina di Jatim berjalan optimal</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:54:31 +0700</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>Kepala Badan Karantina Indonesia (Barantin) Abdul Kadir Karding memastikan pelayanan pemeriksaan dan tindakan ...</t>
+        </is>
+      </c>
+      <c r="F775" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G775" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686844/barantin-pastikan-pelayanan-karantina-di-jatim-berjalan-optimal</t>
+        </is>
+      </c>
+      <c r="H775" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/ANTARA-2026-08-09T191443.484.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I775" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Kasus temuan 995 senjata, sekolah di Jaksel terapkan PJJ total selama sepekan</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:53:22 +0700</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>Sekolah swasta di kawasan Pondok Pinang, Kebayoran Lama, Jakarta Selatan (Jaksel) menerapkan sistem pembelajaran jarak ...</t>
+        </is>
+      </c>
+      <c r="F776" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G776" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686840/kasus-temuan-995-senjata-sekolah-di-jaksel-terapkan-pjj-total-selama-sepekan</t>
+        </is>
+      </c>
+      <c r="H776" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_203301330.jpg</t>
+        </is>
+      </c>
+      <c r="I776" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>Ambeien bisa sembuh sendiri tanpa operasi? Ini penjelasannya</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:52:53 +0700</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>Ambeien atau wasir merupakan salah satu gangguan kesehatan yang cukup umum dialami masyarakat. Meski sering dianggap ...</t>
+        </is>
+      </c>
+      <c r="F777" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G777" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686839/ambeien-bisa-sembuh-sendiri-tanpa-operasi-ini-penjelasannya</t>
+        </is>
+      </c>
+      <c r="H777" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2021/12/01/hemorrhoids-g0b8475a98_1280.jpg</t>
+        </is>
+      </c>
+      <c r="I777" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Anggota DPR-BNPB lakukan penguatan literasi kebencanaan di Batola</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:52:40 +0700</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>Anggota Komisi VIII DPR Sandi Fitrian Noor berkolaborasi dengan Direktorat Sistem Penanggulangan Bencana BNPB melakukan ...</t>
+        </is>
+      </c>
+      <c r="F778" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G778" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686835/anggota-dpr-bnpb-lakukan-penguatan-literasi-kebencanaan-di-batola</t>
+        </is>
+      </c>
+      <c r="H778" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_20260809_213657.jpg</t>
+        </is>
+      </c>
+      <c r="I778" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Kemenkum DIY gratiskan 30 pencatatan hak cipta di Malioboro</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:52:16 +0700</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>Kantor Wilayah Kementerian Hukum Daerah Istimewa Yogyakarta memfasilitasi 30 pencatatan hak cipta secara gratis bagi ...</t>
+        </is>
+      </c>
+      <c r="F779" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G779" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686831/kemenkum-diy-gratiskan-30-pencatatan-hak-cipta-di-malioboro</t>
+        </is>
+      </c>
+      <c r="H779" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_20260809_155915.jpg</t>
+        </is>
+      </c>
+      <c r="I779" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>38 atlet Indonesia raih medali dari Kejuaraan Taekwondo Asia</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:44:46 +0700</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>Pengurus Besar Taekwondo Indonesia (PBTI) mengumumkan 28 atlet berhasil meraih medali dalam 8th Asian Taekwondo ...</t>
+        </is>
+      </c>
+      <c r="F780" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G780" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686827/38-atlet-indonesia-raih-medali-dari-kejuaraan-taekwondo-asia</t>
+        </is>
+      </c>
+      <c r="H780" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/ec82d92b-a972-4557-9899-d419b6651b1f.jpeg</t>
+        </is>
+      </c>
+      <c r="I780" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>E-Sports Kapolri Cup 2026 Diikuti 35.936 Peserta, Pecahkan 3 Rekor MURI</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:59:47 +0700</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>E-Sports Kapolri Cup 2026 ditutup meriah di Jakarta, melibatkan 35.936 peserta.  Selain itu juga mencatatkan tiga rekor Museum Rekor-Dunia Indonesia (MURI).</t>
+        </is>
+      </c>
+      <c r="F781" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G781" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611313/e-sports-kapolri-cup-2026-diikuti-35-936-peserta-pecahkan-3-rekor-muri</t>
+        </is>
+      </c>
+      <c r="H781" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kapolri-jenderal-listyo-sigit-prabowo-menutup-e-sports-kapolri-cup-2026-dok-istimewa-1786283925475_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I781" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>1.476 Akademisi TEP Dibekali Kemampuan Narasi Digital Berbasis Empati</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:56:17 +0700</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Chayyara Zulghifary</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>Kementrans membekali 1.476 akademisi TEP 2026 tentang komunikasi publik berbasis empati untuk memperkuat kawasan transmigrasi dan interaksi dengan masyarakat.</t>
+        </is>
+      </c>
+      <c r="F782" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G782" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611310/1-476-akademisi-tep-dibekali-kemampuan-narasi-digital-berbasis-empati</t>
+        </is>
+      </c>
+      <c r="H782" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kementerian-transmigrasi-membekali-1476-akademisi-yang-tergabung-dalam-tim-ekspedisi-patriot-tep-2026-tentang-pentingnya-komun-1786283093819.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I782" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Kepala BNN: Modifikasi Ketamin Lewat Liquid Vape Sangat Sulit Dideteksi</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:51:56 +0700</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Kadek Melda Luxiana</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>Kepala BNN, Komjen Suyudi menyoroti modus penyalahgunaan ketamin. Salah satu yang sulit dideteksi yakni memodivikasi lewat liquid vape.</t>
+        </is>
+      </c>
+      <c r="F783" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G783" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611308/kepala-bnn-modifikasi-ketamin-lewat-liquid-vape-sangat-sulit-dideteksi</t>
+        </is>
+      </c>
+      <c r="H783" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kepala-bnn-komjen-suyudi-ario-seto-saat-konferensi-pers-penyelundupan-zat-psikotropika-ketamin-seberat-1298-kilogram-atau-hamp-1786283495790_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I783" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Kapolri Ajak Generasi Muda Jadi Duta Kamtibmas di Ruang Digital</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:36:15 +0700</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>Kapolri mengajak generasi muda memanfaatkan perkembangan teknologi sebagai ruang berkarya, berprestasi, sekaligus berkontribusi menjaga keamanan dunia digital.</t>
+        </is>
+      </c>
+      <c r="F784" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G784" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611289/kapolri-ajak-generasi-muda-jadi-duta-kamtibmas-di-ruang-digital</t>
+        </is>
+      </c>
+      <c r="H784" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kapolri-jenderal-listyo-sigit-prabowo-dok-polri-1786282511671_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I784" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Antusiasme Tinggi, 35 Ribu Peserta Ramaikan E-Sports Kapolri Cup 2026</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:30:14 +0700</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>Ajang yang digelar secara berjenjang mulai tingkat Polres hingga nasional itu mencatat antusiasme tinggi melibatkan 35.936 peserta dalam 7 kategori perlombaan.</t>
+        </is>
+      </c>
+      <c r="F785" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G785" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611285/antusiasme-tinggi-35-ribu-peserta-ramaikan-e-sports-kapolri-cup-2026</t>
+        </is>
+      </c>
+      <c r="H785" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kapolri-jenderal-listyo-sigit-prabowo-dokist-1786282174958_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I785" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>Houthi Serang Kilang Milik Raksasa Minyak Arab Saudi</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:00:49 +0700</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>Pasukan bersenjata Houthi Yaman dikabarkan melakukan serangan terhadap kilang milik raksasa minyak Arab Saudi, Aramco, Minggu (9/8/2026) pagi.</t>
+        </is>
+      </c>
+      <c r="F786" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G786" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8611265/houthi-serang-kilang-milik-raksasa-minyak-arab-saudi</t>
+        </is>
+      </c>
+      <c r="H786" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/04/09/ilustrasi-kilang-minyak-bumi-1775700731890_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I786" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Israel Siap Serang Iran Sendirian Jika AS Putuskan Damai</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:20:13 +0700</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>Israel dilaporkan tengah mempersiapkan kemungkinan melakukan serangan sepihak ke Iran jika perang Washington vs Teheran berakhir.</t>
+        </is>
+      </c>
+      <c r="F787" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G787" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260809170557-120-1390356/israel-siap-serang-iran-sendirian-jika-as-putuskan-damai</t>
+        </is>
+      </c>
+      <c r="H787" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/09/30/benjamin-netanyahu-1759177133099_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I787" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Iran Ngotot Tak Bakal Buka Selat Hormuz Sampai AS Penuhi Tuntutan</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:30:03 +0700</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>Iran menegaskan tak akan membuka Selat Hormuz sebelum AS memenuhi syarat yang diajukan Teheran, termasuk pemberian kompensasi atas kerusakan akibat perang.</t>
+        </is>
+      </c>
+      <c r="F788" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G788" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260809182933-120-1390364/iran-ngotot-tak-bakal-buka-selat-hormuz-sampai-as-penuhi-tuntutan</t>
+        </is>
+      </c>
+      <c r="H788" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/06/15/kesepakatan-damai-di-depan-mata-selat-hormuz-segera-buka-1781505172624_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Maskapai Jetstar dan Qatar Airways Hampir Tabrakan di Bandara Sydney</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:30:36 +0700</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>Pesawat Jetstar hampir bertabrakan dengan pesawat Qatar Airways di Bandara Sydney, Australia, Minggu (9/8) pagi, hingga menyebabkan seorang awak kabin terluka.</t>
+        </is>
+      </c>
+      <c r="F789" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G789" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260809173054-113-1390359/maskapai-jetstar-qatar-airways-hampir-tabrakan-di-bandara-sydney</t>
+        </is>
+      </c>
+      <c r="H789" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/02/27/nyalang-edisi-28-februari-2026-1772191228577_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I789" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Timteng Makin Panas, Houthi Bom Situs Minyak Saudi dan Wilayah Yaman</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:13:25 +0700</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>Milisi yang menguasai Yaman Houthi menggempur fasilitas minyak Arab Saudi di dekat pesisir Laut Merah menyusul konflik yang memanas di antara kedua pihak ini.</t>
+        </is>
+      </c>
+      <c r="F790" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G790" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260809180312-120-1390363/timteng-makin-panas-houthi-bom-situs-minyak-saudi-wilayah-yaman</t>
+        </is>
+      </c>
+      <c r="H790" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/09/17/israel-palestiniansyemen-missiles_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I790" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>AS Marah China Klaim Cagar Alam Nasional di Laut China Selatan</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:10:00 +0700</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>Amerika Serikat menolak aturan baru China yang memberlakukan cagar alam nasional di Scarborough Reef, Laut China Selatan (LCS).</t>
+        </is>
+      </c>
+      <c r="F791" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G791" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260809162055-113-1390338/as-marah-china-klaim-cagar-alam-nasional-di-laut-china-selatan</t>
+        </is>
+      </c>
+      <c r="H791" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2021/09/17/pulau-spratly_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I791" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Cerita Haru Korban Selamat dari Penembakan Massal di Sekolah Thailand</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:30:41 +0700</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>Khim, korban selamat penembakan di sekolah Thailand, menceritakan upaya melarikan diri dan momen menegangkan saat bersembunyi.</t>
+        </is>
+      </c>
+      <c r="F792" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G792" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260809151245-106-1390320/cerita-haru-korban-selamat-dari-penembakan-massal-di-sekolah-thailand</t>
+        </is>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/penembakan-sekolah-di-thailand-1786076745948_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I792" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Jaring Bibit Atlet, Kapolri Instruksikan Polsek hingga Polda Rutin Gelar Turnamen E-Sports</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:08:32 +0700</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>Kapolri menutup ajang E-Sports Kapolri Cup 2026 yang digelar di Indonesia Arena, Senayan, Jakarta Pusat, Minggu (9/8/2026) malam.</t>
+        </is>
+      </c>
+      <c r="F793" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G793" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866095/jaring-bibit-atlet-kapolri-instruksikan-polsek-hingga-polda-rutin-gelar-turnamen-e-sports</t>
+        </is>
+      </c>
+      <c r="H793" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/QmgtZbIL65368-l6y6kWQUq_tEM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kapolri-Jenderal-Polisi-Listyo-Sigit-Prabowo-memberikan-sambutan-esport.jpg</t>
+        </is>
+      </c>
+      <c r="I793" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>BPS Targetkan Sensus Ekonomi 2026 Tuntas 100 Persen pada 17 Agustus</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:50:44 +0700</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>BPS merilis laporan perkembangan terbaru mengenai capaian pelaksanaan Sensus Ekonomi 2026 (SE2026) di seluruh Indonesia.</t>
+        </is>
+      </c>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866094/bps-targetkan-sensus-ekonomi-2026-tuntas-100-persen-pada-17-agustus</t>
+        </is>
+      </c>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/F9rZc4PGtQnpYxYHZituBFKuuoA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kepala-BPS-Amalia-Adininggar-Widyasanti-Podcast-di-Tribunnews_20260808_161633.jpg</t>
+        </is>
+      </c>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Klasemen MotoGP 2026 Terbaru: Bezzecchi Melonjak ke P2, Marc Marquez Tetap Top 5</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:40:15 +0700</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>Klasemen MotoGP 2026 terbaru dengan Marco Bezzecchi melesat ke posisi kedua sedangkan Marc Marquez masih berada di lima besar.</t>
+        </is>
+      </c>
+      <c r="F795" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G795" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866093/klasemen-motogp-2026-terbaru-bezzecchi-melonjak-ke-p2-marc-marquez-tetap-top-5</t>
+        </is>
+      </c>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/3MLG1vozM3YvZqsFCnSZnDo5bzc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Jorge-Martin-dan-Marco-Bezzecchi-MotoGP-Brasil-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Cerita Humanis Sensus Ekonomi 2026: Temukan Nenek Usia 100 Tahun yang Masih Mahir Menjahit</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:38:46 +0700</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>Di tengah proses sensus rumah tangga, petugas mendapati seorang nenek yang telah genap berusia 100 tahun pada bulan Mei lalu.</t>
+        </is>
+      </c>
+      <c r="F796" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866092/cerita-humanis-sensus-ekonomi-2026-temukan-nenek-usia-100-tahun-yang-masih-mahir-menjahit</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/z6GkWu0NKfz0Zaif-Mo6Xw5C5Gc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/sensus-ekonomi-2026-ppl-dkn-jakbar.jpg</t>
+        </is>
+      </c>
+      <c r="I796" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Doa agar Terhindar dari Penyesalan dan Kehinaan di Hari Kiamat</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:33:14 +0700</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>Orang yang tidak bertaubat hingga kematiannya akan masuk menjadi orang yang menyesal dan terhina di hari kiamat. Berikut doa agar dilindungi Allah.</t>
+        </is>
+      </c>
+      <c r="F797" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G797" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/lifestyle/7866091/doa-agar-terhindar-dari-penyesalan-dan-kehinaan-di-hari-kiamat</t>
+        </is>
+      </c>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8gzz-QTNliKeK_p_ID0RcRMyUXU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/DOA-AGAR-SELAMAT-DI-HARI-KIAMAT-345324532.jpg</t>
+        </is>
+      </c>
+      <c r="I797" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>HP Biasa Mulai Ditinggalkan, Ponsel Jenis Ini Guncang Pasar 2026</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:00:17 +0700</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>Industri ponsel global diprediksi berubah besar pada 2026, dengan HP lipat tumbuh pesat hingga 30%, sementara HP konvensional menyusut.</t>
+        </is>
+      </c>
+      <c r="F798" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260809190316-37-757746/hp-biasa-mulai-ditinggalkan-ponsel-jenis-ini-guncang-pasar-2026</t>
+        </is>
+      </c>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/04/07/harga-laptop-masih-mengalami-kenaikan-di-beberapa-toko-itc-kuningan-jakarta-selasa-742026-1775551030645_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I798" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Hasil Klasemen Moto3 2026, Veda Ega Pratama Bertahan di Posisi 6</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:28:55 +0700</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>Veda Ega Pratama mengoleksi 97 poin di klasemen sementara Moto3 2026 bersama Honda Team Asia.</t>
+        </is>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G799" t="inlineStr">
+        <is>
+          <t>https://otomotif.kompas.com/read/2026/08/09/212815515/hasil-klasemen-moto3-2026-veda-ega-pratama-bertahan-di-posisi-6</t>
+        </is>
+      </c>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/qX_kW7KvheqAfued2WwRubyuIFk=/0x0:3751x2501/1200x675/filters:watermark(data/photo/2026/01/30/697c81750a668.png,0,-0,1)/data/photo/2026/07/13/6a54088886ae4.jpg</t>
+        </is>
+      </c>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Sosok Perempuan Viral di Kasus Bos Royal Phone Ambarawa, Polisi Ungkap Fakta Sebenarnya</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:28:55 +0700</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>Perempuan viral disebut terlibat dalam kasus pembunuhan bos Royal Phone Ambarawa. Polisi ungkap fakta sebenarnya.</t>
+        </is>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/09/202828278/sosok-perempuan-viral-di-kasus-bos-royal-phone-ambarawa-polisi-ungkap-fakta</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/MOq4rRFJXp6J8zjl7NVtC_Xzxls=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/07/6a755d6d525c7.jpg</t>
+        </is>
+      </c>
+      <c r="I800" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>Advertorial</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Punya Wishlist Mobil, Motor, atau Rumah? Event Menarik Ini Patut Ditunggu</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:28:55 +0700</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>BCA EXPO 2026 segera hadir dengan penawaran KPR, KKB, dan KSM. Simak cara siapkan rencana finansial matang sebelum mewujudkan kendaraan dan rumah impi</t>
+        </is>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>https://biz.kompas.com/read/2026/08/09/195103028/punya-wishlist-mobil-motor-atau-rumah-event-menarik-ini-patut-ditunggu</t>
+        </is>
+      </c>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/aHkyqSUs53sLkdg_9IkNSq-QCn4=/0x0:1200x800/1200x675/data/photo/2026/08/09/6a787792b4c09.jpg</t>
+        </is>
+      </c>
+      <c r="I801" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I765"/>
+  <autoFilter ref="A1:I801"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 15:23 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$801</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$822</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I801"/>
+  <dimension ref="A1:I822"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -38085,8 +38085,998 @@
         </is>
       </c>
     </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Veda Ega finis posisi sembilan pada Moto3 Inggris 2026</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:13:07 +0700</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>25 poin
+2. Álvaro Carpe - +0.701 - 20 poin
+3. Valentín Perrone - +0.991 - 16 poin
+4. Adrián ...</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686892/veda-ega-finis-posisi-sembilan-pada-moto3-inggris-2026</t>
+        </is>
+      </c>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/21/Latihan-pembalap-nasional-Moto2-dan-Moto3-di-Mandalika-210726-AS-4.jpg</t>
+        </is>
+      </c>
+      <c r="I802" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Kisah JPO 'Tanpa Hubungan' di Rasuna Said Bakal Tinggal Kenangan</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:00:35 +0700</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>JPO di Jalan HR Rasuna Said akan dibongkar karena tidak terhubung dengan LRT dan tidak ramah disabilitas. Proses pembongkaran ditargetkan selesai tiga minggu.</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G803" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611368/kisah-jpo-tanpa-hubungan-di-rasuna-said-bakal-tinggal-kenangan</t>
+        </is>
+      </c>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/konektivitas-jpo-rasuna-said-disorot-efisiensi-mobilitas-kawasan-bisnis-jadi-sorotan-1785989995559_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Viral Maling Bobol Rumah Warga Malah Tertidur Pulas di Lampung</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:49:50 +0700</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>Tommy Saputra</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>Seorang pria di Pringsewu, Lampung, tertangkap saat mencuri dan tertidur di rumah yang dibobol. Pelaku, IM, adalah residivis pencurian.</t>
+        </is>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611357/viral-maling-bobol-rumah-warga-malah-tertidur-pulas-di-lampung</t>
+        </is>
+      </c>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/maling-ketiduran-di-rumah-korban-berujung-ditangkap-1786199485325_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Cerita Duta Anti-bullying Komnas PA Pernah Speak Up Kasus Pelecehan Anak</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:43:53 +0700</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>Adhfar Aulia Syuhada</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>Komnas Anak mengangkat lima Duta Anak Anti-bullying, termasuk Chacha dan Malik, untuk menyuarakan isu pelecehan dan bullying.</t>
+        </is>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G805" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611351/cerita-duta-anti-bullying-komnas-pa-pernah-speak-up-kasus-pelecehan-anak</t>
+        </is>
+      </c>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/komnas-anak-mengangkat-lima-duta-anak-anti-bullying-termasuk-chacha-dan-malik-adhfardetikcom-1786286594559_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Ajak Generasi Muda Jadi Duta Kamtibmas, Kapolri: Laporkan Lewat Layanan 110</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:24:23 +0700</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>Kapolri Cup 2026 jadi momentum bagi Polri merangkul generasi muda E-Sports. Kapolri mengajak atlet jadi Duta Kamtibmas dan aktif lawan kejahatan siber.</t>
+        </is>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611343/ajak-generasi-muda-jadi-duta-kamtibmas-kapolri-laporkan-lewat-layanan-110</t>
+        </is>
+      </c>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kapolri-jenderal-listyo-sigit-prabowo-ajak-atlet-dan-penikmat-gim-digital-untuk-mengambil-peran-aktif-menjaga-keamanan-ruang-d-1786285379118.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I806" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Trump Siap Kucurkan Rp 53 T buat Proyek Mineral Kritis &amp;amp; Baterai</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:00:13 +0700</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>Kita sedang merebut kembali tempat Amerika yang seharusnya sebagai negara adidaya mineral dunia, kata Trump.</t>
+        </is>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G807" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8611271/trump-siap-kucurkan-rp-53-t-buat-proyek-mineral-kritis-baterai</t>
+        </is>
+      </c>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/presiden-as-donald-trump-saat-seremoni-penandatanganan-perintah-eksekutif-membatasi-hak-kewarganegaraan-berdasarkan-tempat-kel-1786086100834_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I807" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Transjakarta Kelola Transportasi ke Kepulauan Seribu Mulai 2027</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:30:13 +0700</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>Gubenur DKI Jakarta Pramono Anung menyebut Transjakarta akan mengelola transportasi laut hingga mencakup wilayah Kepulauan Seribu mulai 2027.</t>
+        </is>
+      </c>
+      <c r="F808" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G808" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260809194659-92-1390375/transjakarta-kelola-transportasi-ke-kepulauan-seribu-mulai-2027</t>
+        </is>
+      </c>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/06/21/pramono-siapkan-dukuh-atas-jadi-hub-6-moda-1782013873984_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I808" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Kado HUT ke-81 RI, Naik Transportasi DKI Cuma Rp1 pada 17 Agustus</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:30:25 +0700</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>Pemprov DKI Jakarta menerapkan tarif khusus naik semua transportasi umum di Jakarta cuma Rp1 pada 17 Agustus mendatang.</t>
+        </is>
+      </c>
+      <c r="F809" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G809" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260809155233-92-1390328/kado-hut-ke-81-ri-naik-transportasi-dki-cuma-rp1-pada-17-agustus</t>
+        </is>
+      </c>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/04/masyarakat-menggunakan-transportasi-umum-mrt-jakarta-1785841998352_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I809" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Lebih Terjangkau, Kuy Beli Kulkas dan AC di Transmart Full Day Sale</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>Transmart Full Day Sale balik lagi hari ini, Minggu (9/8), bawa diskon gede-gedean 50 persen plus 20 persen. Serbu Transmart terdekat sekarang.</t>
+        </is>
+      </c>
+      <c r="F810" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807123606-97-1389672/lebih-terjangkau-kuy-beli-kulkas-ac-di-transmart-full-day-sale</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/10/transmart-full-day-sale-1783668437996_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Kapolri Ajak Duta Kamtibmas Gen Z Aktif Laporkan Judi Online dan Kejahatan Siber</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:56:17 +0700</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>Kapolri Jenderal Listyo Sigit Prabowo memberikan pesan khusus kepada para pemuda untuk melaporkan berbagai bentuk kejahatan di dunia digital</t>
+        </is>
+      </c>
+      <c r="F811" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G811" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866102/kapolri-ajak-duta-kamtibmas-gen-z-aktif-laporkan-judi-online-dan-kejahatan-siber</t>
+        </is>
+      </c>
+      <c r="H811" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/BwRRI08g2W0vhFKXAz051rDmBDk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kapolri-Pimpin-Upacara-Kenaikan-Pangkat-87-Perwira-Tinggi_20260630_144044.jpg</t>
+        </is>
+      </c>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Koperasi Desa Dinilai Jadi Kunci Kemandirian Ekonomi</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:48:58 +0700</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>Rocky Gerung di Maiyah Kebangsaan UNSIQ: koperasi desa jangan dibatalkan, berantas korupsi tanpa hentikan program kerakyatan.</t>
+        </is>
+      </c>
+      <c r="F812" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866101/koperasi-desa-dinilai-jadi-kunci-kemandirian-ekonomi</t>
+        </is>
+      </c>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/RH311ouFpQuSYWbUK5q-n45olXQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Maiyah-Kebangsaan-yang-digelar-Gerakan-Mantap-Pilih-Prabowo.jpg</t>
+        </is>
+      </c>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>130 Ribu Jemaah Hadiri Zikir Kebangsaan HUT ke-81 RI di Masjid Istiqlal</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:47:25 +0700</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>jumlah jemaah yang menghadiri Zikir Kebangsaan, Doa Keselamatan Bangsa, dan Haul Pendiri NKRI di Masjid Istiqlal mencapai sekitar 130 ribu orang</t>
+        </is>
+      </c>
+      <c r="F813" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G813" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866100/130-ribu-jemaah-hadiri-zikir-kebangsaan-hut-ke-81-ri-di-masjid-istiqlal</t>
+        </is>
+      </c>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Y066mRZVnPn0n9bY6M3jPBxEe-U=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Zikir-Kebangsaan-Doa-Keselamatan-Bangsa.jpg</t>
+        </is>
+      </c>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Kata Herry IP setelah Anak Didiknya Juara Korea Masters 2026: Uji Coba Belum Selesai</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:35:51 +0700</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>Herry IP apresiasi gelar Tee Kai Wun/Roy King Yap di Korea Masters 2026 sambil menegaskan proses uji coba ganda putra Malaysia masih panjang.</t>
+        </is>
+      </c>
+      <c r="F814" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866099/kata-herry-ip-setelah-anak-didiknya-juara-korea-masters-2026-uji-coba-belum-selesai</t>
+        </is>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/olMURgR7arNgdKd1jOjYkI-cC_k=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Herry-IP-Resmi-Latih-Malaysia.jpg</t>
+        </is>
+      </c>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Buntut Temuan 996 Senpi di Sekolah Swasta Jaksel, Komnas Anak Ingin Cek Kondisi Psikologis Siswa</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:27:37 +0700</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>Ketua Komnas PA DKI Jakarta Cornelia Agatha menanggapi kasus temuan 996 senjata di sebuah sekolah swasta di daerah Kebayoran Lama, Jakarta Selatan.</t>
+        </is>
+      </c>
+      <c r="F815" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G815" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866098/buntut-temuan-996-senpi-di-sekolah-swasta-jaksel-komnas-anak-ingin-cek-kondisi-psikologis-siswa</t>
+        </is>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/wl8XiYd5H7OuJH96q3GMPDd3wgM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cornelia-agatha-jadi-sarah-di-film-akhir-kisah-cinta-si-doel_20200123_043253.jpg</t>
+        </is>
+      </c>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Niat Mau Rayakan Pernikahan Cristiano Ronaldo dengan Georgina, Ribuan Pasang Mata Salah Sasaran</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:25:28 +0700</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>Ribuan orang yang berkumpul di depan Katedral Funchal di Madeira tertipu dengan rumor tentang pernikahan Cristiano Ronaldo dengan Georgina Rodriguez.</t>
+        </is>
+      </c>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866097/niat-mau-rayakan-pernikahan-cristiano-ronaldo-dengan-georgina-ribuan-pasang-mata-salah-sasaran</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/7LkET5PoSOkqurBXDmIhoMnwHvo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/momen-terburuk-georgina-rodriguez-saat-bayi-laki-lakinya-meninggal.jpg</t>
+        </is>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Jemaah Doa Bersama HUT RI di Masjid Istiqlal Membludak, Menag Gandeng Tangan Habib Luthfi Saat Tiba</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:25:23 +0700</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>Pengunjung acara Doa Keselamatan Bangsa, Zikir Kebangsaan, dan Haul Pendiri NKRI Dalam Rangka HUT Ke-81 RI di Masjid Istiqlal membludak</t>
+        </is>
+      </c>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866096/jemaah-doa-bersama-hut-ri-di-masjid-istiqlal-membludak-menag-gandeng-tangan-habib-luthfi-saat-tiba</t>
+        </is>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/QVgtkojKnE8qASQet9-RlLWvSrI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Acara-Doa-Keselamatan-Bangsa-Zikir-Kebangsaan.jpg</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Transformasi Digital, Bank Jakarta Perbarui Situs dan Perkuat Ekosistem</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Perkembangan layanan digital mendorong perbankan untuk tidak hanya memperbarui teknologi, tetapi juga meningkatkan pengalaman nasabah. Bank Jakarta merespons perubahan tersebut dengan memperbarui laman resmi sekaligus memperkuat strategi...</t>
+        </is>
+      </c>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tji6po416/transformasi-digital-bank-jakarta-perbarui-situs-dan-perkuat-ekosistem</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260809200631-670.png</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Yayasan Ungkap Awal Mula Penemuan Senjata Api di Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:54:58 +0700</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>Pihak yayasan mengungkap kronologi awal penemuan senjata, narkoba, hingga rekaman video pornografi, di sekolah Jaksel.</t>
+        </is>
+      </c>
+      <c r="F819" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G819" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265818/yayasan-ungkap-awal-mula-penemuan-senjata-api-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/YAVOExu6fnI0Yew1ROoX836YmpQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319668/original/013460500_1786264819-71184.jpg</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Bank Jakarta Jadi Sponsor Persija, Dirut Singgung Target yang Tak Ada di Kontrak Shin Tae-yong</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:23:39 +0700</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>Bank Jakarta resmi sponsori Persija 2026/2027 dengan target juara sebagai hadiah HUT Jakarta ke-500. Kolaborasi ini selaras filosofi STY dan transformasi Bank Jakarta.</t>
+        </is>
+      </c>
+      <c r="F820" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G820" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/09/22193941/bank-jakarta-jadi-sponsor-persija-dirut-singgung-target-yang-tak-ada-di</t>
+        </is>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/kvw4cI2G_y7jnHMVMxq751GbJ0s=/160x107:1440x960/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/09/6a787ef5ecf08.jpg</t>
+        </is>
+      </c>
+      <c r="I820" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Java United Tunjuk Fabio Lefundes sebagai Pelatih Jelang Super League 2026-2027</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:23:39 +0700</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>Fabio Lefundes resmi diangkat sebagai pelatih Java United FC jelang bergulirnya Super League 2026-2027.</t>
+        </is>
+      </c>
+      <c r="F821" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>https://bola.kompas.com/read/2026/08/09/21140028/java-united-tunjuk-fabio-lefundes-sebagai-pelatih-jelang-super-league-2026-2027</t>
+        </is>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/pFO_LUYesVYcTjPaQMGpj25674o=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/05/22/6a0fc604788aa.jpg</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Grand Livina Ditabrak 2 Truk Tronton di Bekasi, Pengemudi Taksi Online Tewas</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:23:39 +0700</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>Kecelakaan maut melibatkan Grand Livina dan dua truk tronton di Bekasi. Sopir taksi online N tewas. Gagal rem picu tabrakan beruntun tragis di Simpang Lampu Merah Sawo.</t>
+        </is>
+      </c>
+      <c r="F822" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/09/20111991/grand-livina-ditabrak-2-truk-tronton-di-bekasi-pengemudi-taksi-online</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/DTJIqqUtfU5i4KPCgE3RNTyjxN4=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/09/6a7878bd0c684.jpg</t>
+        </is>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I801"/>
+  <autoFilter ref="A1:I822"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 16:24 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$822</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$860</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I822"/>
+  <dimension ref="A1:I860"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -39075,8 +39075,1797 @@
         </is>
       </c>
     </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Akhir pekan jadi momen orang tua melepas rindu di Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>ANTARA - Akhir pekan menjadi momen yang dinantikan para orang tua siswa Sekolah Rakyat Terintegrasi Tiga Provinsi Aceh. ...</t>
+        </is>
+      </c>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686901/akhir-pekan-jadi-momen-orang-tua-melepas-rindu-di-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AKHIR-PEKAN-JADI-MOMEN-ORANG-TUA-MELEPAS-RINDU-DI-SEKOLAH-RAKYAT.jpg</t>
+        </is>
+      </c>
+      <c r="I823" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Putri sulung Gus Dur berharap Muktamar NU berjalan baik</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:09:23 +0700</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>Putri sulung Presiden ke-4 RI Abdurrahman Wahid (Gus Dur) Alissa Wahid berharap, Muktamar Nahdlatul Ulama (NU) dapat ...</t>
+        </is>
+      </c>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686917/putri-sulung-gus-dur-berharap-muktamar-nu-berjalan-baik</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/241580.jpg</t>
+        </is>
+      </c>
+      <c r="I824" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>PSSI segera evaluasi total kegagalan Piala AFF 2026</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:07:07 +0700</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>Persatuan Sepak Bola Seluruh Indonesia (PSSI) segera melakukan evaluasi total setelah Timnas Indonesia gagal melaju ke ...</t>
+        </is>
+      </c>
+      <c r="F825" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686915/pssi-segera-evaluasi-total-kegagalan-piala-aff-2026</t>
+        </is>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/kongres-biasa-pssi-2026-2833315.jpg</t>
+        </is>
+      </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Pemkab Bekasi terapkan pertanian modern peralihan pola konvensional</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:06:47 +0700</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>Pemerintah Kabupaten Bekasi, Jawa Barat mulai menerapkan sistem pertanian modern sebagai peralihan dari pola tanam padi ...</t>
+        </is>
+      </c>
+      <c r="F826" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686911/pemkab-bekasi-terapkan-pertanian-modern-peralihan-pola-konvensional</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG-20260809-019.jpg</t>
+        </is>
+      </c>
+      <c r="I826" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Monitoring aktif KMP Mutiara Sentosa II resmi berakhir</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>ANTARA - Kantor SAR Surabaya mengakhiri monitoring aktif terhadap insiden KMP Mutiara Sentosa II di perairan utara ...</t>
+        </is>
+      </c>
+      <c r="F827" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G827" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686883/monitoring-aktif-kmp-mutiara-sentosa-ii-resmi-berakhir</t>
+        </is>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/MONITORING-AKTIF-KMP-MUTIARA-SENTOSA-II-RESMI-BERAKHIR.jpg</t>
+        </is>
+      </c>
+      <c r="I827" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Raul Fernandez tak terbendung pada MotoGP Inggris 2026</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:55:20 +0700</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>25 poin
+2. Jorge Martín - +2.540 - 20 poin
+3. Marco Bezzecchi - +3.713 - 16 poin
+4. Álex ...</t>
+        </is>
+      </c>
+      <c r="F828" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686908/raul-fernandez-tak-terbendung-pada-motogp-inggris-2026</t>
+        </is>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/10/04/marco-bezzecchi-juara-sprint-race-motogp-indonesia-2638345.jpg</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Kebakaran Bromo meluas, satgas dibentuk dan titik api baru muncul</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:49:41 +0700</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>ANTARA - ‎Upaya penanganan kebakaran di kawasan Taman Nasional Bromo Tengger Semeru terus diperkuat melalui ...</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686904/kebakaran-bromo-meluas-satgas-dibentuk-dan-titik-api-baru-muncul</t>
+        </is>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KEBAKARAN-BROMO-MELUAS-SATGAS-DIBENTUK-DAN-TITIK-API-BARU-MUNCUL.jpg</t>
+        </is>
+      </c>
+      <c r="I829" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Sambut HUT RI, KBRI KL hadirkan layanan paspor di akhir pekan</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:46:03 +0700</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>ANTARA - KBRI Kuala Lumpur menghadirkan layanan penggantian paspor pada akhir pekan bagi WNI di Malaysia. Program ...</t>
+        </is>
+      </c>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686869/sambut-hut-ri-kbri-kl-hadirkan-layanan-paspor-di-akhir-pekan</t>
+        </is>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SAMBUT-HUT-RI-KBRI-KL-HADIRKAN-LAYANAN-PASPOR-DI-AKHIR-PEKAN.jpg</t>
+        </is>
+      </c>
+      <c r="I830" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Gulkarmat Jaktim evakuasi dua pekerja proyek yang tertimpa turap</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:24:04 +0700</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>Petugas Suku Dinas Penanggulangan Kebakaran dan Penyelamatan (Gulkarmat) Jakarta Timur (Jaktim) mengevakuasi dua ...</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G831" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686899/gulkarmat-jaktim-evakuasi-dua-pekerja-proyek-yang-tertimpa-turap</t>
+        </is>
+      </c>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_220608901.jpg</t>
+        </is>
+      </c>
+      <c r="I831" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Kapolri apresiasi antusiasme peserta E-Sports Kapolri Cup 2026</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:19:41 +0700</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>Kepala kepolisian Republik Indonesia (Kapolri) Drs. Listyo Sigit Prabowo, M.Si. mengapresiasi antusiasme peserta ...</t>
+        </is>
+      </c>
+      <c r="F832" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686895/kapolri-apresiasi-antusiasme-peserta-e-sports-kapolri-cup-2026</t>
+        </is>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000131535.jpg</t>
+        </is>
+      </c>
+      <c r="I832" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>IESR sebut strategi multijalur jadi kunci percepatan PLTS 100 GW</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:15:20 +0700</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>Institute for Essential Services Reform (IESR) menilai bahwa keberhasilan program pembangkit listrik tenaga surya ...</t>
+        </is>
+      </c>
+      <c r="F833" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G833" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686893/iesr-sebut-strategi-multijalur-jadi-kunci-percepatan-plts-100-gw</t>
+        </is>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_20260809_220019.jpg</t>
+        </is>
+      </c>
+      <c r="I833" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Golkar ubah pola kaderisasi untuk gaet Gen Z menuju Pemilu 2029</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:10:37 +0700</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>Ketua Bidang Kepemudaan dan Olahraga DPP Partai Golkar Said Aldi Al Idrus mengatakan pola kaderisasi politik perlu ...</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686891/golkar-ubah-pola-kaderisasi-untuk-gaet-gen-z-menuju-pemilu-2029</t>
+        </is>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1000582857.jpg</t>
+        </is>
+      </c>
+      <c r="I834" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Filosofi sepak bola STY sejalan dengan transformasi Bank Jakarta</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:59:56 +0700</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>Filosofi permainan cepat, agresif, dan mengutamakan kerja sama tim yang diterapkan pelatih Persija Jakarta, Shin ...</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G835" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686889/filosofi-sepak-bola-sty-sejalan-dengan-transformasi-bank-jakarta</t>
+        </is>
+      </c>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_212330479.jpg</t>
+        </is>
+      </c>
+      <c r="I835" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>BI catat minat investasi capai Rp73 triliun di Pamor Borneo 2026</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:54:37 +0700</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>Bank Indonesia Provinsi Kalimantan Selatan mencatat minat investasi Rp73 triliun dari 20 investor domestik dan ...</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686887/bi-catat-minat-investasi-capai-rp73-triliun-di-pamor-borneo-2026</t>
+        </is>
+      </c>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_1796.jpeg</t>
+        </is>
+      </c>
+      <c r="I836" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Yayasan sekolah di Jaksel minta perlindungan KPAI soal temuan senjata</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:49:27 +0700</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>Yayasan sekolah swasta di kawasan Pondok Pinang, Kebayoran Lama, Jakarta Selatan meminta perlindungan dan pendampingan ...</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G837" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686880/yayasan-sekolah-di-jaksel-minta-perlindungan-kpai-soal-temuan-senjata</t>
+        </is>
+      </c>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/InShot_20260809_210842901.jpg</t>
+        </is>
+      </c>
+      <c r="I837" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Transnusa resmikan penerbangan perdana rute Jakarta-Bangkok</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:48:24 +0700</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>PT Transnusa Aviation Mandiri (Transnusa) resmi mengoperasikan penerbangan perdana (inaugural flight) rute ...</t>
+        </is>
+      </c>
+      <c r="F838" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G838" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686879/transnusa-resmikan-penerbangan-perdana-rute-jakarta-bangkok</t>
+        </is>
+      </c>
+      <c r="H838" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_0485.jpeg</t>
+        </is>
+      </c>
+      <c r="I838" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Kaki gatal terus? Kenali 5 penyebab, cara mengatasi dan mencegahnya</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:38:09 +0700</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>Kaki gatal merupakan keluhan yang cukup sering dialami banyak orang dan dapat muncul akibat berbagai faktor, mulai dari ...</t>
+        </is>
+      </c>
+      <c r="F839" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G839" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686877/kaki-gatal-terus-kenali-5-penyebab-cara-mengatasi-dan-mencegahnya</t>
+        </is>
+      </c>
+      <c r="H839" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/01/20/banjir-masih-merendam-desa-pasir-ampo-di-tangerang-2709206.jpg</t>
+        </is>
+      </c>
+      <c r="I839" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Thorslund hentikan Cherneka untuk rebut juara sejati bantam putri</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:35:45 +0700</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>Petinju Denmark, Dina Thorslund, mengalahkan Cherneka Johnson melalui kemenangan angka untuk merebut gelar juara sejati ...</t>
+        </is>
+      </c>
+      <c r="F840" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G840" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686875/thorslund-hentikan-cherneka-untuk-rebut-juara-sejati-bantam-putri</t>
+        </is>
+      </c>
+      <c r="H840" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/29dbaeea-01b6-4e8b-b4f6-183a585e42e8.jpeg</t>
+        </is>
+      </c>
+      <c r="I840" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Destinasi wisata di sekitar Bromo masih aman dikunjungi wisatawan</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:34:58 +0700</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>Kepala Dinas Kepemudaan, Olahraga dan Pariwisata (Disporapar) Kabupaten Probolinggo, Jawa Timur, Heri Mulyadi ...</t>
+        </is>
+      </c>
+      <c r="F841" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G841" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686873/destinasi-wisata-di-sekitar-bromo-masih-aman-dikunjungi-wisatawan</t>
+        </is>
+      </c>
+      <c r="H841" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/WhatsApp-Image-2026-08-09-at-16.34.57-1200x630.jpeg</t>
+        </is>
+      </c>
+      <c r="I841" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Sudah Padam, Kebakaran di Mal Nipah Makassar Diduga Akibat Korsleting</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:06:35 +0700</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>Reinhard Sopla</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>Kebakaran di Mal Nipah, Makassar, diduga akibat korsleting listrik. Api padam dalam 15 menit dan tak ada korban jiwa.</t>
+        </is>
+      </c>
+      <c r="F842" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G842" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611400/sudah-padam-kebakaran-di-mal-nipah-makassar-diduga-akibat-korsleting</t>
+        </is>
+      </c>
+      <c r="H842" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kebakaran-terjadi-di-mal-nipah-makassar-1786291264697_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I842" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Mal Nipah Makassar Kebakaran, Polisi Cek ke Lokasi</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:52:02 +0700</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>Reinhard Soplantila</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda Mal Nipah di Makassar pada 9 Agustus 2026. Belum diketahui penyebab kebakaran.</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611392/mal-nipah-makassar-kebakaran-polisi-cek-ke-lokasi</t>
+        </is>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/mal-nipah-makassar-kebakaran-1786285903782_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I843" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Brimob Polda Metro Bantu Tangani Kebakaran Gudang di Kosambi</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:42:26 +0700</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>Personel Brimob Polda Metro Jaya terlibat dalam penanganan kebakaran di Pergudangan Sentra Kosambi, Tangerang untuk memastikan keamanan dan respons cepat.</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611384/brimob-polda-metro-bantu-tangani-kebakaran-gudang-di-kosambi</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/brimob-polda-metro-jaya-bantu-tangani-kebakaran-gudang-di-kosambi-tangerang-dok-istimewa-1786290122276_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I844" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>3.200 Orang Bentangkan Bendera 500 Meter di Festival Merah Putih Bogor</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:27:02 +0700</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>M Solihin</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Bogor menggelar Festival Merah Putih ke-11, melibatkan 3.200 orang dan bendera 500 meter. Acara ini memperkuat nasionalisme dan dampak ekonomi.</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611378/3-200-orang-bentangkan-bendera-500-meter-di-festival-merah-putih-bogor</t>
+        </is>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/bendera-sepanjang-500-meter-diarak-di-kota-bogor-dokumen-pemkot-bogor-1786289203352_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I845" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Kapal Bawa 1,3 Ton Ketamin Disergap, Kepala BNN Beri Peringatan ke Sindikat Narkoba!</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:51:56 +0700</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>Kadek Melda Luxiana</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>Kepala BNN, Komjen Suyudi menyoroti modus penyalahgunaan ketamin. Salah satu yang sulit dideteksi yakni memodivikasi lewat liquid vape.</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611308/kapal-bawa-1-3-ton-ketamin-disergap-kepala-bnn-beri-peringatan-ke-sindikat-narkoba</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kepala-bnn-komjen-suyudi-ario-seto-saat-konferensi-pers-penyelundupan-zat-psikotropika-ketamin-seberat-1298-kilogram-atau-hamp-1786283495790_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I846" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Cihuy! Fandy Christian Go Public dengan Pacar Baru</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:01:13 +0700</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>wes</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>Pesinetron Fandy Christian akhirnya go public dengan kekasih baru, Marisa.</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8611302/cihuy-fandy-christian-go-public-dengan-pacar-baru</t>
+        </is>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/fandy-christian-1786276563371_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I847" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Sah! Dea Annisa Resmi Jadi Istri Mazaki Ahmad, Tampil Manglingi Berhijab</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:52:28 +0700</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>Desi Puspasari</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>Dea Annisa resmi menikah dengan Mazaki Ahmad, 9 Agustus 2026. Akad nikah berlangsung outdoor dengan nuansa putih, menandai cinta mereka yang telah dua tahun.</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8611363/sah-dea-annisa-resmi-jadi-istri-mazaki-ahmad-tampil-manglingi-berhijab</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/dea-annisa-1786274150781_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I848" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Momen Ijab Kabul Mazaki Ahmad dan Dea Annisa</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:50:47 +0700</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>Desi Puspasari</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>Mazaki Ahmad resmi menikahi Dea Annisa. Ini momen ijab kabul Mazaki Ahmad yang digelar pada Minggu (9/8/2026).</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8611294/momen-ijab-kabul-mazaki-ahmad-dan-dea-annisa</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/dea-annisa-1786274150956_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I849" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Fandy Christian Punya Pacar Baru, Dahlia Poland Ikut Senang</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:34:16 +0700</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>Dahlia Poland bahagia mendengar mantan suaminya, Fandy Christian, punya pacar baru. Ia berharap Fandy menemukan kebahagiaan dan hubungan yang langgeng.</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8611150/fandy-christian-punya-pacar-baru-dahlia-poland-ikut-senang</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/08/05/fandy-christian-dan-dahlia-poland-1754384716934_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I850" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Andika Dirawat di RS, Praz Teguh Manggung Bareng Kangen Band</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:28:11 +0700</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>wes</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>Praz Teguh menggantikan Andika Kangen Band yang sedang menjalani perawatan di rumah sakit.</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G851" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8611142/andika-dirawat-di-rs-praz-teguh-manggung-bareng-kangen-band</t>
+        </is>
+      </c>
+      <c r="H851" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kangen-band-1786268973889_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I851" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Kejutan di Panggung IFW 2026</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:47:57 +0700</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>prih febriani</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>Desainer Kukuh Hariyawan hadir di Indonesia Fashion Week 2026 dengan karya Kebaya Adhikari, menggabungkan kebaya, gajah, dan bendungan untuk pelestarian budaya.</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8611188/kejutan-di-panggung-ifw-2026</t>
+        </is>
+      </c>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kebaya-adhikari-1786239919980_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I852" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Fangfang Tak Persoalkan Vicky Prasetyo Nikah Lagi, Asal Penuhi Kewajiban ke Anak</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:17:29 +0700</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>Fangfang kini tidak mempermasalahkan rencana Vicky Prasetyo untuk menikah lagi, asalkan Vicky memenuhi tanggung jawabnya sebagai ayah untuk anak mereka.</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610998/fangfang-tak-persoalkan-vicky-prasetyo-nikah-lagi-asal-penuhi-kewajiban-ke-anak</t>
+        </is>
+      </c>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/15/vicky-prasetyo-1781525836079_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I853" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Aldi Taher Jual Rumah, Ngaku Masih Kurang Rp1 Miliar</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:24:16 +0700</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>Aldi Taher menjual rumah di Jagakarsa untuk pindah ke Rawamangun demi merawat ibunya. Ia butuh tambahan Rp1 miliar untuk mewujudkan rencana tersebut.</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610817/aldi-taher-jual-rumah-ngaku-masih-kurang-rp1-miliar</t>
+        </is>
+      </c>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/04/09/aldi-taher-1775693660069_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I854" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Salsa Kritik Konsumsi Pejabat, Usul Menu Makanan DPR hingga Acara 17 Agustus Pakai MBG Rp 15 Ribu</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:59:00 +0700</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>TribunNews.com menyajikan berita dan video terkini dari regional, nasional dan internasional dengan sudut pandang dan nilai-nilai lokal</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G855" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/</t>
+        </is>
+      </c>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>https://asset-2.tribunnews.com/tribunnews/foto/bank/images/logo-tribunnews1_20160901_101844.jpg</t>
+        </is>
+      </c>
+      <c r="I855" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Dari Kursi Pengemudi Hingga Ekosistem Transportasi, Hino Menjaga Indonesia Tetap Bergerak</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:15:25 +0700</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG -- Sebut saja namanya Sarib. Pria paruh baya asal Pemalang ini merupakan pengemudi bus antarkota antarprovinsi (AKAP) dengan trayek Jakarta-Kendal. Saat Republika menemuinya di Terminal Pulo Gebang, Kamis...</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjiftp348/dari-kursi-pengemudi-hingga-ekosistem-transportasi-hino-menjaga-indonesia-tetap-bergerak</t>
+        </is>
+      </c>
+      <c r="H856" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/hino-meluncurkan-bus-rm-280-abs-retarder-di-giias_260809230919-332.jpeg</t>
+        </is>
+      </c>
+      <c r="I856" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Menko Airlangga Lihat Langsung SUV Jetour T2 i-DM di GIIAS 2026, Kendaraan Resmi KTT G20 Afsel</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:39:20 +0700</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG -- Menteri Koordinator Bidang Perekonomian Airlangga Hartarto mengunjungi booth Jetour dalam ajang GAIKINDO Indonesia International Auto Show (GIIAS) 2026 di ICE BSD City, Tangerang, Jumat (7/8/2026). Dalam kunjungan...</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjie5k348/menko-airlangga-lihat-langsung-suv-jetour-t2-idm-di-giias-2026-kendaraan-resmi-ktt-g20-afsel</t>
+        </is>
+      </c>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/menteri-koordinator-bidang-perekonomian-airlangga-hartarto-mengunjungi-booth-jetour_260809223721-880.jpg</t>
+        </is>
+      </c>
+      <c r="I857" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Arai Agaska Punya Mimpi Besar Tembus Moto3 Bersama Yamaha</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:24:33 +0700</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>Pebalap Yamaha Racing Indonesia asal Lombok, Nusa Tenggara Barat, Arai Agaska, memiliki harapan besar untuk melangkah ke Moto3.</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/motogp/read/2026/08/09/23111678/arai-agaska-punya-mimpi-besar-tembus-moto3-bersama-yamaha</t>
+        </is>
+      </c>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/-rxlJgkPJ4009jcBHbL5vVkBv84=/124x0:1204x720/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/08/09/6a78a5671c5f8.jpeg</t>
+        </is>
+      </c>
+      <c r="I858" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Hasil Moto3 Inggris 2026: Veda Ega Finis ke-9, Almansa Pemenang</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:24:33 +0700</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>Veda Ega Pratama finis di posisi kesembilan pada race Moto3 Inggris 2026 di Sirkuit Silvestone, Minggu (9/8).</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/motogp/read/2026/08/09/21234928/hasil-moto3-inggris-2026-veda-ega-finis-ke-9-almansa-pemenang</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/t1irFL-7dTnjQvBHxJMMV5MD6Ss=/0x0:3529x2353/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/07/13/6a540887cc365.jpg</t>
+        </is>
+      </c>
+      <c r="I859" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Update Klasemen MotoGP 2026: Jorge Martin Belum Goyah di Puncak</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:24:33 +0700</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>Berikut ini adalah update klasemen MotoGP 2026 usai gelaran main race seri Inggris di Sirkuit Silverstone, Minggu (9/8/2026).</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/motogp/read/2026/08/09/20213168/update-klasemen-motogp-2026-jorge-martin-belum-goyah-di-puncak</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/AXMOiGoa2H6nw-ZlaOXqn3Yp7Fc=/0x406:1440x1366/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2025/07/19/687b4470f294f.jpg</t>
+        </is>
+      </c>
+      <c r="I860" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I822"/>
+  <autoFilter ref="A1:I860"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 17:25 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$860</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$876</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I860"/>
+  <dimension ref="A1:I876"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -40864,8 +40864,760 @@
         </is>
       </c>
     </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Aceh Barat salurkan Rp6 miliar perbaiki 1.308 ha sawah</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:37:39 +0700</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>Dinas Pertanian Tanaman Pangan dan Hortikultura Kabupaten Aceh Barat hingga saat ini telah menyalurkan dana swakelola ...</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686927/acehbarat-salurkan-rp6-miliar-perbaiki1308-ha-sawah</t>
+        </is>
+      </c>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/20260809-optimalisasi-lahan-satgas-prr-aceh-barat.jpeg</t>
+        </is>
+      </c>
+      <c r="I861" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Gempa magnitudo 5,5 guncang Enggano, Bengkulu pada Minggu malam</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:33:22 +0700</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) melaporkan gempa dengan magnitudo 5,5 mengguncang tenggara ...</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686923/gempa-magnitudo-55-guncang-enggano-bengkulu-pada-minggu-malam</t>
+        </is>
+      </c>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/24/1000817496.jpg</t>
+        </is>
+      </c>
+      <c r="I862" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Gubernur Sumut dukung lahirnya tenaga kesehatan di Kepulauan Nias</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:27:18 +0700</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>Gubernur Sumatera Utara (Sumut) Bobby Nasution menyatakan komitmen mendukung lahirnya tenaga kesehatan lewat ...</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G863" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686921/gubernur-sumut-dukung-lahirnya-tenaga-kesehatan-di-kepulauan-nias</t>
+        </is>
+      </c>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/1001038397.jpg</t>
+        </is>
+      </c>
+      <c r="I863" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Kapolri Ajak Jajaran Rutin Gelar Kompetisi E-sport: Perkembangannya Luar Biasa</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:57:36 +0700</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>Kapolri Jenderal Listyo Sigit Prabowo mendorong kompetisi E-Sports di Indonesia untuk mengembangkan atlet muda.</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8611408/kapolri-ajak-jajaran-rutin-gelar-kompetisi-e-sport-perkembangannya-luar-biasa</t>
+        </is>
+      </c>
+      <c r="H864" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/09/kapolri-jenderal-listyo-sigit-prabowo-ajak-atlet-dan-penikmat-gim-digital-untuk-mengambil-peran-aktif-menjaga-keamanan-ruang-d-1786285379118_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I864" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>FOTO: Serangan Rusia Hantam Salah Satu Stadion Terbesar di Ukraina</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:27:22 +0700</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>Serangan Rusia menghantam salah satu stadion sepak bola terbesar di Ukraina pada Jumat (7/8). Fasilitas stadion rusak parah dan dua orang dilaporkan terluka.</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G865" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260809160606-136-1390331/foto-serangan-rusia-hantam-salah-satu-stadion-terbesar-di-ukraina</t>
+        </is>
+      </c>
+      <c r="H865" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/serangan-rusia-hantam-salah-satu-stadion-terbesar-di-ukraina-1786266092829_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I865" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Zelensky: 50 Ribu Tentara Korea Utara Akan Dikerahkan Bantu Rusia</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:30:03 +0700</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>Zelensky mengklaim Korea Utara akan mengerahkan hingga 50 ribu tentara ke Rusia untuk berperang membantu sekutunya tersebut.</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G866" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260809211242-134-1390385/zelensky-50-ribu-tentara-korea-utara-akan-dikerahkan-bantu-rusia</t>
+        </is>
+      </c>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/05/18/presiden-ukrina-volodymyr-zelensky_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I866" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Bidik 50 Kursi DPR RI, Nazaruddin Minta Kader PRI Turun ke Rakyat</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:12:51 +0700</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>Partai Rakyat Indonesia (PRI) mulai memanaskan mesin politiknya untuk menyongsong Pemilu 2029.</t>
+        </is>
+      </c>
+      <c r="F867" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G867" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866108/bidik-50-kursi-dpr-ri-nazaruddin-minta-kader-pri-turun-ke-rakyat</t>
+        </is>
+      </c>
+      <c r="H867" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/vUfem-lAgtqpYCpD1rbJDJiAoM4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Muhammad-Nazaruddin-saat-menghadiri-perayaan-HUT-ke-1-PRI.jpg</t>
+        </is>
+      </c>
+      <c r="I867" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Apakah 'tombol darurat' mampu menghentikan AI yang berbalik menyerang?</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:04:22 +0700</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>Kasus pertama yang terkonfirmasi mengenai sistem kecerdasan buatan (AI) yang secara mandiri meretas sebuah perusahaan sungguhan telah…</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G868" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866107/apakah-tombol-darurat-mampu-menghentikan-ai-yang-berbalik-menyerang</t>
+        </is>
+      </c>
+      <c r="H868" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/s4LgaZqUTCv6bS8tnP8pxqHEyeI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/BBC-Indonesia178fe5c0-8f53-11f1-b8ee-9b3c26ad07bb.png.jpg</t>
+        </is>
+      </c>
+      <c r="I868" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Anji dan John LBF Dukung Pengembangan Domino sebagai Olahraga Prestasi</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:01:51 +0700</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>Turnamen Olahraga Domino (ORADO) diikuti mahasiswa, karyawan, dan masyarakat umum, Minggu (9/8/2025).</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G869" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866106/anji-dan-john-lbf-dukung-pengembangan-domino-sebagai-olahraga-prestasi</t>
+        </is>
+      </c>
+      <c r="H869" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/NPKsr9M1oq-mHTDZA1plqm1WUAM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Turnamen-domi.jpg</t>
+        </is>
+      </c>
+      <c r="I869" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Menag: Istiqlal Masuk Bursa Efek untuk Kelola Dana Wakaf Umat</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:00:44 +0700</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>Masjid Istiqlal telah masuk ke bursa efek sebagai bagian dari upaya pengelolaan dana wakaf umat</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G870" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866105/menag-istiqlal-masuk-bursa-efek-untuk-kelola-dana-wakaf-umat</t>
+        </is>
+      </c>
+      <c r="H870" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/p9XocUaw3k1M-0Qky8GR2peni2w=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Zikir-Kebangsaan-Doa-Keselamatan-Bangsa-dan-Haul-Pendiri-NKRI-di-Masjid-Istiqlal.jpg</t>
+        </is>
+      </c>
+      <c r="I870" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Kepala BPS Ajak Masyarakat Beri Jawaban Jujur Demi Akurasi Data Sensus Ekonomi 2026</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:14:57 +0700</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>BPS memaparkan perbedaan esensial dari pelaksanaan Sensus Ekonomi 2026 (SE2026) dibandingkan dengan jenis sensus nasional lainnya.</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G871" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866104/kepala-bps-ajak-masyarakat-beri-jawaban-jujur-demi-akurasi-data-sensus-ekonomi-2026</t>
+        </is>
+      </c>
+      <c r="H871" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/RzezeCRHWo96T6if7Qd9OD9LXDQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kepala-BPS-Amalia-Adininggar-Widyasanti-Podcast-di-Tribunnews_20260808_161626.jpg</t>
+        </is>
+      </c>
+      <c r="I871" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Harapan Jemaah Doa Bersama HUT Ke-81 RI di Masjid Istiqlal: Semoga Presiden Semakin Adil</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:08:28 +0700</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>Jemaah acara Doa Keselamatan Bangsa, Zikir Kebangsaan, dan Haul Pendiri NKRI Dalam Rangka HUT Ke-81 RI mengungkap berbagai harapan.</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G872" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866103/harapan-jemaah-doa-bersama-hut-ke-81-ri-di-masjid-istiqlal-semoga-presiden-semakin-adil</t>
+        </is>
+      </c>
+      <c r="H872" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/_ymkDXJTIlUP_oqxYr17X-zOlj4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Doa-Keselamatan-Bangsa-Zikir-Kebangsaan-dan-Haul-Pendiri-NKRI.jpg</t>
+        </is>
+      </c>
+      <c r="I872" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>GIIAS 2026 Umumkan Pemenang Penghargaan Exhibitor Night</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:55:49 +0700</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG -- GAIKINDO Indonesia International Auto Show (GIIAS) 2026 memberikan sejumlah penghargaan kepada peserta pameran dalam acara Exhibitor Night yang digelar Sabtu (8/8/2026). Penghargaan diberikan untuk berbagai kategori, mulai...</t>
+        </is>
+      </c>
+      <c r="F873" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G873" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjihp1348/giias-2026-umumkan-pemenang-penghargaan-exhibitor-night</t>
+        </is>
+      </c>
+      <c r="H873" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/pemberian-penghargaan-dalam-acara-exhibitor-night-di-giias_260809235424-105.jpg</t>
+        </is>
+      </c>
+      <c r="I873" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Mengenal Cara Kerja Teknologi i-DM pada Jetour T1 dan T2</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:48:54 +0700</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG -- Mesin bensin tidak selalu menjadi sumber tenaga utama. Motor listrik juga tidak bekerja sendirian. Pada dua SUV plug-in hybrid Jetour, keduanya dapat bekerja bergantian maupun bersamaan...</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G874" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjihdi348/mengenal-cara-kerja-teknologi-idm-pada-jetour-t1-dan-t2</t>
+        </is>
+      </c>
+      <c r="H874" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/jetour-t1_260809234817-394.png</t>
+        </is>
+      </c>
+      <c r="I874" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Hino, dari Kursi Pengemudi, Mengantar Cinta, Hingga Menggerakkan Ekonomi Negeri</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:15:25 +0700</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG -- Sebut saja namanya Sarib. Pria paruh baya asal Pemalang ini merupakan pengemudi bus antarkota antarprovinsi (AKAP) dengan trayek Jakarta-Kendal. Saat Republika menemuinya di Terminal Pulo Gebang, Jakarta...</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G875" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjiftp348/hino-dari-kursi-pengemudi-mengantar-cinta-hingga-menggerakkan-ekonomi-negeri</t>
+        </is>
+      </c>
+      <c r="H875" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/hino-meluncurkan-bus-rm-280-abs-retarder-di-giias_260809230919-332.jpeg</t>
+        </is>
+      </c>
+      <c r="I875" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Prabowo Minta Anak Cucu Perusahaan BUMN Dipangkas</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:43:47 +0700</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>Prabowo memerintahkan agar layer-layer dan anak cucu perusahaan BUMN dipangkas, khususnya Pertamina dan PLN.</t>
+        </is>
+      </c>
+      <c r="F876" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G876" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265862/prabowo-minta-anak-cucu-perusahaan-bumn-dipangkas</t>
+        </is>
+      </c>
+      <c r="H876" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/0mv-LGhFT4AXOKZbsiEFbMXmvZE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319861/original/026201600_1786293566-Screenshot_20260809_231044_Instagram.jpg</t>
+        </is>
+      </c>
+      <c r="I876" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I860"/>
+  <autoFilter ref="A1:I876"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 22:22 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$876</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$899</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I876"/>
+  <dimension ref="A1:I899"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -41616,8 +41616,1089 @@
         </is>
       </c>
     </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>DPR Dukung Pemerintah Perketat Naturalisasi WNA Demi Lindungi Aset RI</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 23:31:25 +0700</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>Ketua Komisi XIII DPR Willy Aditya mendorong pemerintah memperketat naturalisasi, tak cuma berdasarkan status atlet maupun ikatan pernikahan.</t>
+        </is>
+      </c>
+      <c r="F877" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G877" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809142909-12-1390305/dpr-dukung-pemerintah-perketat-naturalisasi-wna-demi-lindungi-aset-ri</t>
+        </is>
+      </c>
+      <c r="H877" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/05/06/ketua-dpp-nasdem-willy-aditya-2_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I877" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Basarnas Akhiri Monitoring Insiden Kebakaran KMP Mutiara Sentosa II</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 22:50:29 +0700</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>Badan SAR Nasional menghentikan monitoring KMP Mutiara Sentosa II setelah tidak ada tanda korban. 238 penumpang terdata, 233 selamat, 5 meninggal.</t>
+        </is>
+      </c>
+      <c r="F878" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G878" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809211730-20-1390388/basarnas-akhiri-monitoring-insiden-kebakaran-kmp-mutiara-sentosa-ii</t>
+        </is>
+      </c>
+      <c r="H878" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/03/evakuasi-korban-kebakaran-km-mutiara-sentosa-ii-1785712804674_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I878" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Penggeledahan Sepekan KPK di Bengkulu, Sita Dokumen-Barang Elektronik</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 21:00:34 +0700</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>KPK melakukan penggeledahan di Bengkulu terkait kasus dugaan korupsi Bupati Rejang Lebong, M Fikri Thobari, menyita dokumen dan barang elektronik.</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G879" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809202933-12-1390380/penggeledahan-sepekan-kpk-di-bengkulu-sita-dokumen-barang-elektronik</t>
+        </is>
+      </c>
+      <c r="H879" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/03/05/ilustrasi-gedung-kpk-2_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I879" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>KPK Geledah 15 Lokasi Terkait Kasus Pemerasan Bupati Pemalang</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:40:18 +0700</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>KPK menggeledah 15 lokasi terkait kasus pemerasan Bupati Pemalang, Anom Widiyantoro.</t>
+        </is>
+      </c>
+      <c r="F880" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G880" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809202318-12-1390378/kpk-geledah-15-lokasi-terkait-kasus-pemerasan-bupati-pemalang</t>
+        </is>
+      </c>
+      <c r="H880" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/03/05/ilustrasi-gedung-kpk-8_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I880" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Kebakaran Gunung Gede, Ratusan Petugas Masih Berupaya Padamkan Api</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 20:10:00 +0700</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>Sekitar 150 petugas gabungan dan relawan masih berupaya memadamkan api yang membakar lahan di sekitar kawah Wadon Gunung Gede.</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G881" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809183137-20-1390365/kebakaran-gunung-gede-ratusan-petugas-masih-berupaya-padamkan-api</t>
+        </is>
+      </c>
+      <c r="H881" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/bb-tnggp-tutup-jalur-pendakian-karena-kebakaran-alun-alun-suryakancana-1786099073263_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I881" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Pendiri Yayasan Sekolah Harapan Ibu Buka Suara soal Temuan 995 Senjata</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:50:38 +0700</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>Pendiri Yayasan Sekolah Islam Harapan Ibu merespons temuan 996 senjata dan ekstrakurikuler menembak di dalam sekolah.</t>
+        </is>
+      </c>
+      <c r="F882" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G882" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809184334-12-1390369/pendiri-yayasan-sekolah-harapan-ibu-buka-suara-soal-temuan-995-senjata</t>
+        </is>
+      </c>
+      <c r="H882" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/sterilisasi-sekolah-swasta-usai-temuan-senjata-api-1786268268243_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I882" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Sumenep Siapkan Lahan 7,1 Hektare Jadi Lokasi Sekolah Rakyat Permanen</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:25:11 +0700</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>Lahan milik pemda yang awalnya diperuntukkan untuk sport center tersebut berlokasi di Desa Gunggung, Kecamatan Batuan, persis di seberang Universitas Wiraraja.</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G883" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809184722-25-1390371/sumenep-siapkan-lahan-71-hektare-jadi-lokasi-sekolah-rakyat-permanen</t>
+        </is>
+      </c>
+      <c r="H883" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/kemensos-1786273016901_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I883" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>FOTO: Ribuan Pesilat Ramaikan HBKB Jakarta</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:10:39 +0700</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>CNN Indonesia/Febria Adha L</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>Lebih dari 6.000 pesilat dari berbagai perguruan memadati kawasan Bundaran HI saat Hari Bebas Kendaraan Bermotor (HBKB) di Bundaran HI, Jakarta, Minggu (9/8).</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G884" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809121629-22-1390263/foto-ribuan-pesilat-ramaikan-hbkb-jakarta</t>
+        </is>
+      </c>
+      <c r="H884" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/ribuan-pesilat-ramaikan-hbkb-jakarta-1786251385492_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I884" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Bos Padel di Bandung Kena Denda Rp100 Juta dan Wajib Tanam 1.000 Pohon</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:00:26 +0700</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>Pemerintah menjatuhkan sanksi Rp100 juta dan penanaman 1.000 pohon kepada pemilik lapangan padel di Bandung yang menebang 10 pohon secara ilegal.</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G885" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809173431-12-1390360/bos-padel-di-bandung-kena-denda-rp100-juta-dan-wajib-tanam-1000-pohon</t>
+        </is>
+      </c>
+      <c r="H885" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/02/10-pohon-peneduh-bandung-ditebang-farhan-ancam-pidanakan-bos-padel-1785656870697_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I885" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Bedah Rumah Orang Tua Siswa Sekolah Rakyat Madura Mulai Berjalan</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:40:15 +0700</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>Khusus untuk Kabupaten Sumenep, kuota tersedia sebanyak 50 titik. Dari jumlah tersebut, delapan di antaranya sudah lolos verifikasi.</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G886" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809183724-25-1390366/bedah-rumah-orang-tua-siswa-sekolah-rakyat-madura-mulai-berjalan</t>
+        </is>
+      </c>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/kemensos-1786273016752_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I886" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Kebakaran Besar di Pasar Jagong Jeget Aceh Hanguskan 96 Unit Kios</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>Sedikitnya 96 unit kios atau ruko berkonstruksi kayu ludes dilalap api imbas kebakaran hebat yang melanda kawasan Pasar Jagong Jeget, Aceh Tengah.</t>
+        </is>
+      </c>
+      <c r="F887" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G887" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809171348-20-1390357/kebakaran-besar-di-pasar-jagong-jeget-aceh-hanguskan-96-unit-kios</t>
+        </is>
+      </c>
+      <c r="H887" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2021/07/19/ilustrasi-kebakaran-2_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I887" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Seskab Teddy Disambut Puisi Siswa SR 'Dari Jalanan Menuju Harapan'</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:20:01 +0700</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>Siswa Sekolah Rakyat tampil percaya diri di Politeknik Penerbangan Indonesia, menunjukkan bakat dan perubahan hidup berkat akses pendidikan berkualitas.</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G888" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809180252-25-1390362/seskab-teddy-disambut-puisi-siswa-sr-dari-jalanan-menuju-harapan</t>
+        </is>
+      </c>
+      <c r="H888" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/kemensos-1786272851441_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I888" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Respons TNI dan Polri soal Pramuka Garuda Bisa Daftar Tanpa Tes</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:10:36 +0700</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>TNI dan Polri angkat suara soal pemegang sertifikat Pramuka Garuda bisa bergabung dengan dua lembaga tersebut tanpa mengikuti tes seleksi.</t>
+        </is>
+      </c>
+      <c r="F889" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G889" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809165822-12-1390354/respons-tni-dan-polri-soal-pramuka-garuda-bisa-daftar-tanpa-tes</t>
+        </is>
+      </c>
+      <c r="H889" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2020/08/14/peringatan-hari-pramuka-kala-pandemi-13_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I889" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>Polresta Banyumas Serahkan Pengusutan Kasus Sutrimo ke Polda Metro</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:50:58 +0700</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>Polresta Banyumas serahkan kasus kematian Sutrimo ke Polda Metro Jaya. Penyidik akan lakukan ekshumasi untuk menyelidiki kejanggalan.</t>
+        </is>
+      </c>
+      <c r="F890" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G890" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809162159-12-1390339/polresta-banyumas-serahkan-pengusutan-kasus-sutrimo-ke-polda-metro</t>
+        </is>
+      </c>
+      <c r="H890" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/keluarga-sutrimo-didampingi-kuasa-hukum-membuat-laporan-ke-polresta-banyumas-1786243465746_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I890" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Duga Penebangan 10 Pohon Terencana, DPRD Bandung Desak Langkah Hukum</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:15:04 +0700</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>Mengapresiasi teguran Wali Kota akan penebangan 10 pohon baru-baru ini, DPRD Kota Bandung menilai perlu perlu tindaklanjut berupa proses hukum.</t>
+        </is>
+      </c>
+      <c r="F891" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G891" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809162544-25-1390340/duga-penebangan-10-pohon-terencana-dprd-bandung-desak-langkah-hukum</t>
+        </is>
+      </c>
+      <c r="H891" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/dprd-kota-bandung-1785922771499_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I891" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Tembok Pembatas SD di Sleman Roboh Timpa Peserta Jalan Sehat, 10 Luka</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 17:00:01 +0700</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>Sepuluh peserta jalan sehat di Sleman, DIY mengalami luka-luka hingga dilarikan ke rumah sakit usai tertimpa tembok pembatas milik SDN Minomartani 2, Ngaglik.</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G892" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809154256-20-1390325/tembok-pembatas-sd-di-sleman-roboh-timpa-peserta-jalan-sehat-10-luka</t>
+        </is>
+      </c>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/01/22/tembok-roboh-tewaskan-tiga-orang-di-tebet_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I892" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Gudang Paket, Plastik dan Suku Cadang Terbakar di Kosambi Tangerang</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:55:52 +0700</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda tiga gudang di Kawasan Pergudangan Sentra Kosambi, Kecamatan Kosambi, Kabupaten Tangerang, Banten, Minggu (9/8).</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G893" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809165321-20-1390353/gudang-paket-plastik-dan-suku-cadang-terbakar-di-kosambi-tangerang</t>
+        </is>
+      </c>
+      <c r="H893" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/12/24/ilustrasi-memadamkan-api_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I893" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>DPRD Bandung Perketat Pengawasan Pembangunan RSUD dan Gedung Inspektorat</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:55:18 +0700</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>DPRD Kota Bandung memetakan risiko pembangunan RSUD dan Gedung Inspektorat, FGD membahas mitigasi untuk memastikan proyek berjalan sesuai target dan anggaran.</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G894" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809163918-25-1390343/dprd-bandung-perketat-pengawasan-pembangunan-rsud-gedung-inspektorat</t>
+        </is>
+      </c>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/dprd-kota-bandung-1786267044990_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I894" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Curiga Kopi Diludahi, Satpam Tusuk Pegawai KPU Wajo Sulsel</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>Polisi menangkap seorang sekuriti KPU Kabupaten Wajo, Sulawesi Selatan, karena diduga telah menikam pegawai KPU gara-gara perkara secangkir kopi.</t>
+        </is>
+      </c>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G895" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809152852-12-1390322/curiga-kopi-diludahi-satpam-tusuk-pegawai-kpu-wajo-sulsel</t>
+        </is>
+      </c>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2015/05/27/b61083a3-a4c6-4f2b-a038-aca96f8daba0_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I895" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Penjelasan PO soal Viral Klakson Bus Suara Jokowi 'Saya Akan Lawan!'</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 16:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>Manajemen Perusahaan Otobus (PO) MTrans memberikan klarifikasi terkait video viral bus dengan klakson potongan suara pidato Presiden ke-7 RI Jokowi.</t>
+        </is>
+      </c>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G896" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809150809-20-1390318/penjelasan-po-soal-viral-klakson-bus-suara-jokowi-saya-akan-lawan</t>
+        </is>
+      </c>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/humas-resources-development-hrd-mtrans-jhony-sasongko-po-bus-pakai-klakson-suara-jokowi-saya-akan-lawan-1786263134836_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I896" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Polisi Usut Identitas Staf Kejagung Terkait Kematian Janggal Sutrimo</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:30:26 +0700</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>Polisi selidiki kematian Sutrimo dengan mendalami sosok Febrio Adiono, staf Kejagung yang terlibat sebagai pengantar jasad.</t>
+        </is>
+      </c>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G897" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809144908-12-1390308/polisi-usut-identitas-staf-kejagung-terkait-kematian-janggal-sutrimo</t>
+        </is>
+      </c>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/keluarga-sutrimo-didampingi-kuasa-hukum-membuat-laporan-ke-polresta-banyumas-1786243465746_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I897" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Meresahkan Warga, Pengemis di Kudus Sehari Raup Rp540 Ribu</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:10:05 +0700</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>Pengemis perempuan inisial J (40) dianggap meresahkan warga karena kerap meminta warga dan peziarah dengan cara memaksa di kawasan Menara Kudus.</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G898" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809141747-20-1390303/meresahkan-warga-pengemis-di-kudus-sehari-raup-rp540-ribu</t>
+        </is>
+      </c>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/pengemis-berinisial-j-yang-kedapatan-mengantongi-rp-540-ribu-sehari-saat-diciduk-satpol-pp-kabupaten-kudus-1786260611092_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I898" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Pelaku Mutilasi Gay di Depok Pernah Jadi Guru Matematika dan Masuk TV</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 15:00:21 +0700</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>Polisi mengungkap identitas Saepul, pelaku mutilasi di Depok yang merupakan penyuka sesama jenis alias gay.</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G899" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260809142249-12-1390304/pelaku-mutilasi-gay-di-depok-pernah-jadi-guru-matematika-dan-masuk-tv</t>
+        </is>
+      </c>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/09/saepul-pelaku-pembunuhan-dan-mutilasi-pria-di-pancoran-mas-depok-1786258388237_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I899" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I876"/>
+  <autoFilter ref="A1:I899"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 03:08 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$899</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$900</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I899"/>
+  <dimension ref="A1:I900"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -42697,8 +42697,55 @@
         </is>
       </c>
     </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>DPO Kasus Penembakan Kuala Kencana hingga Mile 69 Ditindak</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:49:08 +0700</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>Polisi melakukan penindakan terhadap seorang pria yang masuk dalam DPO sejumlah kasus penembakan di Papua.</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G900" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265744/dpo-kasus-penembakan-kuala-kencana-hingga-mile-69-ditindak</t>
+        </is>
+      </c>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/17vKsT7Hl4qvLcz2Ln_HgtGrIxQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319751/original/053062700_1786279748-Satgas.jpg</t>
+        </is>
+      </c>
+      <c r="I900" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I899"/>
+  <autoFilter ref="A1:I900"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 07:10 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-09.xlsx
+++ b/data/berita_2026-08-09.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$900</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$902</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I900"/>
+  <dimension ref="A1:I902"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -42744,8 +42744,102 @@
         </is>
       </c>
     </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Duit Warga RI Rp 9,1 Triliun Dimaling, 1.000 Korban Tiap Hari</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 19:15:57 +0700</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>OJK melaporkan 432.637 kasus penipuan digital di Indonesia dengan kerugian Rp9,1 triliun. Penanganan scam menjadi tantangan besar bagi OJK.</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G901" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260809174657-17-757740/duit-warga-ri-rp-91-triliun-dimaling-1000-korban-tiap-hari</t>
+        </is>
+      </c>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/11/kbri-phnom-penh-memberikan-bantuan-kekonsuleran-kepada-sekitar-1100-warga-negara-indonesia-wni-yang-berada-di-fasilitas-detens-1783735309957_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I901" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Laba Berkshire Naik, Abel Mulai Kucurkan Kas Jumbo Warisan Buffett</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Sun, 09 Aug 2026 18:15:39 +0700</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>Berkshire Hathaway catat laba operasional naik 16% di kuartal kedua 2026. CEO Greg Abel aktifkan buyback saham dan investasi, meski segmen asuransi melemah.</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260809154439-17-757735/laba-berkshire-naik-abel-mulai-kucurkan-kas-jumbo-warisan-buffett</t>
+        </is>
+      </c>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2021/05/03/greg-abel_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I902" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I900"/>
+  <autoFilter ref="A1:I902"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>